<commit_message>
Workbook: packed30 family sheet now includes canonical joint-K4 column
Adds canonical pos/macro reference for Qwen rows (heads marked 'not run'
under this recipe) so the packed30-family sheet compares all three
conditions per method.
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -2999,7 +2999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3014,14 +3014,14 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DAIC runtime participant-packed30: v1 vs joint-K4 (official 47-subject test, seed 1337, strict teacher-forced)</t>
+          <t>DAIC runtime participant-packed30: canonical vs v1 vs joint-K4 (official 47-subject test, seed 1337, strict teacher-forced)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Qwen verdict = mean teacher-forced score margin per subject (INVALID counts as wrong; INVALID=0). Heads = logreg_raw / xgb_raw on hidden features, mean depressed probability &gt;= 0.5 per subject. Selected epochs: joint-K4 audio-only 5, audio+text 3; v1 audio-only 3, audio+text 2.</t>
+          <t>Qwen verdict = mean teacher-forced score margin per subject (INVALID counts as wrong; INVALID=0). Heads = logreg_raw / xgb_raw on hidden features, mean depressed probability &gt;= 0.5 per subject. Canonical joint-K4 has no head caches under this recipe (not run). Selected epochs: joint-K4 audio-only 5, audio+text 3; v1 audio-only 3, audio+text 2.</t>
         </is>
       </c>
     </row>
@@ -3053,10 +3053,15 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
+          <t>Canonical joint-K4 (pos / macro)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>Source run</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Local artifact</t>
         </is>
@@ -3082,10 +3087,15 @@
       <c r="E4" s="10" t="n"/>
       <c r="F4" s="10" t="inlineStr">
         <is>
+          <t>0.800 / 0.841</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_audio_text_s1337_05b52c6b (commit 3caa208)</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30/audio_text/&lt;run&gt;/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json (recomputed from predictions)</t>
         </is>
@@ -3113,10 +3123,15 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
+          <t>not run</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_audio_text_s1337_05b52c6b (commit 3caa208)</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30/audio_text/&lt;run&gt;/fold_0/best_model/logreg_raw/metrics.json (recomputed from predictions)</t>
         </is>
@@ -3144,10 +3159,15 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
+          <t>not run</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_audio_text_s1337_05b52c6b (commit 3caa208)</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30/audio_text/&lt;run&gt;/fold_0/best_model/xgb_raw/metrics.json (recomputed from predictions)</t>
         </is>
@@ -3173,10 +3193,15 @@
       <c r="E8" s="10" t="n"/>
       <c r="F8" s="10" t="inlineStr">
         <is>
+          <t>0.522 / 0.683</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_audio_only_s1337_05b52c6b (commit 3caa208)</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30/audio_only/&lt;run&gt;/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json (recomputed from predictions)</t>
         </is>
@@ -3204,10 +3229,15 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
+          <t>not run</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_audio_only_s1337_05b52c6b (commit 3caa208)</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30/audio_only/&lt;run&gt;/fold_0/best_model/logreg_raw/metrics.json (recomputed from predictions)</t>
         </is>
@@ -3235,10 +3265,15 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
+          <t>not run</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_audio_only_s1337_05b52c6b (commit 3caa208)</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30/audio_only/&lt;run&gt;/fold_0/best_model/xgb_raw/metrics.json (recomputed from predictions)</t>
         </is>
@@ -3264,10 +3299,15 @@
       <c r="E12" s="10" t="n"/>
       <c r="F12" s="10" t="inlineStr">
         <is>
+          <t>0.800 / 0.841</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_jointk4_audio_text_s1337_e3b0f1c3 (commit e3b0f1c)</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="H12" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30_jointk4/audio_text/&lt;run&gt;/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json (recomputed from predictions)</t>
         </is>
@@ -3295,10 +3335,15 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
+          <t>not run</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_jointk4_audio_text_s1337_e3b0f1c3 (commit e3b0f1c)</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30_jointk4/audio_text/&lt;run&gt;/fold_0/best_model/logreg_raw/metrics.json (recomputed from predictions)</t>
         </is>
@@ -3326,10 +3371,15 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
+          <t>not run</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_jointk4_audio_text_s1337_e3b0f1c3 (commit e3b0f1c)</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="H14" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30_jointk4/audio_text/&lt;run&gt;/fold_0/best_model/xgb_raw/metrics.json (recomputed from predictions)</t>
         </is>
@@ -3355,10 +3405,15 @@
       <c r="E16" s="10" t="n"/>
       <c r="F16" s="10" t="inlineStr">
         <is>
+          <t>0.522 / 0.683</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_jointk4_audio_only_s1337_e3b0f1c3 (commit e3b0f1c)</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
+      <c r="H16" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30_jointk4/audio_only/&lt;run&gt;/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json (recomputed from predictions)</t>
         </is>
@@ -3386,10 +3441,15 @@
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
+          <t>not run</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_jointk4_audio_only_s1337_e3b0f1c3 (commit e3b0f1c)</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30_jointk4/audio_only/&lt;run&gt;/fold_0/best_model/logreg_raw/metrics.json (recomputed from predictions)</t>
         </is>
@@ -3417,10 +3477,15 @@
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
+          <t>not run</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
           <t>daic_participant_p30_jointk4_audio_only_s1337_e3b0f1c3 (commit e3b0f1c)</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>output_model/experiments/daic_participant_packed30_jointk4/audio_only/&lt;run&gt;/fold_0/best_model/xgb_raw/metrics.json (recomputed from predictions)</t>
         </is>
@@ -3429,7 +3494,7 @@
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Provenance sheet holds the full mapping (commit, job IDs incl. resubmits, eval view, aggregation, audits 44369722/44369723 GPFS PASSED + local evidence audit PASSED).</t>
+          <t>Canonical = preprocessed joint-K4 (2026-08-05 coverage validation; no head caches under this recipe). Provenance sheet holds the full mapping (commit, job IDs incl. resubmits, eval view, aggregation, audits 44369722/44369723 GPFS PASSED + local evidence audit PASSED).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct the record: canonical joint-K4 heads exist (daic_coverage_heads_20260805_04f2e19)
The canonical preprocessed checkpoints DO have logreg_raw/xgb_raw scores
on the complete-coverage (c2_balanced) view; earlier report/workbook
claimed 'not run'. Fill canonical head cells (A+T: 0.7647/0.8157/0.9177
logreg, 0.6429/0.7457/0.8831 xgb; A-only: 0.5714/0.6586/0.8225,
0.3636/0.5846/0.7814), verified locally by recomputation from the synced
predictions_subject_level.jsonl, and add their provenance rows.
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -3021,7 +3021,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Qwen verdict = mean teacher-forced score margin per subject (INVALID counts as wrong; INVALID=0). Heads = logreg_raw / xgb_raw on hidden features, mean depressed probability &gt;= 0.5 per subject. Canonical joint-K4 has no head caches under this recipe (not run). Selected epochs: joint-K4 audio-only 5, audio+text 3; v1 audio-only 3, audio+text 2.</t>
+          <t>Qwen verdict = mean teacher-forced score margin per subject (INVALID counts as wrong; INVALID=0). Heads = logreg_raw / xgb_raw on hidden features, mean depressed probability &gt;= 0.5 per subject. Canonical heads = daic_coverage_heads_20260805_04f2e19 complete-coverage (c2_balanced) view. Selected epochs: joint-K4 audio-only 5, audio+text 3; v1 audio-only 3, audio+text 2.</t>
         </is>
       </c>
     </row>
@@ -3053,7 +3053,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Canonical joint-K4 (pos / macro)</t>
+          <t>Canonical joint-K4 (pos / macro / AUROC)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3087,7 +3087,7 @@
       <c r="E4" s="10" t="n"/>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>0.800 / 0.841</t>
+          <t>0.800 / 0.841 / n/a</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>not run</t>
+          <t>0.765 / 0.816 / 0.918</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>not run</t>
+          <t>0.643 / 0.746 / 0.883</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -3193,7 +3193,7 @@
       <c r="E8" s="10" t="n"/>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>0.522 / 0.683</t>
+          <t>0.522 / 0.683 / n/a</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>not run</t>
+          <t>0.571 / 0.659 / 0.823</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -3265,7 +3265,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>not run</t>
+          <t>0.364 / 0.585 / 0.781</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -3299,7 +3299,7 @@
       <c r="E12" s="10" t="n"/>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>0.800 / 0.841</t>
+          <t>0.800 / 0.841 / n/a</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>not run</t>
+          <t>0.765 / 0.816 / 0.918</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>not run</t>
+          <t>0.643 / 0.746 / 0.883</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -3405,7 +3405,7 @@
       <c r="E16" s="10" t="n"/>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>0.522 / 0.683</t>
+          <t>0.522 / 0.683 / n/a</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>not run</t>
+          <t>0.571 / 0.659 / 0.823</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>not run</t>
+          <t>0.364 / 0.585 / 0.781</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -3494,7 +3494,7 @@
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Canonical = preprocessed joint-K4 (2026-08-05 coverage validation; no head caches under this recipe). Provenance sheet holds the full mapping (commit, job IDs incl. resubmits, eval view, aggregation, audits 44369722/44369723 GPFS PASSED + local evidence audit PASSED).</t>
+          <t>Canonical = preprocessed joint-K4 (Qwen: 2026-08-05 coverage validation; heads: daic_coverage_heads_20260805_04f2e19 c2_balanced, verified locally by recomputation). Provenance sheet holds the full mapping (commit, job IDs incl. resubmits, eval view, aggregation, audits 44369722/44369723 GPFS PASSED + local evidence audit PASSED).</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I186"/>
+  <dimension ref="A1:I190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11695,7 +11695,7 @@
       </c>
       <c r="C183" s="14" t="inlineStr">
         <is>
-          <t>Joint-K4 Audio + Text</t>
+          <t>Canonical Audio + Text</t>
         </is>
       </c>
       <c r="D183" s="14" t="inlineStr">
@@ -11704,26 +11704,26 @@
         </is>
       </c>
       <c r="E183" s="15" t="n">
-        <v>0.7333</v>
+        <v>0.7647</v>
       </c>
       <c r="F183" s="16" t="inlineStr">
         <is>
-          <t>daic_participant_p30_jointk4_&lt;mod&gt;_s1337_e3b0f1c3 selected-epoch head fit (107 vectors, weights 1.0)</t>
+          <t>daic_coverage_heads_20260805_04f2e19 canonical checkpoints (audio_text=daic_main_k4_control_20260804_f26dd45, audio_only=daic_replicates_20ep_s1337_daic_audio_only_selposf1_tf)</t>
         </is>
       </c>
       <c r="G183" s="16" t="inlineStr">
         <is>
-          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, 617 bundles</t>
+          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, complete-coverage (c2_balanced) view</t>
         </is>
       </c>
       <c r="H183" s="16" t="inlineStr">
         <is>
-          <t>output_model/experiments/daic_participant_packed30_jointk4/&lt;modality&gt;/&lt;run&gt;/hidden_classifiers/audio_text/logreg_raw/</t>
+          <t>outputs/daic_coverage_heads/daic_coverage_heads_20260805_04f2e19/audio_text/classical/c2/logreg_raw/</t>
         </is>
       </c>
       <c r="I183" s="16" t="inlineStr">
         <is>
-          <t>matched to audited hidden-classifier outputs</t>
+          <t>recomputed from predictions_subject_level.jsonl (metrics match)</t>
         </is>
       </c>
     </row>
@@ -11740,7 +11740,7 @@
       </c>
       <c r="C184" s="14" t="inlineStr">
         <is>
-          <t>Joint-K4 Audio + Text</t>
+          <t>Canonical Audio + Text</t>
         </is>
       </c>
       <c r="D184" s="14" t="inlineStr">
@@ -11749,26 +11749,26 @@
         </is>
       </c>
       <c r="E184" s="15" t="n">
-        <v>0.7692</v>
+        <v>0.6429</v>
       </c>
       <c r="F184" s="16" t="inlineStr">
         <is>
-          <t>daic_participant_p30_jointk4_&lt;mod&gt;_s1337_e3b0f1c3 selected-epoch head fit (107 vectors, weights 1.0)</t>
+          <t>daic_coverage_heads_20260805_04f2e19 canonical checkpoints (audio_text=daic_main_k4_control_20260804_f26dd45, audio_only=daic_replicates_20ep_s1337_daic_audio_only_selposf1_tf)</t>
         </is>
       </c>
       <c r="G184" s="16" t="inlineStr">
         <is>
-          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, 617 bundles</t>
+          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, complete-coverage (c2_balanced) view</t>
         </is>
       </c>
       <c r="H184" s="16" t="inlineStr">
         <is>
-          <t>output_model/experiments/daic_participant_packed30_jointk4/&lt;modality&gt;/&lt;run&gt;/hidden_classifiers/audio_text/xgb_raw/</t>
+          <t>outputs/daic_coverage_heads/daic_coverage_heads_20260805_04f2e19/audio_text/classical/c2/xgb_raw/</t>
         </is>
       </c>
       <c r="I184" s="16" t="inlineStr">
         <is>
-          <t>matched to audited hidden-classifier outputs</t>
+          <t>recomputed from predictions_subject_level.jsonl (metrics match)</t>
         </is>
       </c>
     </row>
@@ -11785,7 +11785,7 @@
       </c>
       <c r="C185" s="14" t="inlineStr">
         <is>
-          <t>Joint-K4 Audio only</t>
+          <t>Canonical Audio only</t>
         </is>
       </c>
       <c r="D185" s="14" t="inlineStr">
@@ -11794,26 +11794,26 @@
         </is>
       </c>
       <c r="E185" s="15" t="n">
-        <v>0.6471</v>
+        <v>0.5714</v>
       </c>
       <c r="F185" s="16" t="inlineStr">
         <is>
-          <t>daic_participant_p30_jointk4_&lt;mod&gt;_s1337_e3b0f1c3 selected-epoch head fit (107 vectors, weights 1.0)</t>
+          <t>daic_coverage_heads_20260805_04f2e19 canonical checkpoints (audio_text=daic_main_k4_control_20260804_f26dd45, audio_only=daic_replicates_20ep_s1337_daic_audio_only_selposf1_tf)</t>
         </is>
       </c>
       <c r="G185" s="16" t="inlineStr">
         <is>
-          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, 617 bundles</t>
+          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, complete-coverage (c2_balanced) view</t>
         </is>
       </c>
       <c r="H185" s="16" t="inlineStr">
         <is>
-          <t>output_model/experiments/daic_participant_packed30_jointk4/&lt;modality&gt;/&lt;run&gt;/hidden_classifiers/audio_only/logreg_raw/</t>
+          <t>outputs/daic_coverage_heads/daic_coverage_heads_20260805_04f2e19/audio_only/classical/c2/logreg_raw/</t>
         </is>
       </c>
       <c r="I185" s="16" t="inlineStr">
         <is>
-          <t>matched to audited hidden-classifier outputs</t>
+          <t>recomputed from predictions_subject_level.jsonl (metrics match)</t>
         </is>
       </c>
     </row>
@@ -11830,35 +11830,215 @@
       </c>
       <c r="C186" s="14" t="inlineStr">
         <is>
+          <t>Canonical Audio only</t>
+        </is>
+      </c>
+      <c r="D186" s="14" t="inlineStr">
+        <is>
+          <t>XGBoost raw</t>
+        </is>
+      </c>
+      <c r="E186" s="15" t="n">
+        <v>0.3636</v>
+      </c>
+      <c r="F186" s="16" t="inlineStr">
+        <is>
+          <t>daic_coverage_heads_20260805_04f2e19 canonical checkpoints (audio_text=daic_main_k4_control_20260804_f26dd45, audio_only=daic_replicates_20ep_s1337_daic_audio_only_selposf1_tf)</t>
+        </is>
+      </c>
+      <c r="G186" s="16" t="inlineStr">
+        <is>
+          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, complete-coverage (c2_balanced) view</t>
+        </is>
+      </c>
+      <c r="H186" s="16" t="inlineStr">
+        <is>
+          <t>outputs/daic_coverage_heads/daic_coverage_heads_20260805_04f2e19/audio_only/classical/c2/xgb_raw/</t>
+        </is>
+      </c>
+      <c r="I186" s="16" t="inlineStr">
+        <is>
+          <t>recomputed from predictions_subject_level.jsonl (metrics match)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="14" t="inlineStr">
+        <is>
+          <t>DAIC packed30 family</t>
+        </is>
+      </c>
+      <c r="B187" s="14" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C187" s="14" t="inlineStr">
+        <is>
+          <t>Joint-K4 Audio + Text</t>
+        </is>
+      </c>
+      <c r="D187" s="14" t="inlineStr">
+        <is>
+          <t>LogReg raw</t>
+        </is>
+      </c>
+      <c r="E187" s="15" t="n">
+        <v>0.7333</v>
+      </c>
+      <c r="F187" s="16" t="inlineStr">
+        <is>
+          <t>daic_participant_p30_jointk4_&lt;mod&gt;_s1337_e3b0f1c3 selected-epoch head fit (107 vectors, weights 1.0)</t>
+        </is>
+      </c>
+      <c r="G187" s="16" t="inlineStr">
+        <is>
+          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, 617 bundles</t>
+        </is>
+      </c>
+      <c r="H187" s="16" t="inlineStr">
+        <is>
+          <t>hidden_classifiers/audio_text/logreg_raw/</t>
+        </is>
+      </c>
+      <c r="I187" s="16" t="inlineStr">
+        <is>
+          <t>recomputed from predictions_subject_level.jsonl (metrics match)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="14" t="inlineStr">
+        <is>
+          <t>DAIC packed30 family</t>
+        </is>
+      </c>
+      <c r="B188" s="14" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C188" s="14" t="inlineStr">
+        <is>
+          <t>Joint-K4 Audio + Text</t>
+        </is>
+      </c>
+      <c r="D188" s="14" t="inlineStr">
+        <is>
+          <t>XGBoost raw</t>
+        </is>
+      </c>
+      <c r="E188" s="15" t="n">
+        <v>0.7692</v>
+      </c>
+      <c r="F188" s="16" t="inlineStr">
+        <is>
+          <t>daic_participant_p30_jointk4_&lt;mod&gt;_s1337_e3b0f1c3 selected-epoch head fit (107 vectors, weights 1.0)</t>
+        </is>
+      </c>
+      <c r="G188" s="16" t="inlineStr">
+        <is>
+          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, 617 bundles</t>
+        </is>
+      </c>
+      <c r="H188" s="16" t="inlineStr">
+        <is>
+          <t>hidden_classifiers/audio_text/xgb_raw/</t>
+        </is>
+      </c>
+      <c r="I188" s="16" t="inlineStr">
+        <is>
+          <t>recomputed from predictions_subject_level.jsonl (metrics match)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="14" t="inlineStr">
+        <is>
+          <t>DAIC packed30 family</t>
+        </is>
+      </c>
+      <c r="B189" s="14" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C189" s="14" t="inlineStr">
+        <is>
           <t>Joint-K4 Audio only</t>
         </is>
       </c>
-      <c r="D186" s="14" t="inlineStr">
+      <c r="D189" s="14" t="inlineStr">
+        <is>
+          <t>LogReg raw</t>
+        </is>
+      </c>
+      <c r="E189" s="15" t="n">
+        <v>0.6471</v>
+      </c>
+      <c r="F189" s="16" t="inlineStr">
+        <is>
+          <t>daic_participant_p30_jointk4_&lt;mod&gt;_s1337_e3b0f1c3 selected-epoch head fit (107 vectors, weights 1.0)</t>
+        </is>
+      </c>
+      <c r="G189" s="16" t="inlineStr">
+        <is>
+          <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, 617 bundles</t>
+        </is>
+      </c>
+      <c r="H189" s="16" t="inlineStr">
+        <is>
+          <t>hidden_classifiers/audio_only/logreg_raw/</t>
+        </is>
+      </c>
+      <c r="I189" s="16" t="inlineStr">
+        <is>
+          <t>recomputed from predictions_subject_level.jsonl (metrics match)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="14" t="inlineStr">
+        <is>
+          <t>DAIC packed30 family</t>
+        </is>
+      </c>
+      <c r="B190" s="14" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C190" s="14" t="inlineStr">
+        <is>
+          <t>Joint-K4 Audio only</t>
+        </is>
+      </c>
+      <c r="D190" s="14" t="inlineStr">
         <is>
           <t>XGBoost raw</t>
         </is>
       </c>
-      <c r="E186" s="15" t="n">
+      <c r="E190" s="15" t="n">
         <v>0.2</v>
       </c>
-      <c r="F186" s="16" t="inlineStr">
+      <c r="F190" s="16" t="inlineStr">
         <is>
           <t>daic_participant_p30_jointk4_&lt;mod&gt;_s1337_e3b0f1c3 selected-epoch head fit (107 vectors, weights 1.0)</t>
         </is>
       </c>
-      <c r="G186" s="16" t="inlineStr">
+      <c r="G190" s="16" t="inlineStr">
         <is>
           <t>mean depressed probability &gt;= 0.5 per subject, 47 test subjects, 617 bundles</t>
         </is>
       </c>
-      <c r="H186" s="16" t="inlineStr">
-        <is>
-          <t>output_model/experiments/daic_participant_packed30_jointk4/&lt;modality&gt;/&lt;run&gt;/hidden_classifiers/audio_only/xgb_raw/</t>
-        </is>
-      </c>
-      <c r="I186" s="16" t="inlineStr">
-        <is>
-          <t>matched to audited hidden-classifier outputs</t>
+      <c r="H190" s="16" t="inlineStr">
+        <is>
+          <t>hidden_classifiers/audio_only/xgb_raw/</t>
+        </is>
+      </c>
+      <c r="I190" s="16" t="inlineStr">
+        <is>
+          <t>recomputed from predictions_subject_level.jsonl (metrics match)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook: fix hidden-head provenance run names; refresh hash pins
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -12793,7 +12793,7 @@
       </c>
       <c r="F192" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_daic_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G192" s="16" t="inlineStr">
@@ -12838,7 +12838,7 @@
       </c>
       <c r="F193" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_daic_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G193" s="16" t="inlineStr">
@@ -12928,7 +12928,7 @@
       </c>
       <c r="F195" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_daic_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G195" s="16" t="inlineStr">
@@ -12973,7 +12973,7 @@
       </c>
       <c r="F196" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_daic_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G196" s="16" t="inlineStr">
@@ -13063,7 +13063,7 @@
       </c>
       <c r="F198" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_daic_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G198" s="16" t="inlineStr">
@@ -13108,7 +13108,7 @@
       </c>
       <c r="F199" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_daic_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G199" s="16" t="inlineStr">
@@ -13198,7 +13198,7 @@
       </c>
       <c r="F201" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_cmdc_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G201" s="16" t="inlineStr">
@@ -13243,7 +13243,7 @@
       </c>
       <c r="F202" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_cmdc_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G202" s="16" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="F204" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_cmdc_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G204" s="16" t="inlineStr">
@@ -13378,7 +13378,7 @@
       </c>
       <c r="F205" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_cmdc_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G205" s="16" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F207" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_cmdc_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G207" s="16" t="inlineStr">
@@ -13513,7 +13513,7 @@
       </c>
       <c r="F208" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_cmdc_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G208" s="16" t="inlineStr">
@@ -13603,7 +13603,7 @@
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_turkish_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G210" s="16" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="F211" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_turkish_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G211" s="16" t="inlineStr">
@@ -13738,7 +13738,7 @@
       </c>
       <c r="F213" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_turkish_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G213" s="16" t="inlineStr">
@@ -13783,7 +13783,7 @@
       </c>
       <c r="F214" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_turkish_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G214" s="16" t="inlineStr">
@@ -13873,7 +13873,7 @@
       </c>
       <c r="F216" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_turkish_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G216" s="16" t="inlineStr">
@@ -13918,7 +13918,7 @@
       </c>
       <c r="F217" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_turkish_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G217" s="16" t="inlineStr">
@@ -14008,7 +14008,7 @@
       </c>
       <c r="F219" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_d3tec_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G219" s="16" t="inlineStr">
@@ -14053,7 +14053,7 @@
       </c>
       <c r="F220" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_d3tec_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G220" s="16" t="inlineStr">
@@ -14143,7 +14143,7 @@
       </c>
       <c r="F222" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_d3tec_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G222" s="16" t="inlineStr">
@@ -14188,7 +14188,7 @@
       </c>
       <c r="F223" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_d3tec_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G223" s="16" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="F225" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_d3tec_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G225" s="16" t="inlineStr">
@@ -14323,7 +14323,7 @@
       </c>
       <c r="F226" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_d3tec_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G226" s="16" t="inlineStr">
@@ -14413,7 +14413,7 @@
       </c>
       <c r="F228" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_androids_interview_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G228" s="16" t="inlineStr">
@@ -14458,7 +14458,7 @@
       </c>
       <c r="F229" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_text (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_androids_interview_audio_text (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G229" s="16" t="inlineStr">
@@ -14548,7 +14548,7 @@
       </c>
       <c r="F231" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_androids_interview_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G231" s="16" t="inlineStr">
@@ -14593,7 +14593,7 @@
       </c>
       <c r="F232" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_audio_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_androids_interview_audio_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G232" s="16" t="inlineStr">
@@ -14683,7 +14683,7 @@
       </c>
       <c r="F234" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_androids_interview_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G234" s="16" t="inlineStr">
@@ -14728,7 +14728,7 @@
       </c>
       <c r="F235" s="16" t="inlineStr">
         <is>
-          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_text_only (best-model hidden features)</t>
+          <t>harmonized_v1_harmonized_v1_prod_20260809T171705Z_d1e8130b_androids_interview_text_only (best-model hidden features, retry _r1 feature dirs)</t>
         </is>
       </c>
       <c r="G235" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Add Gemma 4 DAIC comparison sheet and workbook selection entries with provenance
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -13,7 +13,8 @@
     <sheet name="EN vs Native MacroF1" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Merged vs Standalone MacroF1" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="DAIC Packed30 Family" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Provenance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gemma 4 DAIC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Provenance" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5903,7 +5904,303 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I185"/>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Gemma 4 vs Qwen — DAIC official test (seed 1337, fold 0, strict teacher-forced)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Gemma 4: google/gemma-4-12B-it revision 707f0a3b8a3c…, BF16 LoRA (288 decoder modules, rank 16/alpha 32), SDPA, gradient checkpointing, batch 1 x 32 accum x 4 GPUs. Campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae; source a6749b05 (clean main); PR #31; same manifest/split as the Qwen harmonized campaign (72e2dd204b91…/441333e0c888…). Evaluation: original_teacher_forced, harmonized_all_windows_full_coverage, subject mean-score, headline/binary_strict, INVALID counts as wrong (INVALID=0). Qwen column = canonical harmonized _r1 DAIC rows. One seed each — differences are observations, not variance estimates. All values recomputed locally from predictions_subject_level.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Modality</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Macro-F1</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Positive-F1</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Run / attempt / jobs</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Local evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0.7631048387096775</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0.6875000000000001</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>0.7872340425531915</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2; attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805; train 44518086 eval 44518087 (COMPLETED 0:0); selected epoch 3</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_text/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Qwen (harmonized _r1)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0.7353</v>
+      </c>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>harmonized_v1_…_daic_audio_text_r1 (campaign harmonized_v1_prod_20260809T171705Z_d1e8130b; retry registry retry_r1_jobs.tsv)</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1/audio_text/daic/*/fold_0/best_model/standalone_eval(_r1)/metrics_original_teacher_forced.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0.7021276595744681</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only; attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2; train 44517565 eval 44517566 (COMPLETED 0:0); selected epoch n/a</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Qwen (harmonized _r1)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.5392</v>
+      </c>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>harmonized_v1_…_daic_audio_only_r1 (campaign harmonized_v1_prod_20260809T171705Z_d1e8130b; retry registry retry_r1_jobs.tsv)</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1/audio_only/daic/*/fold_0/best_model/standalone_eval(_r1)/metrics_original_teacher_forced.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0.7552083333333333</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.7872340425531915</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only; attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3; train 44517484 eval 44517485 (COMPLETED 0:0); selected epoch 1</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Qwen (harmonized _r1)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0.7353</v>
+      </c>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>harmonized_v1_…_daic_text_only_r1 (campaign harmonized_v1_prod_20260809T171705Z_d1e8130b; retry registry retry_r1_jobs.tsv)</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1/text_only/daic/*/fold_0/best_model/standalone_eval(_r1)/metrics_original_teacher_forced.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Positive-F1/accuracy/precision/recall are shown for Gemma only; the Qwen harmonized rows in the workbook carry macro-F1 (STANDALONE_QWEN) and the same binary-strict headline semantics (values: DAIC audio+text 0.7353, audio-only 0.5392, text-only 0.7353). audio_only Gemma predicted Non-depressed for all 47 subjects (degenerate but valid; run and evidence are sound). No winner is selected from test results.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14206,6 +14503,687 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B186" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C186" s="15" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D186" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 macro-F1</t>
+        </is>
+      </c>
+      <c r="E186" s="16" t="n">
+        <v>0.7631048387096775</v>
+      </c>
+      <c r="F186" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2, attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, source a6749b05 (clean main), PR #31, jobs 44518086/44518087, selected epoch 3, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G186" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H186" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_text/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I186" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON); Slurm COMPLETED 0:0</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B187" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C187" s="15" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D187" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 positive-F1</t>
+        </is>
+      </c>
+      <c r="E187" s="16" t="n">
+        <v>0.6875000000000001</v>
+      </c>
+      <c r="F187" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2, attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, source a6749b05 (clean main), PR #31, jobs 44518086/44518087, selected epoch 3, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G187" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H187" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_text/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I187" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B188" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C188" s="15" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D188" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 accuracy</t>
+        </is>
+      </c>
+      <c r="E188" s="16" t="n">
+        <v>0.7872340425531915</v>
+      </c>
+      <c r="F188" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2, attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, source a6749b05 (clean main), PR #31, jobs 44518086/44518087, selected epoch 3, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G188" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H188" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_text/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I188" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B189" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C189" s="15" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D189" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 confusion matrix</t>
+        </is>
+      </c>
+      <c r="E189" s="15" t="inlineStr">
+        <is>
+          <t>[[26, 7], [3, 11]]</t>
+        </is>
+      </c>
+      <c r="F189" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2, attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, source a6749b05 (clean main), PR #31, jobs 44518086/44518087, selected epoch 3, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G189" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H189" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_text/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2/fold_0/best_model/standalone_eval/confusion_matrix.json</t>
+        </is>
+      </c>
+      <c r="I189" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B190" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C190" s="15" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D190" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 invalid count</t>
+        </is>
+      </c>
+      <c r="E190" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F190" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2, attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, source a6749b05 (clean main), PR #31, jobs 44518086/44518087, selected epoch 3, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G190" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H190" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_text/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_text_r2/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+        </is>
+      </c>
+      <c r="I190" s="17" t="inlineStr">
+        <is>
+          <t>invalid_subjects == 0 in metrics JSON and recomputation</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B191" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C191" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D191" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 macro-F1</t>
+        </is>
+      </c>
+      <c r="E191" s="16" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="F191" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch n/a, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G191" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H191" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I191" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON); Slurm COMPLETED 0:0</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B192" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C192" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D192" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 positive-F1</t>
+        </is>
+      </c>
+      <c r="E192" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F192" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch n/a, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G192" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H192" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I192" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B193" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C193" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D193" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 accuracy</t>
+        </is>
+      </c>
+      <c r="E193" s="16" t="n">
+        <v>0.7021276595744681</v>
+      </c>
+      <c r="F193" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch n/a, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G193" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H193" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I193" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B194" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C194" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D194" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 confusion matrix</t>
+        </is>
+      </c>
+      <c r="E194" s="15" t="inlineStr">
+        <is>
+          <t>[[33, 0], [14, 0]]</t>
+        </is>
+      </c>
+      <c r="F194" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch n/a, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G194" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H194" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/confusion_matrix.json</t>
+        </is>
+      </c>
+      <c r="I194" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B195" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C195" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D195" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 invalid count</t>
+        </is>
+      </c>
+      <c r="E195" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F195" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch n/a, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G195" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H195" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+        </is>
+      </c>
+      <c r="I195" s="17" t="inlineStr">
+        <is>
+          <t>invalid_subjects == 0 in metrics JSON and recomputation</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B196" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C196" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D196" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 macro-F1</t>
+        </is>
+      </c>
+      <c r="E196" s="16" t="n">
+        <v>0.7552083333333333</v>
+      </c>
+      <c r="F196" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G196" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H196" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I196" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON); Slurm COMPLETED 0:0</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B197" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C197" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D197" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 positive-F1</t>
+        </is>
+      </c>
+      <c r="E197" s="16" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F197" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G197" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H197" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I197" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B198" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C198" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D198" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 accuracy</t>
+        </is>
+      </c>
+      <c r="E198" s="16" t="n">
+        <v>0.7872340425531915</v>
+      </c>
+      <c r="F198" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G198" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H198" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I198" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B199" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C199" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D199" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 confusion matrix</t>
+        </is>
+      </c>
+      <c r="E199" s="15" t="inlineStr">
+        <is>
+          <t>[[27, 6], [4, 10]]</t>
+        </is>
+      </c>
+      <c r="F199" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G199" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H199" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/confusion_matrix.json</t>
+        </is>
+      </c>
+      <c r="I199" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B200" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C200" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D200" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 invalid count</t>
+        </is>
+      </c>
+      <c r="E200" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F200" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G200" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H200" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+        </is>
+      </c>
+      <c r="I200" s="17" t="inlineStr">
+        <is>
+          <t>invalid_subjects == 0 in metrics JSON and recomputation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
Record run_config/source_manifest artifacts, post-hoc W&B history, hidden-classifier evidence checks
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -5904,7 +5904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5987,7 +5987,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Gemma 4</t>
+          <t>Gemma 4 teacher-forced head</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
@@ -6024,169 +6024,391 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Qwen (harmonized _r1)</t>
+          <t>Gemma 4 LogReg raw hidden head</t>
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>0.7353</v>
-      </c>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
+        <v>0.7898658718330849</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0.7272727272727273</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0.8085106382978723</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0.631578947368421</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0.8571428571428571</v>
+      </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>harmonized_v1_…_daic_audio_text_r1 (campaign harmonized_v1_prod_20260809T171705Z_d1e8130b; retry registry retry_r1_jobs.tsv)</t>
+          <t>run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412; attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728; extract 44538980 heads 44538981 (COMPLETED 0:0); backend gemma4_hidden_logreg_raw; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0 / heads CANCELLED, wrapper race fixed in PR #45)</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1/audio_text/daic/*/fold_0/best_model/standalone_eval(_r1)/metrics_original_teacher_forced.json</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0.7834101382488479</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0.7096774193548386</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.8085106382978723</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.6470588235294118</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412; attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728; extract 44538980 heads 44538981 (COMPLETED 0:0); backend gemma4_hidden_xgb_raw; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0 / heads CANCELLED, wrapper race fixed in PR #45)</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Qwen harmonized _r1 reference</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0.7353</v>
+      </c>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>harmonized_v1_…_daic_audio_text_r1 (campaign harmonized_v1_prod_20260809T171705Z_d1e8130b; retry registry retry_r1_jobs.tsv)</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1/audio_text/daic/*/fold_0/best_model/standalone_eval(_r1)/metrics_original_teacher_forced.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>Audio only</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Gemma 4</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4 teacher-forced head</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
         <v>0.4125</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E10" s="5" t="n">
         <v>0.7021276595744681</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="9" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only; attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2; train 44517565 eval 44517566 (COMPLETED 0:0); selected epoch 1</t>
         </is>
       </c>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="I10" s="9" t="inlineStr">
         <is>
           <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Audio only</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Qwen (harmonized _r1)</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>0.5392</v>
-      </c>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>harmonized_v1_…_daic_audio_only_r1 (campaign harmonized_v1_prod_20260809T171705Z_d1e8130b; retry registry retry_r1_jobs.tsv)</t>
-        </is>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>output_model/harmonized_v1/audio_only/daic/*/fold_0/best_model/standalone_eval(_r1)/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Gemma 4</t>
+          <t>Gemma 4 LogReg raw hidden head</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.7552083333333333</v>
+        <v>0.6258420085731782</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4347826086956522</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.7872340425531915</v>
+        <v>0.723404255319149</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.625</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only; attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3; train 44517484 eval 44517485 (COMPLETED 0:0); selected epoch 1</t>
+          <t>run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412; attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d; extract 44538982 heads 44538983 (COMPLETED 0:0); backend gemma4_hidden_logreg_raw; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0 / heads CANCELLED, wrapper race fixed in PR #45)</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0.7021276595744681</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412; attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d; extract 44538982 heads 44538983 (COMPLETED 0:0); backend gemma4_hidden_xgb_raw; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0 / heads CANCELLED, wrapper race fixed in PR #45)</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Qwen harmonized _r1 reference</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0.5392</v>
+      </c>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>harmonized_v1_…_daic_audio_only_r1 (campaign harmonized_v1_prod_20260809T171705Z_d1e8130b; retry registry retry_r1_jobs.tsv)</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1/audio_only/daic/*/fold_0/best_model/standalone_eval(_r1)/metrics_original_teacher_forced.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>Text only</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Qwen (harmonized _r1)</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="n">
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4 teacher-forced head</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0.7552083333333333</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0.7872340425531915</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only; attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3; train 44517484 eval 44517485 (COMPLETED 0:0); selected epoch 1</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>0.70625</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>0.7446808510638298</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412; attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58; extract 44538984 heads 44538985 (COMPLETED 0:0); backend gemma4_hidden_logreg_raw; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0 / heads CANCELLED, wrapper race fixed in PR #45)</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0.6948051948051948</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0.7446808510638298</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412; attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58; extract 44538984 heads 44538985 (COMPLETED 0:0); backend gemma4_hidden_xgb_raw; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0 / heads CANCELLED, wrapper race fixed in PR #45)</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Qwen harmonized _r1 reference</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
         <v>0.7353</v>
       </c>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="9" t="inlineStr">
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>harmonized_v1_…_daic_text_only_r1 (campaign harmonized_v1_prod_20260809T171705Z_d1e8130b; retry registry retry_r1_jobs.tsv)</t>
         </is>
       </c>
-      <c r="I12" s="9" t="inlineStr">
+      <c r="I18" s="9" t="inlineStr">
         <is>
           <t>output_model/harmonized_v1/text_only/daic/*/fold_0/best_model/standalone_eval(_r1)/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Positive-F1/accuracy/precision/recall are shown for Gemma only; the Qwen harmonized rows in the workbook carry macro-F1 (STANDALONE_QWEN) and the same binary-strict headline semantics (values: DAIC audio+text 0.7353, audio-only 0.5392, text-only 0.7353). audio_only Gemma predicted Non-depressed for all 47 subjects (degenerate but valid; run and evidence are sound). No winner is selected from test results.</t>
+    <row r="20" ht="110" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Fixed heads: final prompt-token hidden state (float32, 3840) from each Gemma 4 best_model; fit on the saved 107 official training subjects only (audio modes: all packed30 chunks, inverse-chunk weights; text: one vector per subject); test = official 47 subjects, mean depressed probability over chunks at &gt;= 0.5. LogReg: StandardScaler + balanced liblinear C=1.0 max_iter=5000; XGBoost: 300 trees lr 0.03 depth 2 min_child_weight 5 subsample 0.8 colsample 0.25 alpha 1.0 lambda 10.0 hist n_jobs=1; both seed 1337, sklearn 1.7.0 / xgboost 2.1.4. One seed each — differences are observations, not variance estimates. No winner is selected from test results.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -6200,7 +6422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I200"/>
+  <dimension ref="A1:I236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14743,35 +14965,35 @@
       </c>
       <c r="C191" s="15" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D191" s="15" t="inlineStr">
         <is>
-          <t>Gemma 4 macro-F1</t>
+          <t>Gemma 4 LogReg raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E191" s="16" t="n">
-        <v>0.4125</v>
+        <v>0.7898658718330849</v>
       </c>
       <c r="F191" s="17" t="inlineStr">
         <is>
-          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
         </is>
       </c>
       <c r="G191" s="17" t="inlineStr">
         <is>
-          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
         </is>
       </c>
       <c r="H191" s="17" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I191" s="17" t="inlineStr">
         <is>
-          <t>recomputed locally from predictions (matches metrics JSON); Slurm COMPLETED 0:0</t>
+          <t>recomputed locally by verify-local (matches metrics JSON); REPORTABLE</t>
         </is>
       </c>
     </row>
@@ -14788,35 +15010,35 @@
       </c>
       <c r="C192" s="15" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D192" s="15" t="inlineStr">
         <is>
-          <t>Gemma 4 positive-F1</t>
+          <t>Gemma 4 LogReg raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E192" s="16" t="n">
-        <v>0</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="F192" s="17" t="inlineStr">
         <is>
-          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
         </is>
       </c>
       <c r="G192" s="17" t="inlineStr">
         <is>
-          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
         </is>
       </c>
       <c r="H192" s="17" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I192" s="17" t="inlineStr">
         <is>
-          <t>recomputed locally from predictions (matches metrics JSON)</t>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
         </is>
       </c>
     </row>
@@ -14833,35 +15055,35 @@
       </c>
       <c r="C193" s="15" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D193" s="15" t="inlineStr">
         <is>
-          <t>Gemma 4 accuracy</t>
+          <t>Gemma 4 LogReg raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E193" s="16" t="n">
-        <v>0.7021276595744681</v>
+        <v>0.8085106382978723</v>
       </c>
       <c r="F193" s="17" t="inlineStr">
         <is>
-          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
         </is>
       </c>
       <c r="G193" s="17" t="inlineStr">
         <is>
-          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
         </is>
       </c>
       <c r="H193" s="17" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I193" s="17" t="inlineStr">
         <is>
-          <t>recomputed locally from predictions (matches metrics JSON)</t>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
         </is>
       </c>
     </row>
@@ -14878,37 +15100,35 @@
       </c>
       <c r="C194" s="15" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D194" s="15" t="inlineStr">
         <is>
-          <t>Gemma 4 confusion matrix</t>
-        </is>
-      </c>
-      <c r="E194" s="15" t="inlineStr">
-        <is>
-          <t>[[33, 0], [14, 0]]</t>
-        </is>
+          <t>Gemma 4 LogReg raw hidden head precision</t>
+        </is>
+      </c>
+      <c r="E194" s="16" t="n">
+        <v>0.631578947368421</v>
       </c>
       <c r="F194" s="17" t="inlineStr">
         <is>
-          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
         </is>
       </c>
       <c r="G194" s="17" t="inlineStr">
         <is>
-          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
         </is>
       </c>
       <c r="H194" s="17" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/confusion_matrix.json</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I194" s="17" t="inlineStr">
         <is>
-          <t>recomputed locally from predictions (matches metrics JSON)</t>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
         </is>
       </c>
     </row>
@@ -14925,35 +15145,35 @@
       </c>
       <c r="C195" s="15" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D195" s="15" t="inlineStr">
         <is>
-          <t>Gemma 4 invalid count</t>
-        </is>
-      </c>
-      <c r="E195" s="15" t="n">
-        <v>0</v>
+          <t>Gemma 4 LogReg raw hidden head recall</t>
+        </is>
+      </c>
+      <c r="E195" s="16" t="n">
+        <v>0.8571428571428571</v>
       </c>
       <c r="F195" s="17" t="inlineStr">
         <is>
-          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
         </is>
       </c>
       <c r="G195" s="17" t="inlineStr">
         <is>
-          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
         </is>
       </c>
       <c r="H195" s="17" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I195" s="17" t="inlineStr">
         <is>
-          <t>invalid_subjects == 0 in metrics JSON and recomputation</t>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
         </is>
       </c>
     </row>
@@ -14970,35 +15190,37 @@
       </c>
       <c r="C196" s="15" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D196" s="15" t="inlineStr">
         <is>
-          <t>Gemma 4 macro-F1</t>
-        </is>
-      </c>
-      <c r="E196" s="16" t="n">
-        <v>0.7552083333333333</v>
+          <t>Gemma 4 LogReg raw hidden head confusion matrix</t>
+        </is>
+      </c>
+      <c r="E196" s="15" t="inlineStr">
+        <is>
+          <t>[[26, 7], [2, 12]]</t>
+        </is>
       </c>
       <c r="F196" s="17" t="inlineStr">
         <is>
-          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
         </is>
       </c>
       <c r="G196" s="17" t="inlineStr">
         <is>
-          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
         </is>
       </c>
       <c r="H196" s="17" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json</t>
         </is>
       </c>
       <c r="I196" s="17" t="inlineStr">
         <is>
-          <t>recomputed locally from predictions (matches metrics JSON); Slurm COMPLETED 0:0</t>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
         </is>
       </c>
     </row>
@@ -15015,35 +15237,35 @@
       </c>
       <c r="C197" s="15" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D197" s="15" t="inlineStr">
         <is>
-          <t>Gemma 4 positive-F1</t>
+          <t>Gemma 4 XGBoost raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E197" s="16" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7834101382488479</v>
       </c>
       <c r="F197" s="17" t="inlineStr">
         <is>
-          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
         </is>
       </c>
       <c r="G197" s="17" t="inlineStr">
         <is>
-          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
         </is>
       </c>
       <c r="H197" s="17" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I197" s="17" t="inlineStr">
         <is>
-          <t>recomputed locally from predictions (matches metrics JSON)</t>
+          <t>recomputed locally by verify-local (matches metrics JSON); REPORTABLE</t>
         </is>
       </c>
     </row>
@@ -15060,35 +15282,35 @@
       </c>
       <c r="C198" s="15" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D198" s="15" t="inlineStr">
         <is>
-          <t>Gemma 4 accuracy</t>
+          <t>Gemma 4 XGBoost raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E198" s="16" t="n">
-        <v>0.7872340425531915</v>
+        <v>0.7096774193548386</v>
       </c>
       <c r="F198" s="17" t="inlineStr">
         <is>
-          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
         </is>
       </c>
       <c r="G198" s="17" t="inlineStr">
         <is>
-          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
         </is>
       </c>
       <c r="H198" s="17" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I198" s="17" t="inlineStr">
         <is>
-          <t>recomputed locally from predictions (matches metrics JSON)</t>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
         </is>
       </c>
     </row>
@@ -15105,37 +15327,35 @@
       </c>
       <c r="C199" s="15" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D199" s="15" t="inlineStr">
         <is>
-          <t>Gemma 4 confusion matrix</t>
-        </is>
-      </c>
-      <c r="E199" s="15" t="inlineStr">
-        <is>
-          <t>[[27, 6], [4, 10]]</t>
-        </is>
+          <t>Gemma 4 XGBoost raw hidden head accuracy</t>
+        </is>
+      </c>
+      <c r="E199" s="16" t="n">
+        <v>0.8085106382978723</v>
       </c>
       <c r="F199" s="17" t="inlineStr">
         <is>
-          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
         </is>
       </c>
       <c r="G199" s="17" t="inlineStr">
         <is>
-          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
         </is>
       </c>
       <c r="H199" s="17" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/confusion_matrix.json</t>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I199" s="17" t="inlineStr">
         <is>
-          <t>recomputed locally from predictions (matches metrics JSON)</t>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
         </is>
       </c>
     </row>
@@ -15152,35 +15372,1669 @@
       </c>
       <c r="C200" s="15" t="inlineStr">
         <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D200" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head precision</t>
+        </is>
+      </c>
+      <c r="E200" s="16" t="n">
+        <v>0.6470588235294118</v>
+      </c>
+      <c r="F200" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G200" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H200" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I200" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B201" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C201" s="15" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D201" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head recall</t>
+        </is>
+      </c>
+      <c r="E201" s="16" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="F201" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G201" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H201" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I201" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B202" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C202" s="15" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D202" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head confusion matrix</t>
+        </is>
+      </c>
+      <c r="E202" s="15" t="inlineStr">
+        <is>
+          <t>[[27, 6], [3, 11]]</t>
+        </is>
+      </c>
+      <c r="F202" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155659Z-gemma4_daic_audio_text_fixed_heads_20260812t155635z_799cc412-799cc412-5ad76728, source 799cc412 (clean main), PR #46, jobs 44538980/44538981 (COMPLETED 0:0), parent attempt 20260812T031624Z-gemma4_daic_audio_text_seed1337-a6749b05-146c8805, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153613Z-gemma4_daic_audio_text_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-a739f168 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G202" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H202" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_text/daic/gemma4_daic_audio_text_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json</t>
+        </is>
+      </c>
+      <c r="I202" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B203" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C203" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D203" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 macro-F1</t>
+        </is>
+      </c>
+      <c r="E203" s="16" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="F203" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G203" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H203" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I203" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON); Slurm COMPLETED 0:0</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B204" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C204" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D204" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 positive-F1</t>
+        </is>
+      </c>
+      <c r="E204" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F204" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G204" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H204" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I204" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B205" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C205" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D205" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 accuracy</t>
+        </is>
+      </c>
+      <c r="E205" s="16" t="n">
+        <v>0.7021276595744681</v>
+      </c>
+      <c r="F205" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G205" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H205" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I205" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B206" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C206" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D206" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 confusion matrix</t>
+        </is>
+      </c>
+      <c r="E206" s="15" t="inlineStr">
+        <is>
+          <t>[[33, 0], [14, 0]]</t>
+        </is>
+      </c>
+      <c r="F206" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G206" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H206" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/confusion_matrix.json</t>
+        </is>
+      </c>
+      <c r="I206" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B207" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C207" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D207" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 invalid count</t>
+        </is>
+      </c>
+      <c r="E207" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F207" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only, attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, source a6749b05 (clean main), PR #31, jobs 44517565/44517566, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G207" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H207" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/audio_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_audio_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+        </is>
+      </c>
+      <c r="I207" s="17" t="inlineStr">
+        <is>
+          <t>invalid_subjects == 0 in metrics JSON and recomputation</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B208" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C208" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D208" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head macro-F1</t>
+        </is>
+      </c>
+      <c r="E208" s="16" t="n">
+        <v>0.6258420085731782</v>
+      </c>
+      <c r="F208" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G208" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H208" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I208" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON); REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B209" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C209" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D209" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head positive-F1</t>
+        </is>
+      </c>
+      <c r="E209" s="16" t="n">
+        <v>0.4347826086956522</v>
+      </c>
+      <c r="F209" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G209" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H209" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I209" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B210" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C210" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D210" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head accuracy</t>
+        </is>
+      </c>
+      <c r="E210" s="16" t="n">
+        <v>0.723404255319149</v>
+      </c>
+      <c r="F210" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G210" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H210" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I210" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B211" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C211" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D211" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head precision</t>
+        </is>
+      </c>
+      <c r="E211" s="16" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="F211" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G211" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H211" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I211" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B212" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C212" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D212" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head recall</t>
+        </is>
+      </c>
+      <c r="E212" s="16" t="n">
+        <v>0.3571428571428572</v>
+      </c>
+      <c r="F212" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G212" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H212" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I212" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B213" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C213" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D213" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head confusion matrix</t>
+        </is>
+      </c>
+      <c r="E213" s="15" t="inlineStr">
+        <is>
+          <t>[[29, 4], [9, 5]]</t>
+        </is>
+      </c>
+      <c r="F213" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G213" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H213" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json</t>
+        </is>
+      </c>
+      <c r="I213" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B214" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C214" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D214" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head macro-F1</t>
+        </is>
+      </c>
+      <c r="E214" s="16" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="F214" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G214" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H214" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I214" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON); REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B215" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C215" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D215" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head positive-F1</t>
+        </is>
+      </c>
+      <c r="E215" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F215" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G215" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H215" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I215" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B216" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C216" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D216" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head accuracy</t>
+        </is>
+      </c>
+      <c r="E216" s="16" t="n">
+        <v>0.7021276595744681</v>
+      </c>
+      <c r="F216" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G216" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H216" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I216" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B217" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C217" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D217" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head precision</t>
+        </is>
+      </c>
+      <c r="E217" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F217" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G217" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H217" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I217" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B218" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C218" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D218" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head recall</t>
+        </is>
+      </c>
+      <c r="E218" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F218" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G218" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H218" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I218" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B219" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C219" s="15" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D219" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head confusion matrix</t>
+        </is>
+      </c>
+      <c r="E219" s="15" t="inlineStr">
+        <is>
+          <t>[[33, 0], [14, 0]]</t>
+        </is>
+      </c>
+      <c r="F219" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155701Z-gemma4_daic_audio_only_fixed_heads_20260812t155635z_799cc412-799cc412-4fafe36d, source 799cc412 (clean main), PR #46, jobs 44538982/44538983 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_audio_only_seed1337-cca3f4ae-8789edf2, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153615Z-gemma4_daic_audio_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-f9cac152 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G219" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H219" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/audio_only/daic/gemma4_daic_audio_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json</t>
+        </is>
+      </c>
+      <c r="I219" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B220" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C220" s="15" t="inlineStr">
+        <is>
           <t>Text only</t>
         </is>
       </c>
-      <c r="D200" s="15" t="inlineStr">
+      <c r="D220" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 macro-F1</t>
+        </is>
+      </c>
+      <c r="E220" s="16" t="n">
+        <v>0.7552083333333333</v>
+      </c>
+      <c r="F220" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G220" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H220" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I220" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON); Slurm COMPLETED 0:0</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B221" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C221" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D221" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 positive-F1</t>
+        </is>
+      </c>
+      <c r="E221" s="16" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F221" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G221" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H221" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I221" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B222" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C222" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D222" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 accuracy</t>
+        </is>
+      </c>
+      <c r="E222" s="16" t="n">
+        <v>0.7872340425531915</v>
+      </c>
+      <c r="F222" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G222" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H222" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I222" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B223" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C223" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D223" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 confusion matrix</t>
+        </is>
+      </c>
+      <c r="E223" s="15" t="inlineStr">
+        <is>
+          <t>[[27, 6], [4, 10]]</t>
+        </is>
+      </c>
+      <c r="F223" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
+        </is>
+      </c>
+      <c r="G223" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+        </is>
+      </c>
+      <c r="H223" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/confusion_matrix.json</t>
+        </is>
+      </c>
+      <c r="I223" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B224" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C224" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D224" s="15" t="inlineStr">
         <is>
           <t>Gemma 4 invalid count</t>
         </is>
       </c>
-      <c r="E200" s="15" t="n">
+      <c r="E224" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F200" s="17" t="inlineStr">
+      <c r="F224" s="17" t="inlineStr">
         <is>
           <t>campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae, run gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only, attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, source a6749b05 (clean main), PR #31, jobs 44517484/44517485, selected epoch 1, model google/gemma-4-12B-it rev 707f0a3b8a3c…, cfg/manifest/split 72e2dd204b91…/441333e0c888…</t>
         </is>
       </c>
-      <c r="G200" s="17" t="inlineStr">
+      <c r="G224" s="17" t="inlineStr">
         <is>
           <t>official 47-subject test, subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
-      <c r="H200" s="17" t="inlineStr">
+      <c r="H224" s="17" t="inlineStr">
         <is>
           <t>output_model/harmonized_v1_gemma4/text_only/daic/gemma4_harmonized_v1_gemma4_v1_prod_20260812T020449Z_cca3f4ae_daic_text_only/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
-      <c r="I200" s="17" t="inlineStr">
+      <c r="I224" s="17" t="inlineStr">
         <is>
           <t>invalid_subjects == 0 in metrics JSON and recomputation</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B225" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C225" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D225" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head macro-F1</t>
+        </is>
+      </c>
+      <c r="E225" s="16" t="n">
+        <v>0.70625</v>
+      </c>
+      <c r="F225" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G225" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H225" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I225" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON); REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B226" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C226" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D226" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head positive-F1</t>
+        </is>
+      </c>
+      <c r="E226" s="16" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="F226" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G226" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H226" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I226" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B227" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C227" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D227" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head accuracy</t>
+        </is>
+      </c>
+      <c r="E227" s="16" t="n">
+        <v>0.7446808510638298</v>
+      </c>
+      <c r="F227" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G227" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H227" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I227" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B228" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C228" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D228" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head precision</t>
+        </is>
+      </c>
+      <c r="E228" s="16" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="F228" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G228" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H228" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I228" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B229" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C229" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D229" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head recall</t>
+        </is>
+      </c>
+      <c r="E229" s="16" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="F229" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G229" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H229" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I229" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B230" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C230" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D230" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head confusion matrix</t>
+        </is>
+      </c>
+      <c r="E230" s="15" t="inlineStr">
+        <is>
+          <t>[[26, 7], [5, 9]]</t>
+        </is>
+      </c>
+      <c r="F230" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_logreg_raw</t>
+        </is>
+      </c>
+      <c r="G230" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H230" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/logreg/metrics.json</t>
+        </is>
+      </c>
+      <c r="I230" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B231" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C231" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D231" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head macro-F1</t>
+        </is>
+      </c>
+      <c r="E231" s="16" t="n">
+        <v>0.6948051948051948</v>
+      </c>
+      <c r="F231" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G231" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H231" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I231" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON); REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B232" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C232" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D232" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head positive-F1</t>
+        </is>
+      </c>
+      <c r="E232" s="16" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="F232" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G232" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H232" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I232" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B233" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C233" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D233" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head accuracy</t>
+        </is>
+      </c>
+      <c r="E233" s="16" t="n">
+        <v>0.7446808510638298</v>
+      </c>
+      <c r="F233" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G233" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H233" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I233" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B234" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C234" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D234" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head precision</t>
+        </is>
+      </c>
+      <c r="E234" s="16" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="F234" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G234" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H234" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I234" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B235" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C235" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D235" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head recall</t>
+        </is>
+      </c>
+      <c r="E235" s="16" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="F235" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G235" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H235" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I235" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 DAIC</t>
+        </is>
+      </c>
+      <c r="B236" s="15" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C236" s="15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D236" s="15" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head confusion matrix</t>
+        </is>
+      </c>
+      <c r="E236" s="15" t="inlineStr">
+        <is>
+          <t>[[27, 6], [6, 8]]</t>
+        </is>
+      </c>
+      <c r="F236" s="17" t="inlineStr">
+        <is>
+          <t>campaign gemma4-daic-fixed-heads-v1-799cc412, run gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412, attempt 20260812T155703Z-gemma4_daic_text_only_fixed_heads_20260812t155635z_799cc412-799cc412-735f2c58, source 799cc412 (clean main), PR #46, jobs 44538984/44538985 (COMPLETED 0:0), parent attempt 20260812T020449Z-gemma4_daic_text_only_seed1337-cca3f4ae-ed58a7a3, parent adapter 72e2dd204b91…/… split 441333e0c888…, model google/gemma-4-12B-it rev 707f0a3b8a3c…; supersedes 20260812T153617Z-gemma4_daic_text_only_fixed_heads_20260812t153611z_dcfaa142-dcfaa142-066f6db6 (extract FAILED 1:0, heads CANCELLED, wrapper race fixed in PR #45), backend gemma4_hidden_xgb_raw</t>
+        </is>
+      </c>
+      <c r="G236" s="17" t="inlineStr">
+        <is>
+          <t>official 47-subject test, subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_fit_locked_test_evaluation</t>
+        </is>
+      </c>
+      <c r="H236" s="17" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_heads/text_only/daic/gemma4_daic_text_only_fixed_heads_20260812T155635Z_799cc412/fold_0/hidden_classifiers/xgb/metrics.json</t>
+        </is>
+      </c>
+      <c r="I236" s="17" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local (matches metrics JSON)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Gemma vs Qwen DAIC comparison sheet to clean workbook
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Merged vs Standalone MacroF1" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="DAIC Packed30 Family" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Gemma 4 DAIC" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Provenance" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gemma vs Qwen" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Provenance" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6422,6 +6423,269 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Gemma 4 vs Qwen — DAIC official test, macro-F1 (seed 1337, fold 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Macro-F1, binary-strict, best_model, official 47-subject DAIC test. Qwen: harmonized campaign harmonized_v1_prod_20260809T171705Z_d1e8130b (teacher-forced row = Fine-tuned Qwen STANDALONE_QWEN; head rows = harmonized hidden-state heads STANDALONE_HEADS, pooled subject-level). Gemma: campaign gemma4_v1_prod_20260812T020449Z_cca3f4ae (teacher-forced GEMMA4_QWEN, subject mean-score) and fixed-head campaign gemma4-daic-fixed-heads-v1-799cc412 (GEMMA4_HEADS, subject mean probability &gt;= 0.5). One seed each — differences are observations, not variance estimates. Delta = Gemma minus Qwen. Provenance: Provenance sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Modality</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Qwen macro-F1</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Gemma macro-F1</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Δ (Gemma − Qwen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0.7353</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0.7631048387096775</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0.0278</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>LogReg raw hidden head</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0.7432</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0.7898658718330849</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0.0467</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>XGBoost raw hidden head</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0.7353</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0.7834101382488479</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0.0481</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0.5392</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>-0.1267</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>LogReg raw hidden head</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.5583</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.6258420085731782</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>0.0675</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>XGBoost raw hidden head</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0.519</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-0.1065</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0.7353</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.7552083333333333</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>0.0199</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>LogReg raw hidden head</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0.7235</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0.70625</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>-0.0172</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>XGBoost raw hidden head</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0.7457</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0.6948051948051948</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>-0.0509</v>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Teacher-forced = backbone classification without hidden-state heads. Hidden heads classify the final prompt-token hidden state with the locked LogReg/XGBoost implementations. See the 'Gemma 4 DAIC' and 'Summary' sheets for the full metric sets and per-cell provenance.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A14:E14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Add Optuna-100 workbook structure, selections, and safe W&B entries
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -15,9 +15,10 @@
     <sheet name="DAIC Packed30 Family" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Gemma 4 DAIC" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Gemma vs Qwen" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="DAIC LLM Comparison" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="DAIC Head Ablation" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Provenance" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Optuna-100 XGB" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="DAIC LLM Comparison" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="DAIC Head Ablation" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Provenance" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -836,6 +837,557 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DAIC-WOZ LLM literature comparison — official development partition (35 subjects)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Cited literature (DAIC official development partition)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Study</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Backbone</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Modality</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Macro-F1</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Partition</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Comparability</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DepresInstruct (Li et al., 2025)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Qwen2-Audio-7B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.6667</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.7714</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>DAIC development</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>C — reported as F1; shown as Macro-F1 per researcher decision</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.inffus.2025.104077</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DepresInstruct (Li et al., 2025)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Qwen2-7B</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.7272999999999999</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.7429</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DAIC development</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>C — reported as F1; shown as Macro-F1 per researcher decision</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.inffus.2025.104077</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DepresInstruct (Li et al., 2025)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Qwen2-Audio-7B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.7619</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.8571</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>DAIC development</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>C — reported as F1; shown as Macro-F1 per researcher decision</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.inffus.2025.104077</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IT HEARS — Qwen2-7B baseline</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Qwen2-7B</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>DAIC development</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>C — paper reports F1; baseline; no validation/accuracy reported</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2511.19877</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IT HEARS — Qwen2-Audio-7B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Qwen2-Audio-7B</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>DAIC development</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>C — paper reports F1; no validation/accuracy reported</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2511.19877</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Ours — official development (35 subjects, seed 1337, fold 0, best_model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Backbone</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Modality</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Macro-F1</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Positive-F1</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Selected epoch</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Gemma 4 12B IT</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>0.396551724137931</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>0.6571428571428571</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>35</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_officialdev/audio_only/daic/daic_officialdev_gemma4_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions; attempt 20260813T142848Z-dai…</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>0.3859649122807018</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>0.6285714285714286</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7</v>
+      </c>
+      <c r="G12" t="n">
+        <v>35</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_officialdev/audio_only/daic/daic_officialdev_qwen_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions; attempt 20260813T142847Z-dai…</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gemma 4 12B IT</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>0.7552447552447553</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>0.6923076923076924</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>0.7714285714285715</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" t="n">
+        <v>35</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_officialdev/audio_text/daic/daic_officialdev_gemma4_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions; attempt 20260813T142848Z-dai…</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>0.6258503401360545</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>0.4761904761904762</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0.6857142857142857</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" t="n">
+        <v>35</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_officialdev/audio_text/daic/daic_officialdev_qwen_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions; attempt 20260813T142848Z-dai…</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Gemma 4 12B IT</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>0.7822222222222222</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>0.7199999999999999</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>35</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_officialdev/text_only/daic/daic_officialdev_gemma4_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions; attempt 20260813T142849Z-dai…</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>0.7086031452358927</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>0.6086956521739131</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>0.7428571428571429</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>35</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_officialdev/text_only/daic/daic_officialdev_qwen_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>recomputed locally from predictions; attempt 20260813T142848Z-dai…</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1734,7 +2286,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21733,546 +22285,1961 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DAIC-WOZ LLM literature comparison — official development partition (35 subjects)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Cited literature (DAIC official development partition)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Study</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Backbone</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+          <t>Standardized Optuna-100 XGBoost — macro-F1 (not run yet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="90" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Protocol harmonized_optuna100_v1: exactly 100 TPE trials, seeds 1337/1337/1337, 3 subject-grouped inner folds, threshold 0.5, sampling none, pooled inner subject-level macro-F1 objective (merged: unweighted mean of five per-dataset inner macro-F1). Prediction backends qwen_hidden_xgb_optuna100 / gemma4_hidden_xgb_optuna100 (+ _symmetric_merged for merged). Qwen and Gemma paired cells share manifests, splits, weights, view (original_teacher_forced, harmonized_all_windows_full_coverage), namespace headline/binary_strict, and seeds. Fixed historical XGB rows remain in their original sheets, labelled, and are not replaced. All cells blank until evidence exists; not-run fields stay blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Family / Dataset</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Aggregation</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Macro-F1</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Partition</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Comparability</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DepresInstruct (Li et al., 2025)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Qwen2-Audio-7B</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Positive-F1</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Native — D3TEC</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Native — D3TEC</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Native — D3TEC</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Audio only</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>0.6667</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.7714</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>DAIC development</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>C — reported as F1; shown as Macro-F1 per researcher decision</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.inffus.2025.104077</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>DepresInstruct (Li et al., 2025)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Qwen2-7B</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Native — D3TEC</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Native — D3TEC</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Text only</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>0.7272999999999999</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.7429</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>DAIC development</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>C — reported as F1; shown as Macro-F1 per researcher decision</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.inffus.2025.104077</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>DepresInstruct (Li et al., 2025)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Qwen2-Audio-7B</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Native — D3TEC</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Native — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Audio + Text</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>0.7619</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.8571</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>DAIC development</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>C — reported as F1; shown as Macro-F1 per researcher decision</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.inffus.2025.104077</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>IT HEARS — Qwen2-7B baseline</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Qwen2-7B</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Native — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Native — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Native — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Native — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Text only</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>0.5639999999999999</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>DAIC development</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>C — paper reports F1; baseline; no validation/accuracy reported</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2511.19877</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>IT HEARS — Qwen2-Audio-7B</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Qwen2-Audio-7B</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Native — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Native — CMDC</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Audio + Text</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>DAIC development</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>C — paper reports F1; no validation/accuracy reported</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2511.19877</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Ours — official development (35 subjects, seed 1337, fold 0, best_model)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Backbone</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Modality</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Macro-F1</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Positive-F1</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Selected epoch</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>Verification</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Gemma 4 12B IT</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Native — CMDC</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Native — CMDC</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Audio only</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
-        <v>0.396551724137931</v>
-      </c>
-      <c r="D11" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="15" t="n">
-        <v>0.6571428571428571</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="n">
-        <v>35</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/audio_only/daic/daic_officialdev_gemma4_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>recomputed locally from predictions; attempt 20260813T142848Z-dai…</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Qwen</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Native — CMDC</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Audio only</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
-        <v>0.3859649122807018</v>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <v>0.6285714285714286</v>
-      </c>
-      <c r="F12" t="n">
-        <v>7</v>
-      </c>
-      <c r="G12" t="n">
-        <v>35</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>output_model/harmonized_v1_officialdev/audio_only/daic/daic_officialdev_qwen_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>recomputed locally from predictions; attempt 20260813T142847Z-dai…</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Gemma 4 12B IT</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Native — CMDC</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Native — CMDC</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Native — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Audio + Text</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
-        <v>0.7552447552447553</v>
-      </c>
-      <c r="D13" s="15" t="n">
-        <v>0.6923076923076924</v>
-      </c>
-      <c r="E13" s="15" t="n">
-        <v>0.7714285714285715</v>
-      </c>
-      <c r="F13" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" t="n">
-        <v>35</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/audio_text/daic/daic_officialdev_gemma4_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>recomputed locally from predictions; attempt 20260813T142848Z-dai…</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>Qwen</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Native — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Audio + Text</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
-        <v>0.6258503401360545</v>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>0.4761904761904762</v>
-      </c>
-      <c r="E14" s="15" t="n">
-        <v>0.6857142857142857</v>
-      </c>
-      <c r="F14" t="n">
-        <v>2</v>
-      </c>
-      <c r="G14" t="n">
-        <v>35</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>output_model/harmonized_v1_officialdev/audio_text/daic/daic_officialdev_qwen_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>recomputed locally from predictions; attempt 20260813T142848Z-dai…</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Gemma 4 12B IT</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Native — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Native — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Native — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>Text only</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n">
-        <v>0.7822222222222222</v>
-      </c>
-      <c r="D15" s="15" t="n">
-        <v>0.7199999999999999</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F15" t="n">
-        <v>4</v>
-      </c>
-      <c r="G15" t="n">
-        <v>35</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/text_only/daic/daic_officialdev_gemma4_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>recomputed locally from predictions; attempt 20260813T142849Z-dai…</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>Qwen</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Native — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Text only</t>
         </is>
       </c>
-      <c r="C16" s="15" t="n">
-        <v>0.7086031452358927</v>
-      </c>
-      <c r="D16" s="15" t="n">
-        <v>0.6086956521739131</v>
-      </c>
-      <c r="E16" s="15" t="n">
-        <v>0.7428571428571429</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="n">
-        <v>35</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>output_model/harmonized_v1_officialdev/text_only/daic/daic_officialdev_qwen_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>recomputed locally from predictions; attempt 20260813T142848Z-dai…</t>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Native — DAIC-WOZ</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Native — DAIC-WOZ</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Native — DAIC-WOZ</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Native — DAIC-WOZ</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Native — DAIC-WOZ</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Native — DAIC-WOZ</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>English — D3TEC</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>English — D3TEC</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="n"/>
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>English — D3TEC</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="n"/>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>English — D3TEC</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n"/>
+      <c r="F40" s="7" t="n"/>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>English — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="n"/>
+      <c r="F41" s="7" t="n"/>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>English — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="n"/>
+      <c r="F42" s="7" t="n"/>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>English — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="n"/>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>English — Androids Interview</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="n"/>
+      <c r="F44" s="7" t="n"/>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>English — CMDC</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="n"/>
+      <c r="F45" s="7" t="n"/>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>English — CMDC</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="n"/>
+      <c r="F46" s="7" t="n"/>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>English — CMDC</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="n"/>
+      <c r="F47" s="7" t="n"/>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>English — CMDC</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>English — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="7" t="n"/>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>English — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="n"/>
+      <c r="F50" s="7" t="n"/>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>English — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="n"/>
+      <c r="F51" s="7" t="n"/>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>English — Turkish t17</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="n"/>
+      <c r="F52" s="7" t="n"/>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Symmetric merged</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — CV (5-fold)</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n"/>
+      <c r="F54" s="7" t="n"/>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — CV (5-fold)</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n"/>
+      <c r="F55" s="7" t="n"/>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — CV (5-fold)</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="n"/>
+      <c r="F56" s="7" t="n"/>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — CV (5-fold)</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="n"/>
+      <c r="F57" s="7" t="n"/>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — CV (5-fold)</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="n"/>
+      <c r="F58" s="7" t="n"/>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — CV (5-fold)</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n"/>
+      <c r="F59" s="7" t="n"/>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — Final (DAIC official test)</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="n"/>
+      <c r="F60" s="7" t="n"/>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — Final (DAIC official test)</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n"/>
+      <c r="F61" s="7" t="n"/>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — Final (DAIC official test)</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="n"/>
+      <c r="F62" s="7" t="n"/>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — Final (DAIC official test)</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n"/>
+      <c r="F63" s="7" t="n"/>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — Final (DAIC official test)</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="n"/>
+      <c r="F64" s="7" t="n"/>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Symmetric merged — Final (DAIC official test)</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="n"/>
+      <c r="F65" s="7" t="n"/>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>DAIC official development</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>DAIC official development — Official dev</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="n"/>
+      <c r="F67" s="7" t="n"/>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>DAIC official development — Official dev</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="n"/>
+      <c r="F68" s="7" t="n"/>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>DAIC official development — Official dev</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="n"/>
+      <c r="F69" s="7" t="n"/>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>DAIC official development — Official dev</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="n"/>
+      <c r="F70" s="7" t="n"/>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>DAIC official development — Official dev</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Qwen</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="n"/>
+      <c r="F71" s="7" t="n"/>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>DAIC official development — Official dev</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>pooled / fold-mean</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="n"/>
+      <c r="F72" s="7" t="n"/>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>not run yet</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A2:I2"/>
+  <mergeCells count="6">
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh workbook hashes and use a schema-compliant merged parent marker
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -22300,14 +22300,14 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Standardized Optuna-100 XGBoost — macro-F1 (not run yet)</t>
+          <t>Standardized Optuna-100 XGBoost — macro-F1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Protocol harmonized_optuna100_v1: exactly 100 TPE trials, seeds 1337/1337/1337, 3 subject-grouped inner folds, threshold 0.5, sampling none, pooled inner subject-level macro-F1 objective (merged: unweighted mean of five per-dataset inner macro-F1). Prediction backends qwen_hidden_xgb_optuna100 / gemma4_hidden_xgb_optuna100 (+ _symmetric_merged for merged). Qwen and Gemma paired cells share manifests, splits, weights, view (original_teacher_forced, harmonized_all_windows_full_coverage), namespace headline/binary_strict, and seeds. Fixed historical XGB rows remain in their original sheets, labelled, and are not replaced. All cells blank until evidence exists; not-run fields stay blank.</t>
+          <t>Protocol harmonized_optuna100_v1: exactly 100 TPE trials, seeds 1337/1337/1337, 3 subject-grouped inner folds, threshold 0.5, sampling none, pooled inner subject-level macro-F1 objective (merged: unweighted mean of five per-dataset inner macro-F1). Prediction backends qwen_hidden_xgb_optuna100 / gemma4_hidden_xgb_optuna100 (+ _symmetric_merged for merged). Qwen and Gemma paired cells share manifests, splits, weights, view (original_teacher_forced, harmonized_all_windows_full_coverage), namespace headline/binary_strict, and seeds. Values are fold-mean macro-F1 from the qualified group reports; the merged 'Final (DAIC official test)' rows are the single DAIC test fold. Fixed historical XGB rows remain in their original sheets, labelled, and are not replaced.</t>
         </is>
       </c>
     </row>
@@ -22373,14 +22373,16 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0.5234</v>
+      </c>
       <c r="F6" s="7" t="n"/>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/d3tec_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22402,14 +22404,16 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.5832000000000001</v>
+      </c>
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/d3tec_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22431,14 +22435,16 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0.5195</v>
+      </c>
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/d3tec_audio_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22460,14 +22466,16 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.5461</v>
+      </c>
       <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/d3tec_audio_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22489,14 +22497,16 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0.6345</v>
+      </c>
       <c r="F10" s="7" t="n"/>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/d3tec_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22518,14 +22528,16 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.5719</v>
+      </c>
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/d3tec_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22547,14 +22559,16 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0.8542999999999999</v>
+      </c>
       <c r="F12" s="7" t="n"/>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/androids_interview_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22576,14 +22590,16 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0.8565</v>
+      </c>
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/androids_interview_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22605,14 +22621,16 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>0.8109</v>
+      </c>
       <c r="F14" s="7" t="n"/>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/androids_interview_audio_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22634,14 +22652,16 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0.802</v>
+      </c>
       <c r="F15" s="7" t="n"/>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/androids_interview_audio_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22663,14 +22683,16 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>0.8466</v>
+      </c>
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/androids_interview_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22692,14 +22714,16 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0.7482</v>
+      </c>
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/androids_interview_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22721,14 +22745,16 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>0.9251</v>
+      </c>
       <c r="F18" s="7" t="n"/>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/cmdc_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22750,14 +22776,16 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0.9841</v>
+      </c>
       <c r="F19" s="7" t="n"/>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/cmdc_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22779,14 +22807,16 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>0.9516</v>
+      </c>
       <c r="F20" s="7" t="n"/>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/cmdc_audio_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22808,14 +22838,16 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0.9584</v>
+      </c>
       <c r="F21" s="7" t="n"/>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/cmdc_audio_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22837,14 +22869,16 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>0.9539</v>
+      </c>
       <c r="F22" s="7" t="n"/>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/cmdc_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22866,14 +22900,16 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F23" s="7" t="n"/>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/cmdc_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22895,14 +22931,16 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>0.6311</v>
+      </c>
       <c r="F24" s="7" t="n"/>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/turkish_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22924,14 +22962,16 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>0.6819</v>
+      </c>
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/turkish_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22953,14 +22993,16 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>0.5145</v>
+      </c>
       <c r="F26" s="7" t="n"/>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/turkish_audio_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -22982,14 +23024,16 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>0.5671</v>
+      </c>
       <c r="F27" s="7" t="n"/>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/turkish_audio_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23011,14 +23055,16 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>0.5891999999999999</v>
+      </c>
       <c r="F28" s="7" t="n"/>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/turkish_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23040,14 +23086,16 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>0.5208</v>
+      </c>
       <c r="F29" s="7" t="n"/>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/turkish_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23069,14 +23117,16 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>0.7157</v>
+      </c>
       <c r="F30" s="7" t="n"/>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/daic_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23098,14 +23148,16 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0.8157</v>
+      </c>
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/daic_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23127,14 +23179,16 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>0.5760999999999999</v>
+      </c>
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/daic_audio_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23156,14 +23210,16 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>0.7257</v>
+      </c>
       <c r="F33" s="7" t="n"/>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/daic_audio_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23185,14 +23241,16 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>0.7257</v>
+      </c>
       <c r="F34" s="7" t="n"/>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/daic_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23214,14 +23272,16 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>0.7696</v>
+      </c>
       <c r="F35" s="7" t="n"/>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_native/daic_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23250,14 +23310,16 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>0.5982</v>
+      </c>
       <c r="F37" s="7" t="n"/>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/d3tec_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23279,14 +23341,16 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>0.5467</v>
+      </c>
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/d3tec_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23308,14 +23372,16 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>0.5289</v>
+      </c>
       <c r="F39" s="7" t="n"/>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/d3tec_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23337,14 +23403,16 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>0.5599</v>
+      </c>
       <c r="F40" s="7" t="n"/>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/d3tec_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23366,14 +23434,16 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>0.8727</v>
+      </c>
       <c r="F41" s="7" t="n"/>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/androids_interview_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23395,14 +23465,16 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>0.9028</v>
+      </c>
       <c r="F42" s="7" t="n"/>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/androids_interview_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23424,14 +23496,16 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>0.8111</v>
+      </c>
       <c r="F43" s="7" t="n"/>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/androids_interview_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23453,14 +23527,16 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>0.8084</v>
+      </c>
       <c r="F44" s="7" t="n"/>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/androids_interview_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23482,14 +23558,16 @@
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>0.9134</v>
+      </c>
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/cmdc_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23511,14 +23589,16 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>0.9683</v>
+      </c>
       <c r="F46" s="7" t="n"/>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/cmdc_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23540,14 +23620,16 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/cmdc_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23569,14 +23651,16 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="n">
+        <v>0.9398</v>
+      </c>
       <c r="F48" s="7" t="n"/>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/cmdc_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23598,14 +23682,16 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>0.6287</v>
+      </c>
       <c r="F49" s="7" t="n"/>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/turkish_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23627,14 +23713,16 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>0.5928</v>
+      </c>
       <c r="F50" s="7" t="n"/>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/turkish_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23656,14 +23744,16 @@
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="n">
+        <v>0.6584</v>
+      </c>
       <c r="F51" s="7" t="n"/>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/turkish_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23685,14 +23775,16 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>0.6296</v>
+      </c>
       <c r="F52" s="7" t="n"/>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_english/turkish_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23721,14 +23813,16 @@
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v>0.7412</v>
+      </c>
       <c r="F54" s="7" t="n"/>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/audio_text_cv_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23750,14 +23844,16 @@
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="n">
+        <v>0.7644</v>
+      </c>
       <c r="F55" s="7" t="n"/>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/audio_text_cv_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23779,14 +23875,16 @@
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="n">
+        <v>0.7474</v>
+      </c>
       <c r="F56" s="7" t="n"/>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/audio_only_cv_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23808,14 +23906,16 @@
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="n">
+        <v>0.7008</v>
+      </c>
       <c r="F57" s="7" t="n"/>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/audio_only_cv_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23837,14 +23937,16 @@
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v>0.7603</v>
+      </c>
       <c r="F58" s="7" t="n"/>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/text_only_cv_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23866,14 +23968,16 @@
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="n">
+        <v>0.7658</v>
+      </c>
       <c r="F59" s="7" t="n"/>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/text_only_cv_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23895,14 +23999,16 @@
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="n">
+        <v>0.7432</v>
+      </c>
       <c r="F60" s="7" t="n"/>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/audio_text_final_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23924,14 +24030,16 @@
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="n">
+        <v>0.7457</v>
+      </c>
       <c r="F61" s="7" t="n"/>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/audio_text_final_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23953,14 +24061,16 @@
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E62" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="n">
+        <v>0.4728</v>
+      </c>
       <c r="F62" s="7" t="n"/>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/audio_only_final_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -23982,14 +24092,16 @@
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="n">
+        <v>0.5554</v>
+      </c>
       <c r="F63" s="7" t="n"/>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/audio_only_final_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -24011,14 +24123,16 @@
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="n">
+        <v>0.7552</v>
+      </c>
       <c r="F64" s="7" t="n"/>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/text_only_final_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -24040,14 +24154,16 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E65" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="n">
+        <v>0.7631</v>
+      </c>
       <c r="F65" s="7" t="n"/>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_merged/text_only_final_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -24076,14 +24192,16 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E67" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="n">
+        <v>0.5304</v>
+      </c>
       <c r="F67" s="7" t="n"/>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_officialdev/daic_audio_text_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -24105,14 +24223,16 @@
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E68" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="n">
+        <v>0.6830000000000001</v>
+      </c>
       <c r="F68" s="7" t="n"/>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_officialdev/daic_audio_text_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -24134,14 +24254,16 @@
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E69" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="n">
+        <v>0.5727</v>
+      </c>
       <c r="F69" s="7" t="n"/>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_officialdev/daic_audio_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -24163,14 +24285,16 @@
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E70" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="n">
+        <v>0.6686</v>
+      </c>
       <c r="F70" s="7" t="n"/>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_officialdev/daic_audio_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>
@@ -24192,14 +24316,16 @@
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="n">
+        <v>0.6749000000000001</v>
+      </c>
       <c r="F71" s="7" t="n"/>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_officialdev/daic_text_only_qwen/group_report.json</t>
         </is>
       </c>
     </row>
@@ -24221,14 +24347,16 @@
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>pooled / fold-mean</t>
-        </is>
-      </c>
-      <c r="E72" s="7" t="n"/>
+          <t>fold-mean</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="n">
+        <v>0.7086</v>
+      </c>
       <c r="F72" s="7" t="n"/>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>not run yet</t>
+          <t>report:outputs/experiment_reports/optuna100_officialdev/daic_text_only_gemma4/group_report.json</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix merged-final teacher-forced provenance
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -1189,7 +1189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1211,7 +1211,7 @@
     <row r="2" ht="110" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Three main experiments, both models, macro-F1 (binary-strict, best_model, harmonized view). XGBoost uses the standardized search of 100 trials (the default), seed 1337, for both models; the runbook fits no fixed XGB head for Gemma. Delta = Gemma minus Qwen. DAIC = official 47-subject test; CMDC/Turkish = 5-fold mean (train_val); D3TEC/Androids = pooled 5-fold subject-level; merged CV = mean over the five datasets; merged Final = DAIC official test. The merged final teacher-forced test evaluation was not produced as a separate artifact for Gemma, so that row is omitted. Per-cell provenance: Provenance sheet.</t>
+          <t>Three main experiments, both models, macro-F1 (binary-strict, best_model, harmonized view). XGBoost uses the standardized search of 100 trials (the default), seed 1337, for both models; the runbook fits no fixed XGB head for Gemma. Delta = Gemma minus Qwen. DAIC = official 47-subject test; CMDC/Turkish = 5-fold mean (train_val); D3TEC/Androids = pooled 5-fold subject-level; merged CV = mean over the five datasets; merged Final = DAIC official test. Per-cell provenance: Provenance sheet.</t>
         </is>
       </c>
     </row>
@@ -2958,17 +2958,17 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>LogReg head</t>
+          <t>Teacher-forced</t>
         </is>
       </c>
       <c r="E61" s="6" t="n">
-        <v>0.7432</v>
+        <v>0.7631</v>
       </c>
       <c r="F61" s="6" t="n">
-        <v>0.7834101382488479</v>
-      </c>
-      <c r="G61" s="7" t="n">
-        <v>0.0402</v>
+        <v>0.7257294429708223</v>
+      </c>
+      <c r="G61" s="8" t="n">
+        <v>-0.0374</v>
       </c>
     </row>
     <row r="62">
@@ -2989,17 +2989,17 @@
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LogReg head</t>
         </is>
       </c>
       <c r="E62" s="6" t="n">
-        <v>0.743235</v>
+        <v>0.7432</v>
       </c>
       <c r="F62" s="6" t="n">
-        <v>0.745671</v>
+        <v>0.7834101382488479</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0.0024</v>
+        <v>0.0402</v>
       </c>
     </row>
     <row r="63">
@@ -3015,22 +3015,22 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>LogReg head</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E63" s="6" t="n">
-        <v>0.6189</v>
+        <v>0.743235</v>
       </c>
       <c r="F63" s="6" t="n">
-        <v>0.4283783783783783</v>
-      </c>
-      <c r="G63" s="8" t="n">
-        <v>-0.1905</v>
+        <v>0.745671</v>
+      </c>
+      <c r="G63" s="7" t="n">
+        <v>0.0024</v>
       </c>
     </row>
     <row r="64">
@@ -3051,17 +3051,17 @@
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Teacher-forced</t>
         </is>
       </c>
       <c r="E64" s="6" t="n">
-        <v>0.472823</v>
+        <v>0.5332</v>
       </c>
       <c r="F64" s="6" t="n">
-        <v>0.555405</v>
-      </c>
-      <c r="G64" s="7" t="n">
-        <v>0.08260000000000001</v>
+        <v>0.5190058479532164</v>
+      </c>
+      <c r="G64" s="8" t="n">
+        <v>-0.0142</v>
       </c>
     </row>
     <row r="65">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="E65" s="6" t="n">
-        <v>0.7157</v>
+        <v>0.6189</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>0.70625</v>
+        <v>0.4283783783783783</v>
       </c>
       <c r="G65" s="8" t="n">
-        <v>-0.0094</v>
+        <v>-0.1905</v>
       </c>
     </row>
     <row r="66">
@@ -3108,122 +3108,122 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
+          <t>Audio only</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="n">
+        <v>0.472823</v>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>0.555405</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <v>0.08260000000000001</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>Merged — Final (DAIC test)</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
           <t>Text only</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="n">
-        <v>0.755208</v>
-      </c>
-      <c r="F66" s="6" t="n">
-        <v>0.763105</v>
-      </c>
-      <c r="G66" s="7" t="n">
-        <v>0.007900000000000001</v>
-      </c>
-    </row>
-    <row r="67" ht="22" customHeight="1">
-      <c r="A67" s="9" t="inlineStr">
-        <is>
-          <t>English (translated)</t>
-        </is>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>0.7756</v>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>0.7755968169761273</v>
+      </c>
+      <c r="G67" s="10" t="n">
+        <v>-0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Merged — Final (DAIC test)</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>D3TEC</t>
+          <t>Merged</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Teacher-forced</t>
+          <t>LogReg head</t>
         </is>
       </c>
       <c r="E68" s="6" t="n">
-        <v>0.6125</v>
+        <v>0.7157</v>
       </c>
       <c r="F68" s="6" t="n">
-        <v>0.564983</v>
+        <v>0.70625</v>
       </c>
       <c r="G68" s="8" t="n">
-        <v>-0.0475</v>
+        <v>-0.0094</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Merged — Final (DAIC test)</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>D3TEC</t>
+          <t>Merged</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>LogReg head</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E69" s="6" t="n">
-        <v>0.5464</v>
+        <v>0.755208</v>
       </c>
       <c r="F69" s="6" t="n">
-        <v>0.532292</v>
-      </c>
-      <c r="G69" s="8" t="n">
-        <v>-0.0141</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>D3TEC</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-      <c r="E70" s="6" t="n">
-        <v>0.5982</v>
-      </c>
-      <c r="F70" s="6" t="n">
-        <v>0.546749</v>
-      </c>
-      <c r="G70" s="8" t="n">
-        <v>-0.0515</v>
+        <v>0.763105</v>
+      </c>
+      <c r="G69" s="7" t="n">
+        <v>0.007900000000000001</v>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>English (translated)</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
@@ -3248,13 +3248,13 @@
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>0.5465</v>
+        <v>0.6125</v>
       </c>
       <c r="F71" s="6" t="n">
-        <v>0.4936</v>
+        <v>0.564983</v>
       </c>
       <c r="G71" s="8" t="n">
-        <v>-0.0529</v>
+        <v>-0.0475</v>
       </c>
     </row>
     <row r="72">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
@@ -3279,13 +3279,13 @@
         </is>
       </c>
       <c r="E72" s="6" t="n">
-        <v>0.5226</v>
+        <v>0.5464</v>
       </c>
       <c r="F72" s="6" t="n">
-        <v>0.596902</v>
-      </c>
-      <c r="G72" s="7" t="n">
-        <v>0.0743</v>
+        <v>0.532292</v>
+      </c>
+      <c r="G72" s="8" t="n">
+        <v>-0.0141</v>
       </c>
     </row>
     <row r="73">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
@@ -3310,13 +3310,13 @@
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>0.5289</v>
+        <v>0.5982</v>
       </c>
       <c r="F73" s="6" t="n">
-        <v>0.5599460000000001</v>
-      </c>
-      <c r="G73" s="7" t="n">
-        <v>0.031</v>
+        <v>0.546749</v>
+      </c>
+      <c r="G73" s="8" t="n">
+        <v>-0.0515</v>
       </c>
     </row>
     <row r="74">
@@ -3327,12 +3327,12 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Androids Interview</t>
+          <t>D3TEC</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
@@ -3341,13 +3341,13 @@
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>0.8873</v>
+        <v>0.5465</v>
       </c>
       <c r="F74" s="6" t="n">
-        <v>0.876968</v>
+        <v>0.4936</v>
       </c>
       <c r="G74" s="8" t="n">
-        <v>-0.0103</v>
+        <v>-0.0529</v>
       </c>
     </row>
     <row r="75">
@@ -3358,12 +3358,12 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Androids Interview</t>
+          <t>D3TEC</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
@@ -3372,13 +3372,13 @@
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>0.8802</v>
+        <v>0.5226</v>
       </c>
       <c r="F75" s="6" t="n">
-        <v>0.902794</v>
+        <v>0.596902</v>
       </c>
       <c r="G75" s="7" t="n">
-        <v>0.0226</v>
+        <v>0.0743</v>
       </c>
     </row>
     <row r="76">
@@ -3389,12 +3389,12 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Androids Interview</t>
+          <t>D3TEC</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>0.8727</v>
+        <v>0.5289</v>
       </c>
       <c r="F76" s="6" t="n">
-        <v>0.902794</v>
+        <v>0.5599460000000001</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>0.0301</v>
+        <v>0.031</v>
       </c>
     </row>
     <row r="77">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
@@ -3434,13 +3434,13 @@
         </is>
       </c>
       <c r="E77" s="6" t="n">
-        <v>0.7921</v>
+        <v>0.8873</v>
       </c>
       <c r="F77" s="6" t="n">
-        <v>0.744654</v>
+        <v>0.876968</v>
       </c>
       <c r="G77" s="8" t="n">
-        <v>-0.0474</v>
+        <v>-0.0103</v>
       </c>
     </row>
     <row r="78">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
@@ -3465,13 +3465,13 @@
         </is>
       </c>
       <c r="E78" s="6" t="n">
-        <v>0.8298</v>
+        <v>0.8802</v>
       </c>
       <c r="F78" s="6" t="n">
-        <v>0.83016</v>
-      </c>
-      <c r="G78" s="10" t="n">
-        <v>0.0004</v>
+        <v>0.902794</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>0.0226</v>
       </c>
     </row>
     <row r="79">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
@@ -3496,13 +3496,13 @@
         </is>
       </c>
       <c r="E79" s="6" t="n">
-        <v>0.8111</v>
+        <v>0.8727</v>
       </c>
       <c r="F79" s="6" t="n">
-        <v>0.808427</v>
-      </c>
-      <c r="G79" s="8" t="n">
-        <v>-0.0027</v>
+        <v>0.902794</v>
+      </c>
+      <c r="G79" s="7" t="n">
+        <v>0.0301</v>
       </c>
     </row>
     <row r="80">
@@ -3513,12 +3513,12 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>CMDC</t>
+          <t>Androids Interview</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
@@ -3527,13 +3527,13 @@
         </is>
       </c>
       <c r="E80" s="6" t="n">
-        <v>0.9856</v>
+        <v>0.7921</v>
       </c>
       <c r="F80" s="6" t="n">
-        <v>0.955419</v>
+        <v>0.744654</v>
       </c>
       <c r="G80" s="8" t="n">
-        <v>-0.0302</v>
+        <v>-0.0474</v>
       </c>
     </row>
     <row r="81">
@@ -3544,12 +3544,12 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>CMDC</t>
+          <t>Androids Interview</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
@@ -3558,13 +3558,13 @@
         </is>
       </c>
       <c r="E81" s="6" t="n">
-        <v>0.9856</v>
+        <v>0.8298</v>
       </c>
       <c r="F81" s="6" t="n">
-        <v>0.9263479999999999</v>
-      </c>
-      <c r="G81" s="8" t="n">
-        <v>-0.0593</v>
+        <v>0.83016</v>
+      </c>
+      <c r="G81" s="10" t="n">
+        <v>0.0004</v>
       </c>
     </row>
     <row r="82">
@@ -3575,12 +3575,12 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>CMDC</t>
+          <t>Androids Interview</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
@@ -3589,13 +3589,13 @@
         </is>
       </c>
       <c r="E82" s="6" t="n">
-        <v>0.9134</v>
+        <v>0.8111</v>
       </c>
       <c r="F82" s="6" t="n">
-        <v>0.96828</v>
-      </c>
-      <c r="G82" s="7" t="n">
-        <v>0.0549</v>
+        <v>0.808427</v>
+      </c>
+      <c r="G82" s="8" t="n">
+        <v>-0.0027</v>
       </c>
     </row>
     <row r="83">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
@@ -3620,13 +3620,13 @@
         </is>
       </c>
       <c r="E83" s="6" t="n">
-        <v>0.9713000000000001</v>
+        <v>0.9856</v>
       </c>
       <c r="F83" s="6" t="n">
-        <v>0.957439</v>
+        <v>0.955419</v>
       </c>
       <c r="G83" s="8" t="n">
-        <v>-0.0139</v>
+        <v>-0.0302</v>
       </c>
     </row>
     <row r="84">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
@@ -3651,13 +3651,13 @@
         </is>
       </c>
       <c r="E84" s="6" t="n">
-        <v>0.9698</v>
+        <v>0.9856</v>
       </c>
       <c r="F84" s="6" t="n">
-        <v>0.969835</v>
-      </c>
-      <c r="G84" s="10" t="n">
-        <v>0</v>
+        <v>0.9263479999999999</v>
+      </c>
+      <c r="G84" s="8" t="n">
+        <v>-0.0593</v>
       </c>
     </row>
     <row r="85">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
@@ -3682,13 +3682,13 @@
         </is>
       </c>
       <c r="E85" s="6" t="n">
-        <v>0.9698</v>
+        <v>0.9134</v>
       </c>
       <c r="F85" s="6" t="n">
-        <v>0.939796</v>
-      </c>
-      <c r="G85" s="8" t="n">
-        <v>-0.03</v>
+        <v>0.96828</v>
+      </c>
+      <c r="G85" s="7" t="n">
+        <v>0.0549</v>
       </c>
     </row>
     <row r="86">
@@ -3699,12 +3699,12 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>CMDC</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
@@ -3713,13 +3713,13 @@
         </is>
       </c>
       <c r="E86" s="6" t="n">
-        <v>0.6294999999999999</v>
+        <v>0.9713000000000001</v>
       </c>
       <c r="F86" s="6" t="n">
-        <v>0.669119</v>
-      </c>
-      <c r="G86" s="7" t="n">
-        <v>0.0396</v>
+        <v>0.957439</v>
+      </c>
+      <c r="G86" s="8" t="n">
+        <v>-0.0139</v>
       </c>
     </row>
     <row r="87">
@@ -3730,12 +3730,12 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>CMDC</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
@@ -3744,13 +3744,13 @@
         </is>
       </c>
       <c r="E87" s="6" t="n">
-        <v>0.6076</v>
+        <v>0.9698</v>
       </c>
       <c r="F87" s="6" t="n">
-        <v>0.599564</v>
-      </c>
-      <c r="G87" s="8" t="n">
-        <v>-0.008</v>
+        <v>0.969835</v>
+      </c>
+      <c r="G87" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -3761,12 +3761,12 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>CMDC</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
@@ -3775,13 +3775,13 @@
         </is>
       </c>
       <c r="E88" s="6" t="n">
-        <v>0.6287</v>
+        <v>0.9698</v>
       </c>
       <c r="F88" s="6" t="n">
-        <v>0.592804</v>
+        <v>0.939796</v>
       </c>
       <c r="G88" s="8" t="n">
-        <v>-0.0359</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="89">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
@@ -3806,13 +3806,13 @@
         </is>
       </c>
       <c r="E89" s="6" t="n">
-        <v>0.6641</v>
+        <v>0.6294999999999999</v>
       </c>
       <c r="F89" s="6" t="n">
-        <v>0.6774</v>
+        <v>0.669119</v>
       </c>
       <c r="G89" s="7" t="n">
-        <v>0.0133</v>
+        <v>0.0396</v>
       </c>
     </row>
     <row r="90">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
@@ -3837,13 +3837,13 @@
         </is>
       </c>
       <c r="E90" s="6" t="n">
-        <v>0.5944</v>
+        <v>0.6076</v>
       </c>
       <c r="F90" s="6" t="n">
-        <v>0.6014350000000001</v>
-      </c>
-      <c r="G90" s="7" t="n">
-        <v>0.007</v>
+        <v>0.599564</v>
+      </c>
+      <c r="G90" s="8" t="n">
+        <v>-0.008</v>
       </c>
     </row>
     <row r="91">
@@ -3859,26 +3859,119 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>0.6287</v>
+      </c>
+      <c r="F91" s="6" t="n">
+        <v>0.592804</v>
+      </c>
+      <c r="G91" s="8" t="n">
+        <v>-0.0359</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
           <t>Text only</t>
         </is>
       </c>
-      <c r="D91" s="5" t="inlineStr">
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="E92" s="6" t="n">
+        <v>0.6641</v>
+      </c>
+      <c r="F92" s="6" t="n">
+        <v>0.6774</v>
+      </c>
+      <c r="G92" s="7" t="n">
+        <v>0.0133</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>LogReg head</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>0.5944</v>
+      </c>
+      <c r="F93" s="6" t="n">
+        <v>0.6014350000000001</v>
+      </c>
+      <c r="G93" s="7" t="n">
+        <v>0.007</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="E91" s="6" t="n">
+      <c r="E94" s="6" t="n">
         <v>0.6584</v>
       </c>
-      <c r="F91" s="6" t="n">
+      <c r="F94" s="6" t="n">
         <v>0.629565</v>
       </c>
-      <c r="G91" s="8" t="n">
+      <c r="G94" s="8" t="n">
         <v>-0.0288</v>
       </c>
     </row>
-    <row r="92" ht="60" customHeight="1">
-      <c r="A92" s="2" t="inlineStr">
+    <row r="95" ht="60" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
         <is>
           <t>Teacher-forced = backbone classification without hidden-state heads. Hidden heads classify the final prompt-token hidden state with the locked LogReg or the standardized XGBoost implementation. See the Provenance sheet for every value's run, aggregation, and local artifact.</t>
         </is>
@@ -3887,8 +3980,8 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A67:G67"/>
-    <mergeCell ref="A92:G92"/>
+    <mergeCell ref="A70:G70"/>
+    <mergeCell ref="A95:G95"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A51:G51"/>
     <mergeCell ref="A5:G5"/>
@@ -4418,7 +4511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I436"/>
+  <dimension ref="A1:I442"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -20527,102 +20620,102 @@
     <row r="359">
       <c r="A359" s="11" t="inlineStr">
         <is>
-          <t>DAIC official development</t>
+          <t>Gemma merged</t>
         </is>
       </c>
       <c r="B359" s="11" t="inlineStr">
         <is>
-          <t>DAIC</t>
+          <t>Final (DAIC test)</t>
         </is>
       </c>
       <c r="C359" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D359" s="11" t="inlineStr">
         <is>
-          <t>Qwen teacher-forced macro-F1</t>
+          <t>Teacher-forced</t>
         </is>
       </c>
       <c r="E359" s="12" t="n">
-        <v>0.3859649122807018</v>
+        <v>0.7257294429708223</v>
       </c>
       <c r="F359" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142847Z-daic_officialdev_qwen_audio_only_seed1337-22f85e6e-9c326e1d, eval eval-7c1ef60108d44e8081fa66cd, selected epoch 7, best_model</t>
+          <t>campaign gemma4_merged_v1_prod_20260816T0000Z_d4ff33e, postprocess job 44684476, source bfc13b4f8b177547a11a9abad526115b712d32ef</t>
         </is>
       </c>
       <c r="G359" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>DAIC official test, 47 subjects, teacher-forced, binary-strict, subject mean-score, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H359" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev/audio_only/daic/daic_officialdev_qwen_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>outputs/symmetric_merged/gemma4/harmonized_v1/audio_text/gemma4_merged_v1_prod_20260816T0000Z_d4ff33e/final/fold_0/gemma4/daic/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I359" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally from synced predictions; REPORTABLE</t>
+          <t>recomputed locally from 47 subject predictions; zero invalid subjects</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="11" t="inlineStr">
         <is>
-          <t>DAIC official development</t>
+          <t>Gemma merged</t>
         </is>
       </c>
       <c r="B360" s="11" t="inlineStr">
         <is>
-          <t>DAIC</t>
+          <t>Final (DAIC test)</t>
         </is>
       </c>
       <c r="C360" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D360" s="11" t="inlineStr">
         <is>
-          <t>Qwen teacher-forced positive-F1</t>
+          <t>LogReg head</t>
         </is>
       </c>
       <c r="E360" s="12" t="n">
-        <v>0</v>
+        <v>0.7834101382488479</v>
       </c>
       <c r="F360" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142847Z-daic_officialdev_qwen_audio_only_seed1337-22f85e6e-9c326e1d, eval eval-7c1ef60108d44e8081fa66cd, selected epoch 7, best_model</t>
+          <t>campaign gemma4_merged_v1_prod_20260816T0000Z_d4ff33e, merged heads</t>
         </is>
       </c>
       <c r="G360" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>Final (DAIC test), LogReg raw hidden head, mean over five datasets</t>
         </is>
       </c>
       <c r="H360" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev/audio_only/daic/daic_officialdev_qwen_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>outputs/symmetric_merged/gemma4/harmonized_v1/audio_text/gemma4_merged_v1_prod_20260816T0000Z_d4ff33e/final/fold_0/heads/logreg/metrics_by_dataset.json</t>
         </is>
       </c>
       <c r="I360" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally from synced predictions; REPORTABLE</t>
+          <t>recomputed from predictions (matches metrics_by_dataset.json)</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="11" t="inlineStr">
         <is>
-          <t>DAIC official development</t>
+          <t>Gemma merged</t>
         </is>
       </c>
       <c r="B361" s="11" t="inlineStr">
         <is>
-          <t>DAIC</t>
+          <t>Final (DAIC test)</t>
         </is>
       </c>
       <c r="C361" s="11" t="inlineStr">
@@ -20632,42 +20725,42 @@
       </c>
       <c r="D361" s="11" t="inlineStr">
         <is>
-          <t>Qwen teacher-forced accuracy</t>
+          <t>Teacher-forced</t>
         </is>
       </c>
       <c r="E361" s="12" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.5190058479532164</v>
       </c>
       <c r="F361" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142847Z-daic_officialdev_qwen_audio_only_seed1337-22f85e6e-9c326e1d, eval eval-7c1ef60108d44e8081fa66cd, selected epoch 7, best_model</t>
+          <t>campaign gemma4_merged_v1_prod_20260816T0000Z_d4ff33e, postprocess job 44684479, source bfc13b4f8b177547a11a9abad526115b712d32ef</t>
         </is>
       </c>
       <c r="G361" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>DAIC official test, 47 subjects, teacher-forced, binary-strict, subject mean-score, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H361" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev/audio_only/daic/daic_officialdev_qwen_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>outputs/symmetric_merged/gemma4/harmonized_v1/audio_only/gemma4_merged_v1_prod_20260816T0000Z_d4ff33e/final/fold_0/gemma4/daic/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I361" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally from synced predictions; REPORTABLE</t>
+          <t>recomputed locally from 47 subject predictions; zero invalid subjects</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="11" t="inlineStr">
         <is>
-          <t>DAIC official development</t>
+          <t>Gemma merged</t>
         </is>
       </c>
       <c r="B362" s="11" t="inlineStr">
         <is>
-          <t>DAIC</t>
+          <t>Final (DAIC test)</t>
         </is>
       </c>
       <c r="C362" s="11" t="inlineStr">
@@ -20677,120 +20770,120 @@
       </c>
       <c r="D362" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 teacher-forced macro-F1</t>
+          <t>LogReg head</t>
         </is>
       </c>
       <c r="E362" s="12" t="n">
-        <v>0.396551724137931</v>
+        <v>0.4283783783783783</v>
       </c>
       <c r="F362" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_only_seed1337-22f85e6e-bb8bbbed, eval eval-6df29e41d91c3bd14a35b17a, selected epoch 1, best_model</t>
+          <t>campaign gemma4_merged_v1_prod_20260816T0000Z_d4ff33e, merged heads</t>
         </is>
       </c>
       <c r="G362" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>Final (DAIC test), LogReg raw hidden head, mean over five datasets</t>
         </is>
       </c>
       <c r="H362" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/audio_only/daic/daic_officialdev_gemma4_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>outputs/symmetric_merged/gemma4/harmonized_v1/audio_only/gemma4_merged_v1_prod_20260816T0000Z_d4ff33e/final/fold_0/heads/logreg/metrics_by_dataset.json</t>
         </is>
       </c>
       <c r="I362" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally from synced predictions; REPORTABLE</t>
+          <t>recomputed from predictions (matches metrics_by_dataset.json)</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="11" t="inlineStr">
         <is>
-          <t>DAIC official development</t>
+          <t>Gemma merged</t>
         </is>
       </c>
       <c r="B363" s="11" t="inlineStr">
         <is>
-          <t>DAIC</t>
+          <t>Final (DAIC test)</t>
         </is>
       </c>
       <c r="C363" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D363" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 teacher-forced positive-F1</t>
+          <t>Teacher-forced</t>
         </is>
       </c>
       <c r="E363" s="12" t="n">
-        <v>0</v>
+        <v>0.7755968169761273</v>
       </c>
       <c r="F363" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_only_seed1337-22f85e6e-bb8bbbed, eval eval-6df29e41d91c3bd14a35b17a, selected epoch 1, best_model</t>
+          <t>campaign gemma4_merged_v1_prod_20260816T0000Z_d4ff33e, postprocess job 44684482, source bfc13b4f8b177547a11a9abad526115b712d32ef</t>
         </is>
       </c>
       <c r="G363" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>DAIC official test, 47 subjects, teacher-forced, binary-strict, subject mean-score, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H363" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/audio_only/daic/daic_officialdev_gemma4_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>outputs/symmetric_merged/gemma4/harmonized_v1/text_only/gemma4_merged_v1_prod_20260816T0000Z_d4ff33e/final/fold_0/gemma4/daic/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I363" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally from synced predictions; REPORTABLE</t>
+          <t>recomputed locally from 47 subject predictions; zero invalid subjects</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="11" t="inlineStr">
         <is>
-          <t>DAIC official development</t>
+          <t>Gemma merged</t>
         </is>
       </c>
       <c r="B364" s="11" t="inlineStr">
         <is>
-          <t>DAIC</t>
+          <t>Final (DAIC test)</t>
         </is>
       </c>
       <c r="C364" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D364" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 teacher-forced accuracy</t>
+          <t>LogReg head</t>
         </is>
       </c>
       <c r="E364" s="12" t="n">
-        <v>0.6571428571428571</v>
+        <v>0.70625</v>
       </c>
       <c r="F364" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_only_seed1337-22f85e6e-bb8bbbed, eval eval-6df29e41d91c3bd14a35b17a, selected epoch 1, best_model</t>
+          <t>campaign gemma4_merged_v1_prod_20260816T0000Z_d4ff33e, merged heads</t>
         </is>
       </c>
       <c r="G364" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>Final (DAIC test), LogReg raw hidden head, mean over five datasets</t>
         </is>
       </c>
       <c r="H364" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/audio_only/daic/daic_officialdev_gemma4_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>outputs/symmetric_merged/gemma4/harmonized_v1/text_only/gemma4_merged_v1_prod_20260816T0000Z_d4ff33e/final/fold_0/heads/logreg/metrics_by_dataset.json</t>
         </is>
       </c>
       <c r="I364" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally from synced predictions; REPORTABLE</t>
+          <t>recomputed from predictions (matches metrics_by_dataset.json)</t>
         </is>
       </c>
     </row>
@@ -20807,7 +20900,7 @@
       </c>
       <c r="C365" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D365" s="11" t="inlineStr">
@@ -20816,11 +20909,11 @@
         </is>
       </c>
       <c r="E365" s="12" t="n">
-        <v>0.6258503401360545</v>
+        <v>0.3859649122807018</v>
       </c>
       <c r="F365" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_audio_text_seed1337-22f85e6e-16e99f52, eval eval-c4dd0ff1892bd0e3a39cc9bb, selected epoch 2, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142847Z-daic_officialdev_qwen_audio_only_seed1337-22f85e6e-9c326e1d, eval eval-7c1ef60108d44e8081fa66cd, selected epoch 7, best_model</t>
         </is>
       </c>
       <c r="G365" s="13" t="inlineStr">
@@ -20830,7 +20923,7 @@
       </c>
       <c r="H365" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev/audio_text/daic/daic_officialdev_qwen_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev/audio_only/daic/daic_officialdev_qwen_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I365" s="13" t="inlineStr">
@@ -20852,7 +20945,7 @@
       </c>
       <c r="C366" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D366" s="11" t="inlineStr">
@@ -20861,11 +20954,11 @@
         </is>
       </c>
       <c r="E366" s="12" t="n">
-        <v>0.4761904761904762</v>
+        <v>0</v>
       </c>
       <c r="F366" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_audio_text_seed1337-22f85e6e-16e99f52, eval eval-c4dd0ff1892bd0e3a39cc9bb, selected epoch 2, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142847Z-daic_officialdev_qwen_audio_only_seed1337-22f85e6e-9c326e1d, eval eval-7c1ef60108d44e8081fa66cd, selected epoch 7, best_model</t>
         </is>
       </c>
       <c r="G366" s="13" t="inlineStr">
@@ -20875,7 +20968,7 @@
       </c>
       <c r="H366" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev/audio_text/daic/daic_officialdev_qwen_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev/audio_only/daic/daic_officialdev_qwen_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I366" s="13" t="inlineStr">
@@ -20897,7 +20990,7 @@
       </c>
       <c r="C367" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D367" s="11" t="inlineStr">
@@ -20906,11 +20999,11 @@
         </is>
       </c>
       <c r="E367" s="12" t="n">
-        <v>0.6857142857142857</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="F367" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_audio_text_seed1337-22f85e6e-16e99f52, eval eval-c4dd0ff1892bd0e3a39cc9bb, selected epoch 2, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142847Z-daic_officialdev_qwen_audio_only_seed1337-22f85e6e-9c326e1d, eval eval-7c1ef60108d44e8081fa66cd, selected epoch 7, best_model</t>
         </is>
       </c>
       <c r="G367" s="13" t="inlineStr">
@@ -20920,7 +21013,7 @@
       </c>
       <c r="H367" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev/audio_text/daic/daic_officialdev_qwen_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev/audio_only/daic/daic_officialdev_qwen_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I367" s="13" t="inlineStr">
@@ -20942,7 +21035,7 @@
       </c>
       <c r="C368" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D368" s="11" t="inlineStr">
@@ -20951,11 +21044,11 @@
         </is>
       </c>
       <c r="E368" s="12" t="n">
-        <v>0.7552447552447553</v>
+        <v>0.396551724137931</v>
       </c>
       <c r="F368" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_text_seed1337-22f85e6e-df9dad6b, eval eval-0eb033332e85c3a84b70b52e, selected epoch 2, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_only_seed1337-22f85e6e-bb8bbbed, eval eval-6df29e41d91c3bd14a35b17a, selected epoch 1, best_model</t>
         </is>
       </c>
       <c r="G368" s="13" t="inlineStr">
@@ -20965,7 +21058,7 @@
       </c>
       <c r="H368" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/audio_text/daic/daic_officialdev_gemma4_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev/audio_only/daic/daic_officialdev_gemma4_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I368" s="13" t="inlineStr">
@@ -20987,7 +21080,7 @@
       </c>
       <c r="C369" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D369" s="11" t="inlineStr">
@@ -20996,11 +21089,11 @@
         </is>
       </c>
       <c r="E369" s="12" t="n">
-        <v>0.6923076923076924</v>
+        <v>0</v>
       </c>
       <c r="F369" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_text_seed1337-22f85e6e-df9dad6b, eval eval-0eb033332e85c3a84b70b52e, selected epoch 2, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_only_seed1337-22f85e6e-bb8bbbed, eval eval-6df29e41d91c3bd14a35b17a, selected epoch 1, best_model</t>
         </is>
       </c>
       <c r="G369" s="13" t="inlineStr">
@@ -21010,7 +21103,7 @@
       </c>
       <c r="H369" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/audio_text/daic/daic_officialdev_gemma4_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev/audio_only/daic/daic_officialdev_gemma4_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I369" s="13" t="inlineStr">
@@ -21032,7 +21125,7 @@
       </c>
       <c r="C370" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D370" s="11" t="inlineStr">
@@ -21041,11 +21134,11 @@
         </is>
       </c>
       <c r="E370" s="12" t="n">
-        <v>0.7714285714285715</v>
+        <v>0.6571428571428571</v>
       </c>
       <c r="F370" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_text_seed1337-22f85e6e-df9dad6b, eval eval-0eb033332e85c3a84b70b52e, selected epoch 2, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_only_seed1337-22f85e6e-bb8bbbed, eval eval-6df29e41d91c3bd14a35b17a, selected epoch 1, best_model</t>
         </is>
       </c>
       <c r="G370" s="13" t="inlineStr">
@@ -21055,7 +21148,7 @@
       </c>
       <c r="H370" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/audio_text/daic/daic_officialdev_gemma4_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev/audio_only/daic/daic_officialdev_gemma4_audio_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I370" s="13" t="inlineStr">
@@ -21077,7 +21170,7 @@
       </c>
       <c r="C371" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D371" s="11" t="inlineStr">
@@ -21086,11 +21179,11 @@
         </is>
       </c>
       <c r="E371" s="12" t="n">
-        <v>0.7086031452358927</v>
+        <v>0.6258503401360545</v>
       </c>
       <c r="F371" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_text_only_seed1337-22f85e6e-713b6d93, eval eval-6a466b499f152ea1b9c3c489, selected epoch 1, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_audio_text_seed1337-22f85e6e-16e99f52, eval eval-c4dd0ff1892bd0e3a39cc9bb, selected epoch 2, best_model</t>
         </is>
       </c>
       <c r="G371" s="13" t="inlineStr">
@@ -21100,7 +21193,7 @@
       </c>
       <c r="H371" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev/text_only/daic/daic_officialdev_qwen_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev/audio_text/daic/daic_officialdev_qwen_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I371" s="13" t="inlineStr">
@@ -21122,7 +21215,7 @@
       </c>
       <c r="C372" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D372" s="11" t="inlineStr">
@@ -21131,11 +21224,11 @@
         </is>
       </c>
       <c r="E372" s="12" t="n">
-        <v>0.6086956521739131</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="F372" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_text_only_seed1337-22f85e6e-713b6d93, eval eval-6a466b499f152ea1b9c3c489, selected epoch 1, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_audio_text_seed1337-22f85e6e-16e99f52, eval eval-c4dd0ff1892bd0e3a39cc9bb, selected epoch 2, best_model</t>
         </is>
       </c>
       <c r="G372" s="13" t="inlineStr">
@@ -21145,7 +21238,7 @@
       </c>
       <c r="H372" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev/text_only/daic/daic_officialdev_qwen_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev/audio_text/daic/daic_officialdev_qwen_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I372" s="13" t="inlineStr">
@@ -21167,7 +21260,7 @@
       </c>
       <c r="C373" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D373" s="11" t="inlineStr">
@@ -21176,11 +21269,11 @@
         </is>
       </c>
       <c r="E373" s="12" t="n">
-        <v>0.7428571428571429</v>
+        <v>0.6857142857142857</v>
       </c>
       <c r="F373" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_text_only_seed1337-22f85e6e-713b6d93, eval eval-6a466b499f152ea1b9c3c489, selected epoch 1, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_audio_text_seed1337-22f85e6e-16e99f52, eval eval-c4dd0ff1892bd0e3a39cc9bb, selected epoch 2, best_model</t>
         </is>
       </c>
       <c r="G373" s="13" t="inlineStr">
@@ -21190,7 +21283,7 @@
       </c>
       <c r="H373" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev/text_only/daic/daic_officialdev_qwen_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev/audio_text/daic/daic_officialdev_qwen_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I373" s="13" t="inlineStr">
@@ -21212,7 +21305,7 @@
       </c>
       <c r="C374" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D374" s="11" t="inlineStr">
@@ -21221,11 +21314,11 @@
         </is>
       </c>
       <c r="E374" s="12" t="n">
-        <v>0.7822222222222222</v>
+        <v>0.7552447552447553</v>
       </c>
       <c r="F374" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142849Z-daic_officialdev_gemma4_text_only_seed1337-22f85e6e-75450bbe, eval eval-8a5d52df50d78e5dbeae4008, selected epoch 4, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_text_seed1337-22f85e6e-df9dad6b, eval eval-0eb033332e85c3a84b70b52e, selected epoch 2, best_model</t>
         </is>
       </c>
       <c r="G374" s="13" t="inlineStr">
@@ -21235,7 +21328,7 @@
       </c>
       <c r="H374" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/text_only/daic/daic_officialdev_gemma4_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev/audio_text/daic/daic_officialdev_gemma4_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I374" s="13" t="inlineStr">
@@ -21257,7 +21350,7 @@
       </c>
       <c r="C375" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D375" s="11" t="inlineStr">
@@ -21266,11 +21359,11 @@
         </is>
       </c>
       <c r="E375" s="12" t="n">
-        <v>0.7199999999999999</v>
+        <v>0.6923076923076924</v>
       </c>
       <c r="F375" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142849Z-daic_officialdev_gemma4_text_only_seed1337-22f85e6e-75450bbe, eval eval-8a5d52df50d78e5dbeae4008, selected epoch 4, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_text_seed1337-22f85e6e-df9dad6b, eval eval-0eb033332e85c3a84b70b52e, selected epoch 2, best_model</t>
         </is>
       </c>
       <c r="G375" s="13" t="inlineStr">
@@ -21280,7 +21373,7 @@
       </c>
       <c r="H375" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/text_only/daic/daic_officialdev_gemma4_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev/audio_text/daic/daic_officialdev_gemma4_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I375" s="13" t="inlineStr">
@@ -21302,7 +21395,7 @@
       </c>
       <c r="C376" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D376" s="11" t="inlineStr">
@@ -21311,11 +21404,11 @@
         </is>
       </c>
       <c r="E376" s="12" t="n">
-        <v>0.8</v>
+        <v>0.7714285714285715</v>
       </c>
       <c r="F376" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142849Z-daic_officialdev_gemma4_text_only_seed1337-22f85e6e-75450bbe, eval eval-8a5d52df50d78e5dbeae4008, selected epoch 4, best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_gemma4_audio_text_seed1337-22f85e6e-df9dad6b, eval eval-0eb033332e85c3a84b70b52e, selected epoch 2, best_model</t>
         </is>
       </c>
       <c r="G376" s="13" t="inlineStr">
@@ -21325,7 +21418,7 @@
       </c>
       <c r="H376" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev/text_only/daic/daic_officialdev_gemma4_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev/audio_text/daic/daic_officialdev_gemma4_audio_text_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I376" s="13" t="inlineStr">
@@ -21337,7 +21430,7 @@
     <row r="377">
       <c r="A377" s="11" t="inlineStr">
         <is>
-          <t>DAIC Head Ablation</t>
+          <t>DAIC official development</t>
         </is>
       </c>
       <c r="B377" s="11" t="inlineStr">
@@ -21347,42 +21440,42 @@
       </c>
       <c r="C377" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D377" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head macro-F1</t>
+          <t>Qwen teacher-forced macro-F1</t>
         </is>
       </c>
       <c r="E377" s="12" t="n">
-        <v>0.5716783216783217</v>
+        <v>0.7086031452358927</v>
       </c>
       <c r="F377" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_text_only_seed1337-22f85e6e-713b6d93, eval eval-6a466b499f152ea1b9c3c489, selected epoch 1, best_model</t>
         </is>
       </c>
       <c r="G377" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
         </is>
       </c>
       <c r="H377" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev/text_only/daic/daic_officialdev_qwen_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I377" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally by verify-local; REPORTABLE</t>
+          <t>recomputed locally from synced predictions; REPORTABLE</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="11" t="inlineStr">
         <is>
-          <t>DAIC Head Ablation</t>
+          <t>DAIC official development</t>
         </is>
       </c>
       <c r="B378" s="11" t="inlineStr">
@@ -21392,42 +21485,42 @@
       </c>
       <c r="C378" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D378" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head positive-F1</t>
+          <t>Qwen teacher-forced positive-F1</t>
         </is>
       </c>
       <c r="E378" s="12" t="n">
-        <v>0.4615384615384615</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="F378" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_text_only_seed1337-22f85e6e-713b6d93, eval eval-6a466b499f152ea1b9c3c489, selected epoch 1, best_model</t>
         </is>
       </c>
       <c r="G378" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
         </is>
       </c>
       <c r="H378" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev/text_only/daic/daic_officialdev_qwen_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I378" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally by verify-local; REPORTABLE</t>
+          <t>recomputed locally from synced predictions; REPORTABLE</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="11" t="inlineStr">
         <is>
-          <t>DAIC Head Ablation</t>
+          <t>DAIC official development</t>
         </is>
       </c>
       <c r="B379" s="11" t="inlineStr">
@@ -21437,42 +21530,42 @@
       </c>
       <c r="C379" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D379" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head accuracy</t>
+          <t>Qwen teacher-forced accuracy</t>
         </is>
       </c>
       <c r="E379" s="12" t="n">
-        <v>0.6</v>
+        <v>0.7428571428571429</v>
       </c>
       <c r="F379" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142848Z-daic_officialdev_qwen_text_only_seed1337-22f85e6e-713b6d93, eval eval-6a466b499f152ea1b9c3c489, selected epoch 1, best_model</t>
         </is>
       </c>
       <c r="G379" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
         </is>
       </c>
       <c r="H379" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev/text_only/daic/daic_officialdev_qwen_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I379" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally by verify-local; REPORTABLE</t>
+          <t>recomputed locally from synced predictions; REPORTABLE</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="11" t="inlineStr">
         <is>
-          <t>DAIC Head Ablation</t>
+          <t>DAIC official development</t>
         </is>
       </c>
       <c r="B380" s="11" t="inlineStr">
@@ -21482,42 +21575,42 @@
       </c>
       <c r="C380" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D380" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head precision</t>
+          <t>Gemma 4 teacher-forced macro-F1</t>
         </is>
       </c>
       <c r="E380" s="12" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.7822222222222222</v>
       </c>
       <c r="F380" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142849Z-daic_officialdev_gemma4_text_only_seed1337-22f85e6e-75450bbe, eval eval-8a5d52df50d78e5dbeae4008, selected epoch 4, best_model</t>
         </is>
       </c>
       <c r="G380" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
         </is>
       </c>
       <c r="H380" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev/text_only/daic/daic_officialdev_gemma4_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I380" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally by verify-local; REPORTABLE</t>
+          <t>recomputed locally from synced predictions; REPORTABLE</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="11" t="inlineStr">
         <is>
-          <t>DAIC Head Ablation</t>
+          <t>DAIC official development</t>
         </is>
       </c>
       <c r="B381" s="11" t="inlineStr">
@@ -21527,42 +21620,42 @@
       </c>
       <c r="C381" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D381" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head recall</t>
+          <t>Gemma 4 teacher-forced positive-F1</t>
         </is>
       </c>
       <c r="E381" s="12" t="n">
-        <v>0.5</v>
+        <v>0.7199999999999999</v>
       </c>
       <c r="F381" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142849Z-daic_officialdev_gemma4_text_only_seed1337-22f85e6e-75450bbe, eval eval-8a5d52df50d78e5dbeae4008, selected epoch 4, best_model</t>
         </is>
       </c>
       <c r="G381" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
         </is>
       </c>
       <c r="H381" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev/text_only/daic/daic_officialdev_gemma4_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I381" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally by verify-local; REPORTABLE</t>
+          <t>recomputed locally from synced predictions; REPORTABLE</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="11" t="inlineStr">
         <is>
-          <t>DAIC Head Ablation</t>
+          <t>DAIC official development</t>
         </is>
       </c>
       <c r="B382" s="11" t="inlineStr">
@@ -21572,35 +21665,35 @@
       </c>
       <c r="C382" s="11" t="inlineStr">
         <is>
-          <t>Audio only</t>
+          <t>Text only</t>
         </is>
       </c>
       <c r="D382" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head macro-F1</t>
+          <t>Gemma 4 teacher-forced accuracy</t>
         </is>
       </c>
       <c r="E382" s="12" t="n">
-        <v>0.4484848484848484</v>
+        <v>0.8</v>
       </c>
       <c r="F382" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T142849Z-daic_officialdev_gemma4_text_only_seed1337-22f85e6e-75450bbe, eval eval-8a5d52df50d78e5dbeae4008, selected epoch 4, best_model</t>
         </is>
       </c>
       <c r="G382" s="13" t="inlineStr">
         <is>
-          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+          <t>official development partition (35 subjects), subject mean-score, teacher-forced, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
         </is>
       </c>
       <c r="H382" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev/text_only/daic/daic_officialdev_gemma4_text_only_seed1337_prod_20260813T150000Z_22f85e6e_22f85e6e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I382" s="13" t="inlineStr">
         <is>
-          <t>recomputed locally by verify-local; REPORTABLE</t>
+          <t>recomputed locally from synced predictions; REPORTABLE</t>
         </is>
       </c>
     </row>
@@ -21622,15 +21715,15 @@
       </c>
       <c r="D383" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head positive-F1</t>
+          <t>Qwen LogReg raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E383" s="12" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.5716783216783217</v>
       </c>
       <c r="F383" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G383" s="13" t="inlineStr">
@@ -21640,7 +21733,7 @@
       </c>
       <c r="H383" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I383" s="13" t="inlineStr">
@@ -21667,15 +21760,15 @@
       </c>
       <c r="D384" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head accuracy</t>
+          <t>Qwen LogReg raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E384" s="12" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.4615384615384615</v>
       </c>
       <c r="F384" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G384" s="13" t="inlineStr">
@@ -21685,7 +21778,7 @@
       </c>
       <c r="H384" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I384" s="13" t="inlineStr">
@@ -21712,15 +21805,15 @@
       </c>
       <c r="D385" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head precision</t>
+          <t>Qwen LogReg raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E385" s="12" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6</v>
       </c>
       <c r="F385" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G385" s="13" t="inlineStr">
@@ -21730,7 +21823,7 @@
       </c>
       <c r="H385" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I385" s="13" t="inlineStr">
@@ -21757,15 +21850,15 @@
       </c>
       <c r="D386" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head recall</t>
+          <t>Qwen LogReg raw hidden head precision</t>
         </is>
       </c>
       <c r="E386" s="12" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="F386" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G386" s="13" t="inlineStr">
@@ -21775,7 +21868,7 @@
       </c>
       <c r="H386" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I386" s="13" t="inlineStr">
@@ -21802,15 +21895,15 @@
       </c>
       <c r="D387" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head macro-F1</t>
+          <t>Qwen LogReg raw hidden head recall</t>
         </is>
       </c>
       <c r="E387" s="12" t="n">
-        <v>0.6499999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="F387" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-e84ce4e0072e72d7eff086bb, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G387" s="13" t="inlineStr">
@@ -21820,7 +21913,7 @@
       </c>
       <c r="H387" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I387" s="13" t="inlineStr">
@@ -21847,15 +21940,15 @@
       </c>
       <c r="D388" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head positive-F1</t>
+          <t>Qwen XGBoost raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E388" s="12" t="n">
-        <v>0.5</v>
+        <v>0.4484848484848484</v>
       </c>
       <c r="F388" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G388" s="13" t="inlineStr">
@@ -21865,7 +21958,7 @@
       </c>
       <c r="H388" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I388" s="13" t="inlineStr">
@@ -21892,15 +21985,15 @@
       </c>
       <c r="D389" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head accuracy</t>
+          <t>Qwen XGBoost raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E389" s="12" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="F389" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G389" s="13" t="inlineStr">
@@ -21910,7 +22003,7 @@
       </c>
       <c r="H389" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I389" s="13" t="inlineStr">
@@ -21937,15 +22030,15 @@
       </c>
       <c r="D390" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head precision</t>
+          <t>Qwen XGBoost raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E390" s="12" t="n">
-        <v>0.625</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="F390" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G390" s="13" t="inlineStr">
@@ -21955,7 +22048,7 @@
       </c>
       <c r="H390" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I390" s="13" t="inlineStr">
@@ -21982,15 +22075,15 @@
       </c>
       <c r="D391" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head recall</t>
+          <t>Qwen XGBoost raw hidden head precision</t>
         </is>
       </c>
       <c r="E391" s="12" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F391" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G391" s="13" t="inlineStr">
@@ -22000,7 +22093,7 @@
       </c>
       <c r="H391" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I391" s="13" t="inlineStr">
@@ -22027,15 +22120,15 @@
       </c>
       <c r="D392" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head macro-F1</t>
+          <t>Qwen XGBoost raw hidden head recall</t>
         </is>
       </c>
       <c r="E392" s="12" t="n">
-        <v>0.396551724137931</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="F392" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T154455Z-daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4-90c6cc39-269b5f37, eval eval-125e3b8f5bcc860eb4369ceb, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G392" s="13" t="inlineStr">
@@ -22045,7 +22138,7 @@
       </c>
       <c r="H392" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_only/daic/daic_officialdev_qwen_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r4/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I392" s="13" t="inlineStr">
@@ -22072,15 +22165,15 @@
       </c>
       <c r="D393" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head positive-F1</t>
+          <t>Gemma 4 LogReg raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E393" s="12" t="n">
-        <v>0</v>
+        <v>0.6499999999999999</v>
       </c>
       <c r="F393" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G393" s="13" t="inlineStr">
@@ -22090,7 +22183,7 @@
       </c>
       <c r="H393" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I393" s="13" t="inlineStr">
@@ -22117,15 +22210,15 @@
       </c>
       <c r="D394" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head accuracy</t>
+          <t>Gemma 4 LogReg raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E394" s="12" t="n">
-        <v>0.6571428571428571</v>
+        <v>0.5</v>
       </c>
       <c r="F394" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G394" s="13" t="inlineStr">
@@ -22135,7 +22228,7 @@
       </c>
       <c r="H394" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I394" s="13" t="inlineStr">
@@ -22162,15 +22255,15 @@
       </c>
       <c r="D395" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head precision</t>
+          <t>Gemma 4 LogReg raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E395" s="12" t="n">
-        <v>0</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="F395" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G395" s="13" t="inlineStr">
@@ -22180,7 +22273,7 @@
       </c>
       <c r="H395" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I395" s="13" t="inlineStr">
@@ -22207,15 +22300,15 @@
       </c>
       <c r="D396" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head recall</t>
+          <t>Gemma 4 LogReg raw hidden head precision</t>
         </is>
       </c>
       <c r="E396" s="12" t="n">
-        <v>0</v>
+        <v>0.625</v>
       </c>
       <c r="F396" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G396" s="13" t="inlineStr">
@@ -22225,7 +22318,7 @@
       </c>
       <c r="H396" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I396" s="13" t="inlineStr">
@@ -22247,20 +22340,20 @@
       </c>
       <c r="C397" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D397" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head macro-F1</t>
+          <t>Gemma 4 LogReg raw hidden head recall</t>
         </is>
       </c>
       <c r="E397" s="12" t="n">
-        <v>0.6577777777777778</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="F397" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-3e3a37d62c53729cf5db69b5, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G397" s="13" t="inlineStr">
@@ -22270,7 +22363,7 @@
       </c>
       <c r="H397" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I397" s="13" t="inlineStr">
@@ -22292,20 +22385,20 @@
       </c>
       <c r="C398" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D398" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head positive-F1</t>
+          <t>Gemma 4 XGBoost raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E398" s="12" t="n">
-        <v>0.5599999999999999</v>
+        <v>0.396551724137931</v>
       </c>
       <c r="F398" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G398" s="13" t="inlineStr">
@@ -22315,7 +22408,7 @@
       </c>
       <c r="H398" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I398" s="13" t="inlineStr">
@@ -22337,20 +22430,20 @@
       </c>
       <c r="C399" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D399" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head accuracy</t>
+          <t>Gemma 4 XGBoost raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E399" s="12" t="n">
-        <v>0.6857142857142857</v>
+        <v>0</v>
       </c>
       <c r="F399" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G399" s="13" t="inlineStr">
@@ -22360,7 +22453,7 @@
       </c>
       <c r="H399" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I399" s="13" t="inlineStr">
@@ -22382,20 +22475,20 @@
       </c>
       <c r="C400" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D400" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head precision</t>
+          <t>Gemma 4 XGBoost raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E400" s="12" t="n">
-        <v>0.5384615384615384</v>
+        <v>0.6571428571428571</v>
       </c>
       <c r="F400" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G400" s="13" t="inlineStr">
@@ -22405,7 +22498,7 @@
       </c>
       <c r="H400" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I400" s="13" t="inlineStr">
@@ -22427,20 +22520,20 @@
       </c>
       <c r="C401" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D401" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head recall</t>
+          <t>Gemma 4 XGBoost raw hidden head precision</t>
         </is>
       </c>
       <c r="E401" s="12" t="n">
-        <v>0.5833333333333334</v>
+        <v>0</v>
       </c>
       <c r="F401" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G401" s="13" t="inlineStr">
@@ -22450,7 +22543,7 @@
       </c>
       <c r="H401" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I401" s="13" t="inlineStr">
@@ -22472,20 +22565,20 @@
       </c>
       <c r="C402" s="11" t="inlineStr">
         <is>
-          <t>Audio + Text</t>
+          <t>Audio only</t>
         </is>
       </c>
       <c r="D402" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head macro-F1</t>
+          <t>Gemma 4 XGBoost raw hidden head recall</t>
         </is>
       </c>
       <c r="E402" s="12" t="n">
-        <v>0.5304437564499485</v>
+        <v>0</v>
       </c>
       <c r="F402" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T151846Z-daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2-1327849b-640f4031, eval eval-ad6e2a2ce408aed6f96f39d3, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G402" s="13" t="inlineStr">
@@ -22495,7 +22588,7 @@
       </c>
       <c r="H402" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_only/daic/daic_officialdev_gemma4_audio_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_1327849b_r2/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I402" s="13" t="inlineStr">
@@ -22522,15 +22615,15 @@
       </c>
       <c r="D403" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head positive-F1</t>
+          <t>Qwen LogReg raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E403" s="12" t="n">
-        <v>0.3157894736842105</v>
+        <v>0.6577777777777778</v>
       </c>
       <c r="F403" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G403" s="13" t="inlineStr">
@@ -22540,7 +22633,7 @@
       </c>
       <c r="H403" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I403" s="13" t="inlineStr">
@@ -22567,15 +22660,15 @@
       </c>
       <c r="D404" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head accuracy</t>
+          <t>Qwen LogReg raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E404" s="12" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.5599999999999999</v>
       </c>
       <c r="F404" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G404" s="13" t="inlineStr">
@@ -22585,7 +22678,7 @@
       </c>
       <c r="H404" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I404" s="13" t="inlineStr">
@@ -22612,15 +22705,15 @@
       </c>
       <c r="D405" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head precision</t>
+          <t>Qwen LogReg raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E405" s="12" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.6857142857142857</v>
       </c>
       <c r="F405" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G405" s="13" t="inlineStr">
@@ -22630,7 +22723,7 @@
       </c>
       <c r="H405" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I405" s="13" t="inlineStr">
@@ -22657,15 +22750,15 @@
       </c>
       <c r="D406" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head recall</t>
+          <t>Qwen LogReg raw hidden head precision</t>
         </is>
       </c>
       <c r="E406" s="12" t="n">
-        <v>0.25</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="F406" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G406" s="13" t="inlineStr">
@@ -22675,7 +22768,7 @@
       </c>
       <c r="H406" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I406" s="13" t="inlineStr">
@@ -22702,15 +22795,15 @@
       </c>
       <c r="D407" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head macro-F1</t>
+          <t>Qwen LogReg raw hidden head recall</t>
         </is>
       </c>
       <c r="E407" s="12" t="n">
-        <v>0.6829710144927537</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F407" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-536fc321c7611b917b42fdf6, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G407" s="13" t="inlineStr">
@@ -22720,7 +22813,7 @@
       </c>
       <c r="H407" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I407" s="13" t="inlineStr">
@@ -22747,15 +22840,15 @@
       </c>
       <c r="D408" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head positive-F1</t>
+          <t>Qwen XGBoost raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E408" s="12" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5304437564499485</v>
       </c>
       <c r="F408" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G408" s="13" t="inlineStr">
@@ -22765,7 +22858,7 @@
       </c>
       <c r="H408" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I408" s="13" t="inlineStr">
@@ -22792,15 +22885,15 @@
       </c>
       <c r="D409" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head accuracy</t>
+          <t>Qwen XGBoost raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E409" s="12" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.3157894736842105</v>
       </c>
       <c r="F409" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G409" s="13" t="inlineStr">
@@ -22810,7 +22903,7 @@
       </c>
       <c r="H409" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I409" s="13" t="inlineStr">
@@ -22837,15 +22930,15 @@
       </c>
       <c r="D410" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head precision</t>
+          <t>Qwen XGBoost raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E410" s="12" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6285714285714286</v>
       </c>
       <c r="F410" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G410" s="13" t="inlineStr">
@@ -22855,7 +22948,7 @@
       </c>
       <c r="H410" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I410" s="13" t="inlineStr">
@@ -22882,15 +22975,15 @@
       </c>
       <c r="D411" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head recall</t>
+          <t>Qwen XGBoost raw hidden head precision</t>
         </is>
       </c>
       <c r="E411" s="12" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="F411" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G411" s="13" t="inlineStr">
@@ -22900,7 +22993,7 @@
       </c>
       <c r="H411" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I411" s="13" t="inlineStr">
@@ -22927,15 +23020,15 @@
       </c>
       <c r="D412" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head macro-F1</t>
+          <t>Qwen XGBoost raw hidden head recall</t>
         </is>
       </c>
       <c r="E412" s="12" t="n">
-        <v>0.6829710144927537</v>
+        <v>0.25</v>
       </c>
       <c r="F412" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-b7d64c2f, eval eval-c9a4f95ffa07bebb8aa2c104, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G412" s="13" t="inlineStr">
@@ -22945,7 +23038,7 @@
       </c>
       <c r="H412" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/audio_text/daic/daic_officialdev_qwen_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I412" s="13" t="inlineStr">
@@ -22972,15 +23065,15 @@
       </c>
       <c r="D413" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head positive-F1</t>
+          <t>Gemma 4 LogReg raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E413" s="12" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6829710144927537</v>
       </c>
       <c r="F413" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G413" s="13" t="inlineStr">
@@ -22990,7 +23083,7 @@
       </c>
       <c r="H413" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I413" s="13" t="inlineStr">
@@ -23017,15 +23110,15 @@
       </c>
       <c r="D414" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head accuracy</t>
+          <t>Gemma 4 LogReg raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E414" s="12" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F414" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G414" s="13" t="inlineStr">
@@ -23035,7 +23128,7 @@
       </c>
       <c r="H414" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I414" s="13" t="inlineStr">
@@ -23062,15 +23155,15 @@
       </c>
       <c r="D415" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head precision</t>
+          <t>Gemma 4 LogReg raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E415" s="12" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="F415" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G415" s="13" t="inlineStr">
@@ -23080,7 +23173,7 @@
       </c>
       <c r="H415" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I415" s="13" t="inlineStr">
@@ -23107,7 +23200,7 @@
       </c>
       <c r="D416" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head recall</t>
+          <t>Gemma 4 LogReg raw hidden head precision</t>
         </is>
       </c>
       <c r="E416" s="12" t="n">
@@ -23115,7 +23208,7 @@
       </c>
       <c r="F416" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G416" s="13" t="inlineStr">
@@ -23125,7 +23218,7 @@
       </c>
       <c r="H416" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I416" s="13" t="inlineStr">
@@ -23147,20 +23240,20 @@
       </c>
       <c r="C417" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D417" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head macro-F1</t>
+          <t>Gemma 4 LogReg raw hidden head recall</t>
         </is>
       </c>
       <c r="E417" s="12" t="n">
-        <v>0.6938775510204083</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F417" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-70d39c1caadc8712d02ae7fb, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G417" s="13" t="inlineStr">
@@ -23170,7 +23263,7 @@
       </c>
       <c r="H417" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I417" s="13" t="inlineStr">
@@ -23192,20 +23285,20 @@
       </c>
       <c r="C418" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D418" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head positive-F1</t>
+          <t>Gemma 4 XGBoost raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E418" s="12" t="n">
-        <v>0.5714285714285715</v>
+        <v>0.6829710144927537</v>
       </c>
       <c r="F418" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G418" s="13" t="inlineStr">
@@ -23215,7 +23308,7 @@
       </c>
       <c r="H418" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I418" s="13" t="inlineStr">
@@ -23237,20 +23330,20 @@
       </c>
       <c r="C419" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D419" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head accuracy</t>
+          <t>Gemma 4 XGBoost raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E419" s="12" t="n">
-        <v>0.7428571428571429</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F419" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G419" s="13" t="inlineStr">
@@ -23260,7 +23353,7 @@
       </c>
       <c r="H419" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I419" s="13" t="inlineStr">
@@ -23282,20 +23375,20 @@
       </c>
       <c r="C420" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D420" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head precision</t>
+          <t>Gemma 4 XGBoost raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E420" s="12" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="F420" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G420" s="13" t="inlineStr">
@@ -23305,7 +23398,7 @@
       </c>
       <c r="H420" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I420" s="13" t="inlineStr">
@@ -23327,20 +23420,20 @@
       </c>
       <c r="C421" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D421" s="11" t="inlineStr">
         <is>
-          <t>Qwen LogReg raw hidden head recall</t>
+          <t>Gemma 4 XGBoost raw hidden head precision</t>
         </is>
       </c>
       <c r="E421" s="12" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F421" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G421" s="13" t="inlineStr">
@@ -23350,7 +23443,7 @@
       </c>
       <c r="H421" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I421" s="13" t="inlineStr">
@@ -23372,20 +23465,20 @@
       </c>
       <c r="C422" s="11" t="inlineStr">
         <is>
-          <t>Text only</t>
+          <t>Audio + Text</t>
         </is>
       </c>
       <c r="D422" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head macro-F1</t>
+          <t>Gemma 4 XGBoost raw hidden head recall</t>
         </is>
       </c>
       <c r="E422" s="12" t="n">
-        <v>0.6026831785345718</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="F422" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T175117Z-daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6-90c6cc39-438b3be6, eval eval-e480a1844b709554d1d22b7c, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G422" s="13" t="inlineStr">
@@ -23395,7 +23488,7 @@
       </c>
       <c r="H422" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/audio_text/daic/daic_officialdev_gemma4_audio_text_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r6/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I422" s="13" t="inlineStr">
@@ -23422,15 +23515,15 @@
       </c>
       <c r="D423" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head positive-F1</t>
+          <t>Qwen LogReg raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E423" s="12" t="n">
-        <v>0.4210526315789474</v>
+        <v>0.6938775510204083</v>
       </c>
       <c r="F423" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G423" s="13" t="inlineStr">
@@ -23440,7 +23533,7 @@
       </c>
       <c r="H423" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I423" s="13" t="inlineStr">
@@ -23467,15 +23560,15 @@
       </c>
       <c r="D424" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head accuracy</t>
+          <t>Qwen LogReg raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E424" s="12" t="n">
-        <v>0.6857142857142857</v>
+        <v>0.5714285714285715</v>
       </c>
       <c r="F424" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G424" s="13" t="inlineStr">
@@ -23485,7 +23578,7 @@
       </c>
       <c r="H424" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I424" s="13" t="inlineStr">
@@ -23512,15 +23605,15 @@
       </c>
       <c r="D425" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head precision</t>
+          <t>Qwen LogReg raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E425" s="12" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.7428571428571429</v>
       </c>
       <c r="F425" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G425" s="13" t="inlineStr">
@@ -23530,7 +23623,7 @@
       </c>
       <c r="H425" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I425" s="13" t="inlineStr">
@@ -23557,15 +23650,15 @@
       </c>
       <c r="D426" s="11" t="inlineStr">
         <is>
-          <t>Qwen XGBoost raw hidden head recall</t>
+          <t>Qwen LogReg raw hidden head precision</t>
         </is>
       </c>
       <c r="E426" s="12" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F426" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G426" s="13" t="inlineStr">
@@ -23575,7 +23668,7 @@
       </c>
       <c r="H426" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I426" s="13" t="inlineStr">
@@ -23602,15 +23695,15 @@
       </c>
       <c r="D427" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head macro-F1</t>
+          <t>Qwen LogReg raw hidden head recall</t>
         </is>
       </c>
       <c r="E427" s="12" t="n">
-        <v>0.7619047619047619</v>
+        <v>0.5</v>
       </c>
       <c r="F427" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-225153901c0e8896c9900e4a, backend qwen_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G427" s="13" t="inlineStr">
@@ -23620,7 +23713,7 @@
       </c>
       <c r="H427" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I427" s="13" t="inlineStr">
@@ -23647,15 +23740,15 @@
       </c>
       <c r="D428" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head positive-F1</t>
+          <t>Qwen XGBoost raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E428" s="12" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6026831785345718</v>
       </c>
       <c r="F428" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G428" s="13" t="inlineStr">
@@ -23665,7 +23758,7 @@
       </c>
       <c r="H428" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I428" s="13" t="inlineStr">
@@ -23692,15 +23785,15 @@
       </c>
       <c r="D429" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head accuracy</t>
+          <t>Qwen XGBoost raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E429" s="12" t="n">
-        <v>0.8</v>
+        <v>0.4210526315789474</v>
       </c>
       <c r="F429" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G429" s="13" t="inlineStr">
@@ -23710,7 +23803,7 @@
       </c>
       <c r="H429" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I429" s="13" t="inlineStr">
@@ -23737,15 +23830,15 @@
       </c>
       <c r="D430" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head precision</t>
+          <t>Qwen XGBoost raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E430" s="12" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.6857142857142857</v>
       </c>
       <c r="F430" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G430" s="13" t="inlineStr">
@@ -23755,7 +23848,7 @@
       </c>
       <c r="H430" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I430" s="13" t="inlineStr">
@@ -23782,15 +23875,15 @@
       </c>
       <c r="D431" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 LogReg raw hidden head recall</t>
+          <t>Qwen XGBoost raw hidden head precision</t>
         </is>
       </c>
       <c r="E431" s="12" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F431" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G431" s="13" t="inlineStr">
@@ -23800,7 +23893,7 @@
       </c>
       <c r="H431" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I431" s="13" t="inlineStr">
@@ -23827,15 +23920,15 @@
       </c>
       <c r="D432" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head macro-F1</t>
+          <t>Qwen XGBoost raw hidden head recall</t>
         </is>
       </c>
       <c r="E432" s="12" t="n">
-        <v>0.6685606060606061</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F432" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-f5173eec4fb4b8a5fb612e04, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T153611Z-daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3-90c6cc39-df721ed6, eval eval-28be66b87b3641742e847e9d, backend qwen_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
       <c r="G432" s="13" t="inlineStr">
@@ -23845,7 +23938,7 @@
       </c>
       <c r="H432" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_officialdev_heads/text_only/daic/daic_officialdev_qwen_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r3/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I432" s="13" t="inlineStr">
@@ -23872,15 +23965,15 @@
       </c>
       <c r="D433" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head positive-F1</t>
+          <t>Gemma 4 LogReg raw hidden head macro-F1</t>
         </is>
       </c>
       <c r="E433" s="12" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.7619047619047619</v>
       </c>
       <c r="F433" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-f5173eec4fb4b8a5fb612e04, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G433" s="13" t="inlineStr">
@@ -23890,7 +23983,7 @@
       </c>
       <c r="H433" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I433" s="13" t="inlineStr">
@@ -23917,15 +24010,15 @@
       </c>
       <c r="D434" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head accuracy</t>
+          <t>Gemma 4 LogReg raw hidden head positive-F1</t>
         </is>
       </c>
       <c r="E434" s="12" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F434" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-f5173eec4fb4b8a5fb612e04, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G434" s="13" t="inlineStr">
@@ -23935,7 +24028,7 @@
       </c>
       <c r="H434" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I434" s="13" t="inlineStr">
@@ -23962,15 +24055,15 @@
       </c>
       <c r="D435" s="11" t="inlineStr">
         <is>
-          <t>Gemma 4 XGBoost raw hidden head precision</t>
+          <t>Gemma 4 LogReg raw hidden head accuracy</t>
         </is>
       </c>
       <c r="E435" s="12" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="F435" s="13" t="inlineStr">
         <is>
-          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-f5173eec4fb4b8a5fb612e04, backend gemma4_hidden_xgb_raw, parent best_model</t>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
         </is>
       </c>
       <c r="G435" s="13" t="inlineStr">
@@ -23980,7 +24073,7 @@
       </c>
       <c r="H435" s="13" t="inlineStr">
         <is>
-          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
       <c r="I435" s="13" t="inlineStr">
@@ -24007,28 +24100,298 @@
       </c>
       <c r="D436" s="11" t="inlineStr">
         <is>
+          <t>Gemma 4 LogReg raw hidden head precision</t>
+        </is>
+      </c>
+      <c r="E436" s="12" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="F436" s="13" t="inlineStr">
+        <is>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
+        </is>
+      </c>
+      <c r="G436" s="13" t="inlineStr">
+        <is>
+          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+        </is>
+      </c>
+      <c r="H436" s="13" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I436" s="13" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local; REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="11" t="inlineStr">
+        <is>
+          <t>DAIC Head Ablation</t>
+        </is>
+      </c>
+      <c r="B437" s="11" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C437" s="11" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D437" s="11" t="inlineStr">
+        <is>
+          <t>Gemma 4 LogReg raw hidden head recall</t>
+        </is>
+      </c>
+      <c r="E437" s="12" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="F437" s="13" t="inlineStr">
+        <is>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-846a6445ccd968563f454777, backend gemma4_hidden_logreg_raw, parent best_model</t>
+        </is>
+      </c>
+      <c r="G437" s="13" t="inlineStr">
+        <is>
+          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+        </is>
+      </c>
+      <c r="H437" s="13" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/logreg/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I437" s="13" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local; REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="11" t="inlineStr">
+        <is>
+          <t>DAIC Head Ablation</t>
+        </is>
+      </c>
+      <c r="B438" s="11" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C438" s="11" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D438" s="11" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head macro-F1</t>
+        </is>
+      </c>
+      <c r="E438" s="12" t="n">
+        <v>0.6685606060606061</v>
+      </c>
+      <c r="F438" s="13" t="inlineStr">
+        <is>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-f5173eec4fb4b8a5fb612e04, backend gemma4_hidden_xgb_raw, parent best_model</t>
+        </is>
+      </c>
+      <c r="G438" s="13" t="inlineStr">
+        <is>
+          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+        </is>
+      </c>
+      <c r="H438" s="13" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I438" s="13" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local; REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="11" t="inlineStr">
+        <is>
+          <t>DAIC Head Ablation</t>
+        </is>
+      </c>
+      <c r="B439" s="11" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C439" s="11" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D439" s="11" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head positive-F1</t>
+        </is>
+      </c>
+      <c r="E439" s="12" t="n">
+        <v>0.5454545454545454</v>
+      </c>
+      <c r="F439" s="13" t="inlineStr">
+        <is>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-f5173eec4fb4b8a5fb612e04, backend gemma4_hidden_xgb_raw, parent best_model</t>
+        </is>
+      </c>
+      <c r="G439" s="13" t="inlineStr">
+        <is>
+          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+        </is>
+      </c>
+      <c r="H439" s="13" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I439" s="13" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local; REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="11" t="inlineStr">
+        <is>
+          <t>DAIC Head Ablation</t>
+        </is>
+      </c>
+      <c r="B440" s="11" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C440" s="11" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D440" s="11" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head accuracy</t>
+        </is>
+      </c>
+      <c r="E440" s="12" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="F440" s="13" t="inlineStr">
+        <is>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-f5173eec4fb4b8a5fb612e04, backend gemma4_hidden_xgb_raw, parent best_model</t>
+        </is>
+      </c>
+      <c r="G440" s="13" t="inlineStr">
+        <is>
+          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+        </is>
+      </c>
+      <c r="H440" s="13" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I440" s="13" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local; REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="11" t="inlineStr">
+        <is>
+          <t>DAIC Head Ablation</t>
+        </is>
+      </c>
+      <c r="B441" s="11" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C441" s="11" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D441" s="11" t="inlineStr">
+        <is>
+          <t>Gemma 4 XGBoost raw hidden head precision</t>
+        </is>
+      </c>
+      <c r="E441" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F441" s="13" t="inlineStr">
+        <is>
+          <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-f5173eec4fb4b8a5fb612e04, backend gemma4_hidden_xgb_raw, parent best_model</t>
+        </is>
+      </c>
+      <c r="G441" s="13" t="inlineStr">
+        <is>
+          <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
+        </is>
+      </c>
+      <c r="H441" s="13" t="inlineStr">
+        <is>
+          <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
+        </is>
+      </c>
+      <c r="I441" s="13" t="inlineStr">
+        <is>
+          <t>recomputed locally by verify-local; REPORTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="11" t="inlineStr">
+        <is>
+          <t>DAIC Head Ablation</t>
+        </is>
+      </c>
+      <c r="B442" s="11" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C442" s="11" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="D442" s="11" t="inlineStr">
+        <is>
           <t>Gemma 4 XGBoost raw hidden head recall</t>
         </is>
       </c>
-      <c r="E436" s="12" t="n">
+      <c r="E442" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="F436" s="13" t="inlineStr">
+      <c r="F442" s="13" t="inlineStr">
         <is>
           <t>campaign prod_20260813T150000Z_22f85e6e, group daic-officialdev-qwen-gemma-v1-22f85e6e473b, source 22f85e6e (clean main), Issue #60 / PR #52, manifest 72e2dd204b91… / split 441333e0c888…, attempt 20260813T163105Z-daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5-90c6cc39-bee30555, eval eval-f5173eec4fb4b8a5fb612e04, backend gemma4_hidden_xgb_raw, parent best_model</t>
         </is>
       </c>
-      <c r="G436" s="13" t="inlineStr">
+      <c r="G442" s="13" t="inlineStr">
         <is>
           <t>official development partition (35 subjects), subject mean probability &gt;= 0.5, binary-strict, harmonized_all_windows_full_coverage, daic_official_train_inner_split_dev_evaluation</t>
         </is>
       </c>
-      <c r="H436" s="13" t="inlineStr">
+      <c r="H442" s="13" t="inlineStr">
         <is>
           <t>output_model/harmonized_v1_gemma4_officialdev_heads/text_only/daic/daic_officialdev_gemma4_text_only_fixed_heads_seed1337_prod_20260813t150000z_22f85e6e_90c6cc39_r5/fold_0/hidden_classifiers/xgb/metrics.json + predictions_subject_level.csv</t>
         </is>
       </c>
-      <c r="I436" s="13" t="inlineStr">
+      <c r="I442" s="13" t="inlineStr">
         <is>
           <t>recomputed locally by verify-local; REPORTABLE</t>
         </is>

</xml_diff>

<commit_message>
Add native versus translated results sheet
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Qwen vs Gemma" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DAIC Packed30 Family" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Provenance" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Native vs EN" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DAIC Packed30 Family" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Provenance" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3996,6 +3997,1070 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Native vs English-translated transcripts — macro-F1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="92" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Paired native and English-translated transcript conditions for Qwen and Gemma 4. Delta = EN minus native; positive means translation improved macro-F1. Teacher-forced and LogReg use the harmonized best_model evidence; XGBoost uses the standardized 100-trial Optuna search, seed 1337. D3TEC/Androids = pooled 5-fold subject-level; CMDC/Turkish = 5-fold mean (train_val). Audio-only is omitted because transcript translation does not create a distinct audio-only experiment. Per-cell evidence is in the Provenance sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Modality</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Qwen native</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Qwen EN</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Qwen Δ (EN − native)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Gemma native</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Gemma EN</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Gemma Δ (EN − native)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>D3TEC</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.5589</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.6125</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0.0536</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.571399</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.564983</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>-0.0064</v>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Qwen more</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>D3TEC</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>LogReg head</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.4988</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.5464</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0.0476</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.498159</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.532292</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0.0341</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>EN better for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>D3TEC</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.523398</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0.5982</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0.07480000000000001</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.5832270000000001</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.546749</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>-0.0365</v>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Qwen more</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>D3TEC</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.6113</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.5465</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>-0.0648</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.550505</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.4936</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>-0.0569</v>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Native better for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>D3TEC</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>LogReg head</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.4651</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0.5226</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>0.0575</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.522456</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.596902</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>0.07439999999999999</v>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>EN better for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>D3TEC</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0.634535</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>0.5289</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>-0.1056</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.571942</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.5599460000000001</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Gemma more</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Androids Interview</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.8606</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>0.8873</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0.0267</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.860541</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.876968</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>0.0164</v>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>~tie for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Androids Interview</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>LogReg head</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>0.8745000000000001</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>0.8802</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>0.0057</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0.8572689999999999</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>0.902794</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>0.0455</v>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Gemma more</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Androids Interview</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0.854305</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>0.8727</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0.0184</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>0.8565469999999999</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>0.902794</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>0.0462</v>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Gemma more</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Androids Interview</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0.7317</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0.7921</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0.0604</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>0.776201</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>0.744654</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>-0.0315</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Qwen more</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Androids Interview</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>LogReg head</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>0.8326</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>0.8298</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>-0.0028</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>0.802669</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>0.83016</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>~tie for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Androids Interview</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>0.846597</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0.8111</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>-0.0355</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>0.748177</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>0.808427</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>0.0603</v>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Gemma more</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>CMDC</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>0.9856</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>0.0156</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>0.955419</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>-0.0446</v>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Qwen more</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>CMDC</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>LogReg head</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>0.9614</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0.9856</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>0.9263479999999999</v>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>-0.0737</v>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Qwen more</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>CMDC</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>0.9250890000000001</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>0.9134</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>-0.0117</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>0.984127</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>0.96828</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>-0.0158</v>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>~tie for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>CMDC</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>0.9713000000000001</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0.9713000000000001</v>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>0.957439</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>0.957439</v>
+      </c>
+      <c r="I20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>~tie for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>CMDC</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>LogReg head</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>0.9698</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>0.956334</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>0.969835</v>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>~tie for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>CMDC</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0.9539</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>0.9698</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>0.0159</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>0.924588</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>0.939796</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>0.0152</v>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>~tie for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>0.6666</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>0.6294999999999999</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>-0.0371</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>0.5657759999999999</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>0.669119</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>0.1033</v>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Gemma more</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>LogReg head</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>0.6289</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>0.6076</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>-0.0213</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>0.618816</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>0.599564</v>
+      </c>
+      <c r="I24" s="8" t="n">
+        <v>-0.0193</v>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>~tie for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Audio + Text</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>0.631141</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>0.6287</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>-0.0024</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>0.681937</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>0.592804</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>-0.0891</v>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Qwen more</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Teacher-forced</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>0.6502</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>0.6641</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>0.0139</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>0.6781779999999999</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>0.6774</v>
+      </c>
+      <c r="I26" s="8" t="n">
+        <v>-0.0008</v>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>~tie for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>LogReg head</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>0.5875</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>0.5944</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>0.558253</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>0.6014350000000001</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>0.0432</v>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>EN helps Gemma more</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Text only</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>0.589237</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>0.6584</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>0.0692</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>0.520832</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>0.629565</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>0.1087</v>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>EN better for both</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Direction uses |Δ| &lt; 0.03 as a practical tie for the compact label only; the exact deltas remain visible. This is descriptive and is not a significance test.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4505,7 +5570,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Update provenance aggregation labels for pooled cells
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -22554,7 +22554,7 @@
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>5-fold mean, teacher-forced, binary-strict, train_val protocol</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -22599,7 +22599,7 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>5-fold mean, teacher-forced, binary-strict, train_val protocol</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -22644,7 +22644,7 @@
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>5-fold mean, teacher-forced, binary-strict, train_val protocol</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
@@ -22689,7 +22689,7 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>Pooled 5-fold subject-level (62 subjects), teacher-forced, binary-strict</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
@@ -22734,7 +22734,7 @@
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>Pooled 5-fold subject-level (62 subjects), teacher-forced, binary-strict</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
@@ -22779,7 +22779,7 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>Pooled 5-fold subject-level (62 subjects), teacher-forced, binary-strict</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
@@ -22824,7 +22824,7 @@
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>Pooled 5-fold subject-level (116 subjects), teacher-forced, binary-strict</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
@@ -22869,7 +22869,7 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>Pooled 5-fold subject-level (116 subjects), teacher-forced, binary-strict</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
@@ -22914,7 +22914,7 @@
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>Pooled 5-fold subject-level (116 subjects), teacher-forced, binary-strict</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
@@ -35397,7 +35397,7 @@
       </c>
       <c r="G291" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H291" s="15" t="inlineStr">
@@ -35442,7 +35442,7 @@
       </c>
       <c r="G292" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H292" s="15" t="inlineStr">
@@ -35487,7 +35487,7 @@
       </c>
       <c r="G293" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H293" s="15" t="inlineStr">
@@ -35532,7 +35532,7 @@
       </c>
       <c r="G294" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H294" s="15" t="inlineStr">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="G295" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H295" s="15" t="inlineStr">
@@ -35622,7 +35622,7 @@
       </c>
       <c r="G296" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H296" s="15" t="inlineStr">
@@ -35667,7 +35667,7 @@
       </c>
       <c r="G297" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H297" s="15" t="inlineStr">
@@ -35712,7 +35712,7 @@
       </c>
       <c r="G298" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H298" s="15" t="inlineStr">
@@ -35757,7 +35757,7 @@
       </c>
       <c r="G299" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H299" s="15" t="inlineStr">
@@ -35802,7 +35802,7 @@
       </c>
       <c r="G300" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H300" s="15" t="inlineStr">
@@ -35847,7 +35847,7 @@
       </c>
       <c r="G301" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H301" s="15" t="inlineStr">
@@ -35892,7 +35892,7 @@
       </c>
       <c r="G302" s="15" t="inlineStr">
         <is>
-          <t>English-translated, pooled 5-fold subject-level (D3TEC/Androids) or 5-fold mean (CMDC/Turkish), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>English-translated, seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H302" s="15" t="inlineStr">
@@ -35937,7 +35937,7 @@
       </c>
       <c r="G303" s="15" t="inlineStr">
         <is>
-          <t>CV (5-fold), teacher-forced, mean over five datasets</t>
+          <t>CV (5-fold), teacher-forced, per-dataset pooled subject-level then unweighted mean over five datasets (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H303" s="15" t="inlineStr">
@@ -35982,7 +35982,7 @@
       </c>
       <c r="G304" s="15" t="inlineStr">
         <is>
-          <t>CV (5-fold), LogReg raw hidden head, mean over five datasets</t>
+          <t>CV (5-fold), LogReg raw hidden head, per-dataset pooled subject-level then unweighted mean over five datasets</t>
         </is>
       </c>
       <c r="H304" s="15" t="inlineStr">
@@ -36027,7 +36027,7 @@
       </c>
       <c r="G305" s="15" t="inlineStr">
         <is>
-          <t>CV (5-fold), teacher-forced, mean over five datasets</t>
+          <t>CV (5-fold), teacher-forced, per-dataset pooled subject-level then unweighted mean over five datasets (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H305" s="15" t="inlineStr">
@@ -36072,7 +36072,7 @@
       </c>
       <c r="G306" s="15" t="inlineStr">
         <is>
-          <t>CV (5-fold), LogReg raw hidden head, mean over five datasets</t>
+          <t>CV (5-fold), LogReg raw hidden head, per-dataset pooled subject-level then unweighted mean over five datasets</t>
         </is>
       </c>
       <c r="H306" s="15" t="inlineStr">
@@ -36117,7 +36117,7 @@
       </c>
       <c r="G307" s="15" t="inlineStr">
         <is>
-          <t>CV (5-fold), teacher-forced, mean over five datasets</t>
+          <t>CV (5-fold), teacher-forced, per-dataset pooled subject-level then unweighted mean over five datasets (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H307" s="15" t="inlineStr">
@@ -36162,7 +36162,7 @@
       </c>
       <c r="G308" s="15" t="inlineStr">
         <is>
-          <t>CV (5-fold), LogReg raw hidden head, mean over five datasets</t>
+          <t>CV (5-fold), LogReg raw hidden head, per-dataset pooled subject-level then unweighted mean over five datasets</t>
         </is>
       </c>
       <c r="H308" s="15" t="inlineStr">
@@ -36252,7 +36252,7 @@
       </c>
       <c r="G310" s="15" t="inlineStr">
         <is>
-          <t>Final (DAIC test), LogReg raw hidden head, mean over five datasets</t>
+          <t>Final (DAIC test), LogReg raw hidden head, per-dataset pooled subject-level then unweighted mean over five datasets</t>
         </is>
       </c>
       <c r="H310" s="15" t="inlineStr">
@@ -36342,7 +36342,7 @@
       </c>
       <c r="G312" s="15" t="inlineStr">
         <is>
-          <t>Final (DAIC test), LogReg raw hidden head, mean over five datasets</t>
+          <t>Final (DAIC test), LogReg raw hidden head, per-dataset pooled subject-level then unweighted mean over five datasets</t>
         </is>
       </c>
       <c r="H312" s="15" t="inlineStr">
@@ -36432,7 +36432,7 @@
       </c>
       <c r="G314" s="15" t="inlineStr">
         <is>
-          <t>Final (DAIC test), LogReg raw hidden head, mean over five datasets</t>
+          <t>Final (DAIC test), LogReg raw hidden head, per-dataset pooled subject-level then unweighted mean over five datasets</t>
         </is>
       </c>
       <c r="H314" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Drop duplicate pre-campaign Turkish rows from pooled audit
Turkish cells come only from the pooled-campaign provenance; the
three-route evidence still carried pre-campaign Turkish folds that
duplicated the workbook rows in the audit and the Pooled vs Fold-Mean
sheet. Exclude dataset=turkish from standalone_rows.
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L196"/>
+  <dimension ref="A1:L166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7168,7 +7168,7 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
@@ -7192,33 +7192,33 @@
         </is>
       </c>
       <c r="F137" s="5" t="n">
-        <v>0.468</v>
+        <v>0.489</v>
       </c>
       <c r="G137" s="5" t="n">
-        <v>0.4621</v>
+        <v>0.4788</v>
       </c>
       <c r="H137" s="5" t="n">
-        <v>0.0058</v>
+        <v>0.0102</v>
       </c>
       <c r="I137" s="5" t="n">
-        <v>0.0862</v>
+        <v>0.1017</v>
       </c>
       <c r="J137" s="5" t="n">
-        <v>0.7931</v>
+        <v>0.8041</v>
       </c>
       <c r="K137" s="5" t="n">
-        <v>0.7927999999999999</v>
+        <v>0.8048</v>
       </c>
       <c r="L137" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f3_f24783ac/fold_3/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f3_f24783ac_logreg-bfe9577d-c4b62436/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s7_f2_b8e9d164/fold_2/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s7_f2_b8e9d164_logreg-bfe9577d-58eec2b5/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e_logreg-bfe9577d-e258bbd9/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765_logreg-bfe9577d-1280f4a3/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
@@ -7242,33 +7242,33 @@
         </is>
       </c>
       <c r="F138" s="5" t="n">
-        <v>0.4324</v>
+        <v>0.4089</v>
       </c>
       <c r="G138" s="5" t="n">
-        <v>0.4084</v>
+        <v>0.4089</v>
       </c>
       <c r="H138" s="5" t="n">
-        <v>0.0241</v>
+        <v>-0.0001</v>
       </c>
       <c r="I138" s="5" t="n">
-        <v>0.0049</v>
+        <v>0.0038</v>
       </c>
       <c r="J138" s="5" t="n">
-        <v>0.8013</v>
+        <v>0.8177</v>
       </c>
       <c r="K138" s="5" t="n">
-        <v>0.7935</v>
+        <v>0.8179</v>
       </c>
       <c r="L138" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s2024_f1_2f041c03/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s7_f1_90dedfd8/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
@@ -7292,33 +7292,33 @@
         </is>
       </c>
       <c r="F139" s="5" t="n">
-        <v>0.5607</v>
+        <v>0.5252</v>
       </c>
       <c r="G139" s="5" t="n">
-        <v>0.5504</v>
+        <v>0.5052</v>
       </c>
       <c r="H139" s="5" t="n">
-        <v>0.0102</v>
+        <v>0.02</v>
       </c>
       <c r="I139" s="5" t="n">
-        <v>0.0867</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="J139" s="5" t="n">
-        <v>0.7095</v>
+        <v>0.6914</v>
       </c>
       <c r="K139" s="5" t="n">
-        <v>0.6992</v>
+        <v>0.6751</v>
       </c>
       <c r="L139" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s7_f0_4cc22340/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s7_f0_4cc22340_xgb_optuna100-bfe9577d-2a77f72a/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e_xgb_optuna100-bfe9577d-7f7ecd36/xgb_optuna100_harmonized_v1/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e_xgb_optuna100-bfe9577d-7f7ecd36/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765_xgb_optuna100-bfe9577d-9f33da38/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
@@ -7342,33 +7342,33 @@
         </is>
       </c>
       <c r="F140" s="5" t="n">
-        <v>0.4982</v>
+        <v>0.509</v>
       </c>
       <c r="G140" s="5" t="n">
-        <v>0.4807</v>
+        <v>0.4936</v>
       </c>
       <c r="H140" s="5" t="n">
-        <v>0.0175</v>
+        <v>0.0154</v>
       </c>
       <c r="I140" s="5" t="n">
-        <v>0.1019</v>
+        <v>0.1024</v>
       </c>
       <c r="J140" s="5" t="n">
-        <v>0.7937</v>
+        <v>0.7872</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>0.7935</v>
+        <v>0.7872</v>
       </c>
       <c r="L140" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s2024_f0_663d32df/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s2024_f0_663d32df_logreg-bfe9577d-f49486eb/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8_logreg-bfe9577d-a745ea9e/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8_logreg-bfe9577d-a745ea9e/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d_logreg-bfe9577d-4aefc02f/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
@@ -7392,33 +7392,33 @@
         </is>
       </c>
       <c r="F141" s="5" t="n">
-        <v>0.4907</v>
+        <v>0.4089</v>
       </c>
       <c r="G141" s="5" t="n">
-        <v>0.4479</v>
+        <v>0.4089</v>
       </c>
       <c r="H141" s="5" t="n">
-        <v>0.0428</v>
+        <v>-0.0001</v>
       </c>
       <c r="I141" s="5" t="n">
-        <v>0.0953</v>
+        <v>0.0038</v>
       </c>
       <c r="J141" s="5" t="n">
-        <v>0.8062</v>
+        <v>0.8177</v>
       </c>
       <c r="K141" s="5" t="n">
-        <v>0.8022</v>
+        <v>0.8179</v>
       </c>
       <c r="L141" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f3_89772359/fold_3/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s2024_f4_7b633d8b/fold_4/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
@@ -7442,33 +7442,33 @@
         </is>
       </c>
       <c r="F142" s="5" t="n">
-        <v>0.5868</v>
+        <v>0.6097</v>
       </c>
       <c r="G142" s="5" t="n">
-        <v>0.5767</v>
+        <v>0.6107</v>
       </c>
       <c r="H142" s="5" t="n">
-        <v>0.0101</v>
+        <v>-0.0011</v>
       </c>
       <c r="I142" s="5" t="n">
-        <v>0.1181</v>
+        <v>0.1292</v>
       </c>
       <c r="J142" s="5" t="n">
-        <v>0.7716</v>
+        <v>0.7886</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>0.767</v>
+        <v>0.7865</v>
       </c>
       <c r="L142" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f4_e6396729/fold_4/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f4_e6396729_xgb_optuna100-bfe9577d-8eba62ae/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s2024_f1_8a47366e/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s2024_f1_8a47366e_xgb_optuna100-bfe9577d-9cab10a5/xgb_optuna100_harmonized_v1/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8_xgb_optuna100-bfe9577d-ca2d5d5a/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d_xgb_optuna100-bfe9577d-8e66f104/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
@@ -7492,33 +7492,33 @@
         </is>
       </c>
       <c r="F143" s="5" t="n">
-        <v>0.68</v>
+        <v>0.6887</v>
       </c>
       <c r="G143" s="5" t="n">
-        <v>0.6802</v>
+        <v>0.6913</v>
       </c>
       <c r="H143" s="5" t="n">
-        <v>-0.0002</v>
+        <v>-0.0027</v>
       </c>
       <c r="I143" s="5" t="n">
-        <v>0.1195</v>
+        <v>0.09569999999999999</v>
       </c>
       <c r="J143" s="5" t="n">
-        <v>0.8</v>
+        <v>0.795</v>
       </c>
       <c r="K143" s="5" t="n">
-        <v>0.794</v>
+        <v>0.7906</v>
       </c>
       <c r="L143" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s2024_f3_1bcf5172/fold_3/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s2024_f3_1bcf5172_logreg-bfe9577d-8949c443/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f2_f0e6d6b7/fold_2/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f2_f0e6d6b7_logreg-bfe9577d-8aab67b3/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57_logreg-bfe9577d-f3c53a19/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db_logreg-bfe9577d-a1db4310/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
@@ -7542,33 +7542,33 @@
         </is>
       </c>
       <c r="F144" s="5" t="n">
-        <v>0.6979</v>
+        <v>0.7069</v>
       </c>
       <c r="G144" s="5" t="n">
-        <v>0.6993</v>
+        <v>0.7052</v>
       </c>
       <c r="H144" s="5" t="n">
-        <v>-0.0014</v>
+        <v>0.0017</v>
       </c>
       <c r="I144" s="5" t="n">
-        <v>0.0901</v>
+        <v>0.1009</v>
       </c>
       <c r="J144" s="5" t="n">
-        <v>0.8129</v>
+        <v>0.8193</v>
       </c>
       <c r="K144" s="5" t="n">
-        <v>0.8099</v>
+        <v>0.8133</v>
       </c>
       <c r="L144" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57_logreg-bfe9577d-f3c53a19/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s2024_f0_3a477ebe/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s2024_f0_3a477ebe_logreg-bfe9577d-e4e33eed/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820_logreg-bfe9577d-8529f031/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489_logreg-bfe9577d-ec33ced8/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
@@ -7592,33 +7592,33 @@
         </is>
       </c>
       <c r="F145" s="5" t="n">
-        <v>0.7192</v>
+        <v>0.7222</v>
       </c>
       <c r="G145" s="5" t="n">
         <v>0.7197</v>
       </c>
       <c r="H145" s="5" t="n">
-        <v>-0.0005</v>
+        <v>0.0025</v>
       </c>
       <c r="I145" s="5" t="n">
-        <v>0.0893</v>
+        <v>0.08890000000000001</v>
       </c>
       <c r="J145" s="5" t="n">
-        <v>0.8346</v>
+        <v>0.8333</v>
       </c>
       <c r="K145" s="5" t="n">
-        <v>0.833</v>
+        <v>0.8288</v>
       </c>
       <c r="L145" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f4_c8c960e8/fold_4/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s7_f4_69ee1472/fold_4/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
@@ -7642,33 +7642,33 @@
         </is>
       </c>
       <c r="F146" s="5" t="n">
-        <v>0.7408</v>
+        <v>0.7024</v>
       </c>
       <c r="G146" s="5" t="n">
-        <v>0.7372</v>
+        <v>0.6963</v>
       </c>
       <c r="H146" s="5" t="n">
-        <v>0.0036</v>
+        <v>0.0061</v>
       </c>
       <c r="I146" s="5" t="n">
-        <v>0.0963</v>
+        <v>0.0764</v>
       </c>
       <c r="J146" s="5" t="n">
-        <v>0.8423</v>
+        <v>0.8214</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>0.8404</v>
+        <v>0.8191000000000001</v>
       </c>
       <c r="L146" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s2024_f3_b7232ba9/fold_3/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f3_2203f400/fold_3/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
@@ -7692,33 +7692,33 @@
         </is>
       </c>
       <c r="F147" s="5" t="n">
-        <v>0.6899</v>
+        <v>0.7</v>
       </c>
       <c r="G147" s="5" t="n">
-        <v>0.6907</v>
+        <v>0.703</v>
       </c>
       <c r="H147" s="5" t="n">
-        <v>-0.0008</v>
+        <v>-0.003</v>
       </c>
       <c r="I147" s="5" t="n">
-        <v>0.1019</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="J147" s="5" t="n">
-        <v>0.8096</v>
+        <v>0.8</v>
       </c>
       <c r="K147" s="5" t="n">
-        <v>0.8058999999999999</v>
+        <v>0.7984</v>
       </c>
       <c r="L147" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f4_c8c960e8/fold_4/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f4_c8c960e8_xgb_optuna100-bfe9577d-8bcbd5bf/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s2024_f0_f6da111d/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s2024_f0_f6da111d_xgb_optuna100-bfe9577d-4101a0ba/xgb_optuna100_harmonized_v1/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57_xgb_optuna100-bfe9577d-dd9d4826/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db_xgb_optuna100-bfe9577d-32f966f6/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
@@ -7742,33 +7742,33 @@
         </is>
       </c>
       <c r="F148" s="5" t="n">
-        <v>0.7381</v>
+        <v>0.6825</v>
       </c>
       <c r="G148" s="5" t="n">
-        <v>0.7388</v>
+        <v>0.6848</v>
       </c>
       <c r="H148" s="5" t="n">
-        <v>-0.0007</v>
+        <v>-0.0022</v>
       </c>
       <c r="I148" s="5" t="n">
-        <v>0.09</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="J148" s="5" t="n">
-        <v>0.8327</v>
+        <v>0.8095</v>
       </c>
       <c r="K148" s="5" t="n">
-        <v>0.8300999999999999</v>
+        <v>0.803</v>
       </c>
       <c r="L148" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s7_f4_14a9e5f1/fold_4/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s7_f4_14a9e5f1_xgb_optuna100-bfe9577d-ed087ef2/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s2024_f1_e71bc79c/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s2024_f1_e71bc79c_xgb_optuna100-bfe9577d-d97e5ea2/xgb_optuna100_harmonized_v1/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820_xgb_optuna100-bfe9577d-7e5ff6e7/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489_xgb_optuna100-bfe9577d-d484976c/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
@@ -7792,33 +7792,33 @@
         </is>
       </c>
       <c r="F149" s="5" t="n">
-        <v>0.6555</v>
+        <v>0.7188</v>
       </c>
       <c r="G149" s="5" t="n">
-        <v>0.6535</v>
+        <v>0.7235</v>
       </c>
       <c r="H149" s="5" t="n">
-        <v>0.002</v>
+        <v>-0.0048</v>
       </c>
       <c r="I149" s="5" t="n">
-        <v>0.06660000000000001</v>
+        <v>0.1409</v>
       </c>
       <c r="J149" s="5" t="n">
-        <v>0.7904</v>
+        <v>0.8125</v>
       </c>
       <c r="K149" s="5" t="n">
-        <v>0.7867</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="L149" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s2024_f1_f578f90e/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s2024_f1_f578f90e_logreg-bfe9577d-ea3ba119/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f4_7d149f64/fold_4/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f4_7d149f64_logreg-bfe9577d-a25c36c1/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357/fold_0/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357_logreg-bfe9577d-47b66836/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea/fold_1/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea_logreg-bfe9577d-9477a678/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
@@ -7842,33 +7842,33 @@
         </is>
       </c>
       <c r="F150" s="5" t="n">
-        <v>0.7113</v>
+        <v>0.6773</v>
       </c>
       <c r="G150" s="5" t="n">
-        <v>0.7141</v>
+        <v>0.6778</v>
       </c>
       <c r="H150" s="5" t="n">
-        <v>-0.0028</v>
+        <v>-0.0005</v>
       </c>
       <c r="I150" s="5" t="n">
-        <v>0.1126</v>
+        <v>0.0623</v>
       </c>
       <c r="J150" s="5" t="n">
-        <v>0.8131</v>
+        <v>0.8118</v>
       </c>
       <c r="K150" s="5" t="n">
-        <v>0.8107</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L150" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f3_a85aecfd/fold_3/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s1337_f3_a85aecfd_logreg-bfe9577d-99bf8af8/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s2024_f0_6ccecf38/fold_0/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s2024_f0_6ccecf38_logreg-bfe9577d-5228f907/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850_logreg-bfe9577d-6c33c214/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034_logreg-bfe9577d-9dcc05f3/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
@@ -7892,33 +7892,33 @@
         </is>
       </c>
       <c r="F151" s="5" t="n">
-        <v>0.6858</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G151" s="5" t="n">
-        <v>0.6831</v>
+        <v>0.6877</v>
       </c>
       <c r="H151" s="5" t="n">
-        <v>0.0027</v>
+        <v>0.0023</v>
       </c>
       <c r="I151" s="5" t="n">
-        <v>0.0545</v>
+        <v>0.0421</v>
       </c>
       <c r="J151" s="5" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.8166</v>
       </c>
       <c r="K151" s="5" t="n">
-        <v>0.8126</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="L151" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s2024_f3_247b3e16/fold_3/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
@@ -7942,33 +7942,33 @@
         </is>
       </c>
       <c r="F152" s="5" t="n">
-        <v>0.7314000000000001</v>
+        <v>0.7421</v>
       </c>
       <c r="G152" s="5" t="n">
-        <v>0.7309</v>
+        <v>0.7403999999999999</v>
       </c>
       <c r="H152" s="5" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0017</v>
       </c>
       <c r="I152" s="5" t="n">
-        <v>0.0999</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="J152" s="5" t="n">
-        <v>0.8396</v>
+        <v>0.8452</v>
       </c>
       <c r="K152" s="5" t="n">
-        <v>0.8375</v>
+        <v>0.8464</v>
       </c>
       <c r="L152" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s7_f2_10e91045/fold_2/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s2024_f1_a4e19b91/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
@@ -7992,33 +7992,33 @@
         </is>
       </c>
       <c r="F153" s="5" t="n">
-        <v>0.6395999999999999</v>
+        <v>0.6791</v>
       </c>
       <c r="G153" s="5" t="n">
-        <v>0.6365</v>
+        <v>0.6792</v>
       </c>
       <c r="H153" s="5" t="n">
-        <v>0.0031</v>
+        <v>-0.0001</v>
       </c>
       <c r="I153" s="5" t="n">
-        <v>0.0703</v>
+        <v>0.066</v>
       </c>
       <c r="J153" s="5" t="n">
-        <v>0.7938</v>
+        <v>0.8208</v>
       </c>
       <c r="K153" s="5" t="n">
-        <v>0.7917999999999999</v>
+        <v>0.8217</v>
       </c>
       <c r="L153" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f4_7d149f64/fold_4/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f4_7d149f64_xgb_optuna100-bfe9577d-2b0231dd/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s7_f0_6a77b88a/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s7_f0_6a77b88a_xgb_optuna100-bfe9577d-d350431d/xgb_optuna100_harmonized_v1/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850_xgb_optuna100-bfe9577d-ccfc176c/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034_xgb_optuna100-bfe9577d-93a65d16/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
@@ -8042,33 +8042,33 @@
         </is>
       </c>
       <c r="F154" s="5" t="n">
-        <v>0.7161999999999999</v>
+        <v>0.7036</v>
       </c>
       <c r="G154" s="5" t="n">
-        <v>0.7201</v>
+        <v>0.7088</v>
       </c>
       <c r="H154" s="5" t="n">
-        <v>-0.0039</v>
+        <v>-0.0052</v>
       </c>
       <c r="I154" s="5" t="n">
-        <v>0.1152</v>
+        <v>0.1274</v>
       </c>
       <c r="J154" s="5" t="n">
-        <v>0.8219</v>
+        <v>0.8098</v>
       </c>
       <c r="K154" s="5" t="n">
-        <v>0.8189</v>
+        <v>0.8055</v>
       </c>
       <c r="L154" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s2024_f0_6ccecf38/fold_0/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s2024_f0_6ccecf38_xgb_optuna100-bfe9577d-7325d402/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s2024_f1_a4e19b91/fold_1/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s2024_f1_a4e19b91_xgb_optuna100-bfe9577d-4b593e0f/xgb_optuna100_harmonized_v1/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357/fold_0/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357_xgb_optuna100-bfe9577d-59c62f9c/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea/fold_1/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea_xgb_optuna100-bfe9577d-0c0bb912/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
@@ -8092,33 +8092,33 @@
         </is>
       </c>
       <c r="F155" s="5" t="n">
-        <v>0.5355</v>
+        <v>0.5672</v>
       </c>
       <c r="G155" s="5" t="n">
-        <v>0.5337</v>
+        <v>0.5714</v>
       </c>
       <c r="H155" s="5" t="n">
-        <v>0.0018</v>
+        <v>-0.0042</v>
       </c>
       <c r="I155" s="5" t="n">
-        <v>0.1212</v>
+        <v>0.1271</v>
       </c>
       <c r="J155" s="5" t="n">
-        <v>0.6929</v>
+        <v>0.7006</v>
       </c>
       <c r="K155" s="5" t="n">
-        <v>0.6836</v>
+        <v>0.6893</v>
       </c>
       <c r="L155" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s2024_f2_7b5b6bb5/fold_2/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s2024_f2_7b5b6bb5_logreg-bfe9577d-b99dc945/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s7_f0_7f309a77/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s7_f0_7f309a77_logreg-bfe9577d-3ede1ec0/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f_logreg-bfe9577d-b7a21ba4/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75_logreg-bfe9577d-07136c2f/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
@@ -8142,33 +8142,33 @@
         </is>
       </c>
       <c r="F156" s="5" t="n">
-        <v>0.5789</v>
+        <v>0.6237</v>
       </c>
       <c r="G156" s="5" t="n">
-        <v>0.5732</v>
+        <v>0.6122</v>
       </c>
       <c r="H156" s="5" t="n">
-        <v>0.0058</v>
+        <v>0.0115</v>
       </c>
       <c r="I156" s="5" t="n">
-        <v>0.08110000000000001</v>
+        <v>0.0575</v>
       </c>
       <c r="J156" s="5" t="n">
-        <v>0.745</v>
+        <v>0.7836</v>
       </c>
       <c r="K156" s="5" t="n">
-        <v>0.737</v>
+        <v>0.7774</v>
       </c>
       <c r="L156" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s2024_f4_57e9259c/fold_4/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s2024_f4_57e9259c_logreg-bfe9577d-e4383bc4/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s2024_f1_659ecae2/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s2024_f1_659ecae2_logreg-bfe9577d-30721950/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d_logreg-bfe9577d-fd85e1d1/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f_logreg-bfe9577d-0453b200/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
@@ -8192,33 +8192,33 @@
         </is>
       </c>
       <c r="F157" s="5" t="n">
-        <v>0.4799</v>
+        <v>0.5185999999999999</v>
       </c>
       <c r="G157" s="5" t="n">
-        <v>0.4425</v>
+        <v>0.4897</v>
       </c>
       <c r="H157" s="5" t="n">
-        <v>0.0373</v>
+        <v>0.0289</v>
       </c>
       <c r="I157" s="5" t="n">
-        <v>0.075</v>
+        <v>0.1008</v>
       </c>
       <c r="J157" s="5" t="n">
-        <v>0.7327</v>
+        <v>0.6951000000000001</v>
       </c>
       <c r="K157" s="5" t="n">
-        <v>0.7193000000000001</v>
+        <v>0.6821</v>
       </c>
       <c r="L157" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f4_6b803db6/fold_4/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s2024_f4_10431e3e/fold_4/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
@@ -8242,33 +8242,33 @@
         </is>
       </c>
       <c r="F158" s="5" t="n">
-        <v>0.508</v>
+        <v>0.5036</v>
       </c>
       <c r="G158" s="5" t="n">
-        <v>0.4807</v>
+        <v>0.4556</v>
       </c>
       <c r="H158" s="5" t="n">
-        <v>0.0272</v>
+        <v>0.048</v>
       </c>
       <c r="I158" s="5" t="n">
-        <v>0.0987</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="J158" s="5" t="n">
-        <v>0.7075</v>
+        <v>0.7806999999999999</v>
       </c>
       <c r="K158" s="5" t="n">
-        <v>0.6963</v>
+        <v>0.7726</v>
       </c>
       <c r="L158" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f2_2e58695a/fold_2/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f3_96ca2a7a/fold_3/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
@@ -8292,33 +8292,33 @@
         </is>
       </c>
       <c r="F159" s="5" t="n">
-        <v>0.6452</v>
+        <v>0.65</v>
       </c>
       <c r="G159" s="5" t="n">
-        <v>0.6425</v>
+        <v>0.6494</v>
       </c>
       <c r="H159" s="5" t="n">
-        <v>0.0027</v>
+        <v>0.0005</v>
       </c>
       <c r="I159" s="5" t="n">
-        <v>0.1408</v>
+        <v>0.1533</v>
       </c>
       <c r="J159" s="5" t="n">
-        <v>0.7881</v>
+        <v>0.7929</v>
       </c>
       <c r="K159" s="5" t="n">
-        <v>0.7857</v>
+        <v>0.7911</v>
       </c>
       <c r="L159" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f4_6b803db6/fold_4/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s1337_f4_6b803db6_xgb_optuna100-bfe9577d-17e8f33a/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s7_f3_09631886/fold_3/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s7_f3_09631886_xgb_optuna100-bfe9577d-c94c45f4/xgb_optuna100_harmonized_v1/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f_xgb_optuna100-bfe9577d-9b93d865/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75_xgb_optuna100-bfe9577d-dc27af92/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -8342,33 +8342,33 @@
         </is>
       </c>
       <c r="F160" s="5" t="n">
-        <v>0.5979</v>
+        <v>0.6149</v>
       </c>
       <c r="G160" s="5" t="n">
-        <v>0.5969</v>
+        <v>0.6143999999999999</v>
       </c>
       <c r="H160" s="5" t="n">
-        <v>0.001</v>
+        <v>0.0005</v>
       </c>
       <c r="I160" s="5" t="n">
-        <v>0.0819</v>
+        <v>0.0613</v>
       </c>
       <c r="J160" s="5" t="n">
-        <v>0.7464</v>
+        <v>0.7561</v>
       </c>
       <c r="K160" s="5" t="n">
-        <v>0.7405</v>
+        <v>0.7523</v>
       </c>
       <c r="L160" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s7_f0_aaf39920/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s7_f0_aaf39920_xgb_optuna100-bfe9577d-2ab93e38/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s7_f4_198d1eed/fold_4/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s7_f4_198d1eed_xgb_optuna100-bfe9577d-9fb46967/xgb_optuna100_harmonized_v1/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d_xgb_optuna100-bfe9577d-4729fcf4/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f_xgb_optuna100-bfe9577d-f16d5f67/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -8392,33 +8392,33 @@
         </is>
       </c>
       <c r="F161" s="5" t="n">
-        <v>0.584</v>
+        <v>0.5663</v>
       </c>
       <c r="G161" s="5" t="n">
-        <v>0.5803</v>
+        <v>0.5605</v>
       </c>
       <c r="H161" s="5" t="n">
-        <v>0.0037</v>
+        <v>0.0059</v>
       </c>
       <c r="I161" s="5" t="n">
-        <v>0.1239</v>
+        <v>0.0781</v>
       </c>
       <c r="J161" s="5" t="n">
-        <v>0.6787</v>
+        <v>0.6711</v>
       </c>
       <c r="K161" s="5" t="n">
-        <v>0.6729000000000001</v>
+        <v>0.6559</v>
       </c>
       <c r="L161" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s2024_f4_8289db83/fold_4/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s2024_f4_8289db83_logreg-bfe9577d-b27e2378/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s2024_f3_79fad815/fold_3/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s2024_f3_79fad815_logreg-bfe9577d-3f4dc9b3/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f0_49e543a1/fold_0/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s1337_f0_49e543a1_logreg-bfe9577d-8abf5ac5/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f1_7a0529bf/fold_1/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s1337_f1_7a0529bf_logreg-bfe9577d-96105eb5/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
@@ -8442,33 +8442,33 @@
         </is>
       </c>
       <c r="F162" s="5" t="n">
-        <v>0.5581</v>
+        <v>0.616</v>
       </c>
       <c r="G162" s="5" t="n">
-        <v>0.5518999999999999</v>
+        <v>0.6127</v>
       </c>
       <c r="H162" s="5" t="n">
-        <v>0.0062</v>
+        <v>0.0033</v>
       </c>
       <c r="I162" s="5" t="n">
-        <v>0.0772</v>
+        <v>0.098</v>
       </c>
       <c r="J162" s="5" t="n">
-        <v>0.6637</v>
+        <v>0.7151999999999999</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>0.6493</v>
+        <v>0.7131999999999999</v>
       </c>
       <c r="L162" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s2024_f4_8f077e9f/fold_4/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s2024_f4_8f077e9f_logreg-bfe9577d-f8e3beee/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f4_a5ff8699/fold_4/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s1337_f4_a5ff8699_logreg-bfe9577d-e47a10a0/classifier/logreg_raw/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30_logreg-bfe9577d-b7d028e5/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd_logreg-bfe9577d-1d78c089/classifier/logreg_raw/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
@@ -8492,33 +8492,33 @@
         </is>
       </c>
       <c r="F163" s="5" t="n">
-        <v>0.4526</v>
+        <v>0.4667</v>
       </c>
       <c r="G163" s="5" t="n">
-        <v>0.4174</v>
+        <v>0.4379</v>
       </c>
       <c r="H163" s="5" t="n">
-        <v>0.0353</v>
+        <v>0.0288</v>
       </c>
       <c r="I163" s="5" t="n">
-        <v>0.0179</v>
+        <v>0.0586</v>
       </c>
       <c r="J163" s="5" t="n">
-        <v>0.7719</v>
+        <v>0.8</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>0.7578</v>
+        <v>0.7957</v>
       </c>
       <c r="L163" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s7_f3_190a5e2a/fold_3/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s2024_f3_79fad815/fold_3/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f0_49e543a1/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f1_7a0529bf/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
@@ -8542,33 +8542,33 @@
         </is>
       </c>
       <c r="F164" s="5" t="n">
-        <v>0.473</v>
+        <v>0.4504</v>
       </c>
       <c r="G164" s="5" t="n">
-        <v>0.4384</v>
+        <v>0.4174</v>
       </c>
       <c r="H164" s="5" t="n">
-        <v>0.0346</v>
+        <v>0.0331</v>
       </c>
       <c r="I164" s="5" t="n">
-        <v>0.075</v>
+        <v>0.0179</v>
       </c>
       <c r="J164" s="5" t="n">
-        <v>0.776</v>
+        <v>0.7527</v>
       </c>
       <c r="K164" s="5" t="n">
-        <v>0.7669</v>
+        <v>0.7373</v>
       </c>
       <c r="L164" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s7_f3_9ec72d12/fold_3/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f4_a5ff8699/fold_4/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
@@ -8592,33 +8592,33 @@
         </is>
       </c>
       <c r="F165" s="5" t="n">
-        <v>0.64</v>
+        <v>0.6804</v>
       </c>
       <c r="G165" s="5" t="n">
-        <v>0.6245000000000001</v>
+        <v>0.6687</v>
       </c>
       <c r="H165" s="5" t="n">
-        <v>0.0155</v>
+        <v>0.0117</v>
       </c>
       <c r="I165" s="5" t="n">
-        <v>0.1234</v>
+        <v>0.09470000000000001</v>
       </c>
       <c r="J165" s="5" t="n">
-        <v>0.8</v>
+        <v>0.8295</v>
       </c>
       <c r="K165" s="5" t="n">
-        <v>0.7979000000000001</v>
+        <v>0.8268</v>
       </c>
       <c r="L165" s="5" t="inlineStr">
         <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s7_f1_7aadb61e/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s7_f1_7aadb61e_xgb_optuna100-bfe9577d-87c76868/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s7_f2_5bcb0a51/fold_2/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s7_f2_5bcb0a51_xgb_optuna100-bfe9577d-47e0faee/xgb_optuna100_harmonized_v1/metrics.json</t>
+          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30_xgb_optuna100-bfe9577d-28adfca1/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd_xgb_optuna100-bfe9577d-667cf4ba/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>standalone</t>
+          <t>turkish_pooled</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
@@ -8642,1524 +8642,24 @@
         </is>
       </c>
       <c r="F166" s="5" t="n">
-        <v>0.663</v>
+        <v>0.637</v>
       </c>
       <c r="G166" s="5" t="n">
-        <v>0.6589</v>
+        <v>0.6306</v>
       </c>
       <c r="H166" s="5" t="n">
-        <v>0.0041</v>
+        <v>0.0063</v>
       </c>
       <c r="I166" s="5" t="n">
-        <v>0.0483</v>
+        <v>0.0293</v>
       </c>
       <c r="J166" s="5" t="n">
-        <v>0.7903</v>
+        <v>0.7882</v>
       </c>
       <c r="K166" s="5" t="n">
-        <v>0.7869</v>
+        <v>0.7843</v>
       </c>
       <c r="L166" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s7_f4_e7ca3056/fold_4/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s7_f4_e7ca3056_xgb_optuna100-bfe9577d-19730929/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s2024_f2_6edf81a7/fold_2/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s2024_f2_6edf81a7_xgb_optuna100-bfe9577d-0df4c697/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B167" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C167" s="4" t="inlineStr">
-        <is>
-          <t>Audio only</t>
-        </is>
-      </c>
-      <c r="D167" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E167" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F167" s="5" t="n">
-        <v>0.489</v>
-      </c>
-      <c r="G167" s="5" t="n">
-        <v>0.4788</v>
-      </c>
-      <c r="H167" s="5" t="n">
-        <v>0.0102</v>
-      </c>
-      <c r="I167" s="5" t="n">
-        <v>0.1017</v>
-      </c>
-      <c r="J167" s="5" t="n">
-        <v>0.8041</v>
-      </c>
-      <c r="K167" s="5" t="n">
-        <v>0.8048</v>
-      </c>
-      <c r="L167" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e_logreg-bfe9577d-e258bbd9/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765_logreg-bfe9577d-1280f4a3/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B168" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C168" s="4" t="inlineStr">
-        <is>
-          <t>Audio only</t>
-        </is>
-      </c>
-      <c r="D168" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E168" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F168" s="5" t="n">
-        <v>0.4089</v>
-      </c>
-      <c r="G168" s="5" t="n">
-        <v>0.4089</v>
-      </c>
-      <c r="H168" s="5" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="I168" s="5" t="n">
-        <v>0.0038</v>
-      </c>
-      <c r="J168" s="5" t="n">
-        <v>0.8177</v>
-      </c>
-      <c r="K168" s="5" t="n">
-        <v>0.8179</v>
-      </c>
-      <c r="L168" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B169" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C169" s="4" t="inlineStr">
-        <is>
-          <t>Audio only</t>
-        </is>
-      </c>
-      <c r="D169" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E169" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F169" s="5" t="n">
-        <v>0.5252</v>
-      </c>
-      <c r="G169" s="5" t="n">
-        <v>0.5052</v>
-      </c>
-      <c r="H169" s="5" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="I169" s="5" t="n">
-        <v>0.06419999999999999</v>
-      </c>
-      <c r="J169" s="5" t="n">
-        <v>0.6914</v>
-      </c>
-      <c r="K169" s="5" t="n">
-        <v>0.6751</v>
-      </c>
-      <c r="L169" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f0_2d90e51e_xgb_optuna100-bfe9577d-7f7ecd36/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_only/audio_only/turkish/tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_only_s1337_f1_38afb765_xgb_optuna100-bfe9577d-9f33da38/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B170" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C170" s="4" t="inlineStr">
-        <is>
-          <t>Audio only</t>
-        </is>
-      </c>
-      <c r="D170" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E170" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F170" s="5" t="n">
-        <v>0.509</v>
-      </c>
-      <c r="G170" s="5" t="n">
-        <v>0.4936</v>
-      </c>
-      <c r="H170" s="5" t="n">
-        <v>0.0154</v>
-      </c>
-      <c r="I170" s="5" t="n">
-        <v>0.1024</v>
-      </c>
-      <c r="J170" s="5" t="n">
-        <v>0.7872</v>
-      </c>
-      <c r="K170" s="5" t="n">
-        <v>0.7872</v>
-      </c>
-      <c r="L170" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8_logreg-bfe9577d-a745ea9e/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d_logreg-bfe9577d-4aefc02f/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B171" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C171" s="4" t="inlineStr">
-        <is>
-          <t>Audio only</t>
-        </is>
-      </c>
-      <c r="D171" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E171" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F171" s="5" t="n">
-        <v>0.4089</v>
-      </c>
-      <c r="G171" s="5" t="n">
-        <v>0.4089</v>
-      </c>
-      <c r="H171" s="5" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="I171" s="5" t="n">
-        <v>0.0038</v>
-      </c>
-      <c r="J171" s="5" t="n">
-        <v>0.8177</v>
-      </c>
-      <c r="K171" s="5" t="n">
-        <v>0.8179</v>
-      </c>
-      <c r="L171" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B172" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C172" s="4" t="inlineStr">
-        <is>
-          <t>Audio only</t>
-        </is>
-      </c>
-      <c r="D172" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E172" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F172" s="5" t="n">
-        <v>0.6097</v>
-      </c>
-      <c r="G172" s="5" t="n">
-        <v>0.6107</v>
-      </c>
-      <c r="H172" s="5" t="n">
-        <v>-0.0011</v>
-      </c>
-      <c r="I172" s="5" t="n">
-        <v>0.1292</v>
-      </c>
-      <c r="J172" s="5" t="n">
-        <v>0.7886</v>
-      </c>
-      <c r="K172" s="5" t="n">
-        <v>0.7865</v>
-      </c>
-      <c r="L172" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f0_216bcec8_xgb_optuna100-bfe9577d-ca2d5d5a/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_only/audio_only/turkish/tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_only_s1337_f1_f57deb8d_xgb_optuna100-bfe9577d-8e66f104/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B173" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C173" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D173" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E173" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F173" s="5" t="n">
-        <v>0.6887</v>
-      </c>
-      <c r="G173" s="5" t="n">
-        <v>0.6913</v>
-      </c>
-      <c r="H173" s="5" t="n">
-        <v>-0.0027</v>
-      </c>
-      <c r="I173" s="5" t="n">
-        <v>0.09569999999999999</v>
-      </c>
-      <c r="J173" s="5" t="n">
-        <v>0.795</v>
-      </c>
-      <c r="K173" s="5" t="n">
-        <v>0.7906</v>
-      </c>
-      <c r="L173" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57_logreg-bfe9577d-f3c53a19/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db_logreg-bfe9577d-a1db4310/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B174" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C174" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D174" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E174" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F174" s="5" t="n">
-        <v>0.7069</v>
-      </c>
-      <c r="G174" s="5" t="n">
-        <v>0.7052</v>
-      </c>
-      <c r="H174" s="5" t="n">
-        <v>0.0017</v>
-      </c>
-      <c r="I174" s="5" t="n">
-        <v>0.1009</v>
-      </c>
-      <c r="J174" s="5" t="n">
-        <v>0.8193</v>
-      </c>
-      <c r="K174" s="5" t="n">
-        <v>0.8133</v>
-      </c>
-      <c r="L174" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820_logreg-bfe9577d-8529f031/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489_logreg-bfe9577d-ec33ced8/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B175" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C175" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D175" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E175" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F175" s="5" t="n">
-        <v>0.7222</v>
-      </c>
-      <c r="G175" s="5" t="n">
-        <v>0.7197</v>
-      </c>
-      <c r="H175" s="5" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="I175" s="5" t="n">
-        <v>0.08890000000000001</v>
-      </c>
-      <c r="J175" s="5" t="n">
-        <v>0.8333</v>
-      </c>
-      <c r="K175" s="5" t="n">
-        <v>0.8288</v>
-      </c>
-      <c r="L175" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B176" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C176" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D176" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E176" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F176" s="5" t="n">
-        <v>0.7024</v>
-      </c>
-      <c r="G176" s="5" t="n">
-        <v>0.6963</v>
-      </c>
-      <c r="H176" s="5" t="n">
-        <v>0.0061</v>
-      </c>
-      <c r="I176" s="5" t="n">
-        <v>0.0764</v>
-      </c>
-      <c r="J176" s="5" t="n">
-        <v>0.8214</v>
-      </c>
-      <c r="K176" s="5" t="n">
-        <v>0.8191000000000001</v>
-      </c>
-      <c r="L176" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B177" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C177" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D177" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E177" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F177" s="5" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G177" s="5" t="n">
-        <v>0.703</v>
-      </c>
-      <c r="H177" s="5" t="n">
-        <v>-0.003</v>
-      </c>
-      <c r="I177" s="5" t="n">
-        <v>0.08160000000000001</v>
-      </c>
-      <c r="J177" s="5" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="K177" s="5" t="n">
-        <v>0.7984</v>
-      </c>
-      <c r="L177" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s1337_f0_216c2b57_xgb_optuna100-bfe9577d-dd9d4826/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_audio_text_s1337_f1_9a5ce3db_xgb_optuna100-bfe9577d-32f966f6/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B178" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C178" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D178" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E178" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F178" s="5" t="n">
-        <v>0.6825</v>
-      </c>
-      <c r="G178" s="5" t="n">
-        <v>0.6848</v>
-      </c>
-      <c r="H178" s="5" t="n">
-        <v>-0.0022</v>
-      </c>
-      <c r="I178" s="5" t="n">
-        <v>0.08309999999999999</v>
-      </c>
-      <c r="J178" s="5" t="n">
-        <v>0.8095</v>
-      </c>
-      <c r="K178" s="5" t="n">
-        <v>0.803</v>
-      </c>
-      <c r="L178" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f0_dd3b8820_xgb_optuna100-bfe9577d-7e5ff6e7/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_audio_text/audio_text/turkish/tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_audio_text_s1337_f1_fdef1489_xgb_optuna100-bfe9577d-d484976c/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B179" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C179" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D179" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E179" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F179" s="5" t="n">
-        <v>0.7188</v>
-      </c>
-      <c r="G179" s="5" t="n">
-        <v>0.7235</v>
-      </c>
-      <c r="H179" s="5" t="n">
-        <v>-0.0048</v>
-      </c>
-      <c r="I179" s="5" t="n">
-        <v>0.1409</v>
-      </c>
-      <c r="J179" s="5" t="n">
-        <v>0.8125</v>
-      </c>
-      <c r="K179" s="5" t="n">
-        <v>0.8090000000000001</v>
-      </c>
-      <c r="L179" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357/fold_0/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357_logreg-bfe9577d-47b66836/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea/fold_1/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea_logreg-bfe9577d-9477a678/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B180" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C180" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D180" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E180" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F180" s="5" t="n">
-        <v>0.6773</v>
-      </c>
-      <c r="G180" s="5" t="n">
-        <v>0.6778</v>
-      </c>
-      <c r="H180" s="5" t="n">
-        <v>-0.0005</v>
-      </c>
-      <c r="I180" s="5" t="n">
-        <v>0.0623</v>
-      </c>
-      <c r="J180" s="5" t="n">
-        <v>0.8118</v>
-      </c>
-      <c r="K180" s="5" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="L180" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850_logreg-bfe9577d-6c33c214/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034_logreg-bfe9577d-9dcc05f3/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B181" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C181" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D181" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E181" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F181" s="5" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="G181" s="5" t="n">
-        <v>0.6877</v>
-      </c>
-      <c r="H181" s="5" t="n">
-        <v>0.0023</v>
-      </c>
-      <c r="I181" s="5" t="n">
-        <v>0.0421</v>
-      </c>
-      <c r="J181" s="5" t="n">
-        <v>0.8166</v>
-      </c>
-      <c r="K181" s="5" t="n">
-        <v>0.8129999999999999</v>
-      </c>
-      <c r="L181" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B182" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C182" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D182" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E182" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F182" s="5" t="n">
-        <v>0.7421</v>
-      </c>
-      <c r="G182" s="5" t="n">
-        <v>0.7403999999999999</v>
-      </c>
-      <c r="H182" s="5" t="n">
-        <v>0.0017</v>
-      </c>
-      <c r="I182" s="5" t="n">
-        <v>0.08740000000000001</v>
-      </c>
-      <c r="J182" s="5" t="n">
-        <v>0.8452</v>
-      </c>
-      <c r="K182" s="5" t="n">
-        <v>0.8464</v>
-      </c>
-      <c r="L182" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B183" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C183" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D183" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E183" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F183" s="5" t="n">
-        <v>0.6791</v>
-      </c>
-      <c r="G183" s="5" t="n">
-        <v>0.6792</v>
-      </c>
-      <c r="H183" s="5" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="I183" s="5" t="n">
-        <v>0.066</v>
-      </c>
-      <c r="J183" s="5" t="n">
-        <v>0.8208</v>
-      </c>
-      <c r="K183" s="5" t="n">
-        <v>0.8217</v>
-      </c>
-      <c r="L183" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f0_7c938850_xgb_optuna100-bfe9577d-ccfc176c/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_audio_text/audio_text/turkish/tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_audio_text_s1337_f1_fcbeb034_xgb_optuna100-bfe9577d-93a65d16/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B184" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C184" s="4" t="inlineStr">
-        <is>
-          <t>Audio + Text</t>
-        </is>
-      </c>
-      <c r="D184" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E184" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F184" s="5" t="n">
-        <v>0.7036</v>
-      </c>
-      <c r="G184" s="5" t="n">
-        <v>0.7088</v>
-      </c>
-      <c r="H184" s="5" t="n">
-        <v>-0.0052</v>
-      </c>
-      <c r="I184" s="5" t="n">
-        <v>0.1274</v>
-      </c>
-      <c r="J184" s="5" t="n">
-        <v>0.8098</v>
-      </c>
-      <c r="K184" s="5" t="n">
-        <v>0.8055</v>
-      </c>
-      <c r="L184" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357/fold_0/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s1337_f0_895b1357_xgb_optuna100-bfe9577d-59c62f9c/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_audio_text/audio_text/turkish/tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea/fold_1/20260903T213549Z-tpq_prod_v1_qwen_english_audio_text_s1337_f1_ec98c7ea_xgb_optuna100-bfe9577d-0c0bb912/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B185" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C185" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D185" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E185" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F185" s="5" t="n">
-        <v>0.5672</v>
-      </c>
-      <c r="G185" s="5" t="n">
-        <v>0.5714</v>
-      </c>
-      <c r="H185" s="5" t="n">
-        <v>-0.0042</v>
-      </c>
-      <c r="I185" s="5" t="n">
-        <v>0.1271</v>
-      </c>
-      <c r="J185" s="5" t="n">
-        <v>0.7006</v>
-      </c>
-      <c r="K185" s="5" t="n">
-        <v>0.6893</v>
-      </c>
-      <c r="L185" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f_logreg-bfe9577d-b7a21ba4/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75_logreg-bfe9577d-07136c2f/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B186" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C186" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D186" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E186" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F186" s="5" t="n">
-        <v>0.6237</v>
-      </c>
-      <c r="G186" s="5" t="n">
-        <v>0.6122</v>
-      </c>
-      <c r="H186" s="5" t="n">
-        <v>0.0115</v>
-      </c>
-      <c r="I186" s="5" t="n">
-        <v>0.0575</v>
-      </c>
-      <c r="J186" s="5" t="n">
-        <v>0.7836</v>
-      </c>
-      <c r="K186" s="5" t="n">
-        <v>0.7774</v>
-      </c>
-      <c r="L186" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d_logreg-bfe9577d-fd85e1d1/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f_logreg-bfe9577d-0453b200/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B187" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C187" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D187" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E187" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F187" s="5" t="n">
-        <v>0.5185999999999999</v>
-      </c>
-      <c r="G187" s="5" t="n">
-        <v>0.4897</v>
-      </c>
-      <c r="H187" s="5" t="n">
-        <v>0.0289</v>
-      </c>
-      <c r="I187" s="5" t="n">
-        <v>0.1008</v>
-      </c>
-      <c r="J187" s="5" t="n">
-        <v>0.6951000000000001</v>
-      </c>
-      <c r="K187" s="5" t="n">
-        <v>0.6821</v>
-      </c>
-      <c r="L187" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B188" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C188" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D188" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E188" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F188" s="5" t="n">
-        <v>0.5036</v>
-      </c>
-      <c r="G188" s="5" t="n">
-        <v>0.4556</v>
-      </c>
-      <c r="H188" s="5" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="I188" s="5" t="n">
-        <v>0.07240000000000001</v>
-      </c>
-      <c r="J188" s="5" t="n">
-        <v>0.7806999999999999</v>
-      </c>
-      <c r="K188" s="5" t="n">
-        <v>0.7726</v>
-      </c>
-      <c r="L188" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B189" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C189" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D189" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E189" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F189" s="5" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="G189" s="5" t="n">
-        <v>0.6494</v>
-      </c>
-      <c r="H189" s="5" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="I189" s="5" t="n">
-        <v>0.1533</v>
-      </c>
-      <c r="J189" s="5" t="n">
-        <v>0.7929</v>
-      </c>
-      <c r="K189" s="5" t="n">
-        <v>0.7911</v>
-      </c>
-      <c r="L189" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s1337_f0_0a150a4f_xgb_optuna100-bfe9577d-9b93d865/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_native_text_only/text_only/turkish/tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_native_text_only_s1337_f1_d1967d75_xgb_optuna100-bfe9577d-dc27af92/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B190" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C190" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D190" s="4" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="E190" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F190" s="5" t="n">
-        <v>0.6149</v>
-      </c>
-      <c r="G190" s="5" t="n">
-        <v>0.6143999999999999</v>
-      </c>
-      <c r="H190" s="5" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="I190" s="5" t="n">
-        <v>0.0613</v>
-      </c>
-      <c r="J190" s="5" t="n">
-        <v>0.7561</v>
-      </c>
-      <c r="K190" s="5" t="n">
-        <v>0.7523</v>
-      </c>
-      <c r="L190" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d/fold_0/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s1337_f0_5c5e083d_xgb_optuna100-bfe9577d-4729fcf4/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_gemma4_english_text_only/text_only/turkish/tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f/fold_1/20260903T213549Z-tpq_prod_v1_gemma4_english_text_only_s1337_f1_b871cb4f_xgb_optuna100-bfe9577d-f16d5f67/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B191" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C191" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D191" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E191" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F191" s="5" t="n">
-        <v>0.5663</v>
-      </c>
-      <c r="G191" s="5" t="n">
-        <v>0.5605</v>
-      </c>
-      <c r="H191" s="5" t="n">
-        <v>0.0059</v>
-      </c>
-      <c r="I191" s="5" t="n">
-        <v>0.0781</v>
-      </c>
-      <c r="J191" s="5" t="n">
-        <v>0.6711</v>
-      </c>
-      <c r="K191" s="5" t="n">
-        <v>0.6559</v>
-      </c>
-      <c r="L191" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f0_49e543a1/fold_0/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s1337_f0_49e543a1_logreg-bfe9577d-8abf5ac5/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f1_7a0529bf/fold_1/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s1337_f1_7a0529bf_logreg-bfe9577d-96105eb5/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B192" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C192" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D192" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E192" s="4" t="inlineStr">
-        <is>
-          <t>LogReg</t>
-        </is>
-      </c>
-      <c r="F192" s="5" t="n">
-        <v>0.616</v>
-      </c>
-      <c r="G192" s="5" t="n">
-        <v>0.6127</v>
-      </c>
-      <c r="H192" s="5" t="n">
-        <v>0.0033</v>
-      </c>
-      <c r="I192" s="5" t="n">
-        <v>0.098</v>
-      </c>
-      <c r="J192" s="5" t="n">
-        <v>0.7151999999999999</v>
-      </c>
-      <c r="K192" s="5" t="n">
-        <v>0.7131999999999999</v>
-      </c>
-      <c r="L192" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30_logreg-bfe9577d-b7d028e5/classifier/logreg_raw/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd_logreg-bfe9577d-1d78c089/classifier/logreg_raw/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B193" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C193" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D193" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E193" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F193" s="5" t="n">
-        <v>0.4667</v>
-      </c>
-      <c r="G193" s="5" t="n">
-        <v>0.4379</v>
-      </c>
-      <c r="H193" s="5" t="n">
-        <v>0.0288</v>
-      </c>
-      <c r="I193" s="5" t="n">
-        <v>0.0586</v>
-      </c>
-      <c r="J193" s="5" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="K193" s="5" t="n">
-        <v>0.7957</v>
-      </c>
-      <c r="L193" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f0_49e543a1/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f1_7a0529bf/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B194" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C194" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D194" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E194" s="4" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="F194" s="5" t="n">
-        <v>0.4504</v>
-      </c>
-      <c r="G194" s="5" t="n">
-        <v>0.4174</v>
-      </c>
-      <c r="H194" s="5" t="n">
-        <v>0.0331</v>
-      </c>
-      <c r="I194" s="5" t="n">
-        <v>0.0179</v>
-      </c>
-      <c r="J194" s="5" t="n">
-        <v>0.7527</v>
-      </c>
-      <c r="K194" s="5" t="n">
-        <v>0.7373</v>
-      </c>
-      <c r="L194" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30/fold_0/best_model/standalone_eval/metrics_original_teacher_forced.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd/fold_1/best_model/standalone_eval/metrics_original_teacher_forced.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B195" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C195" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D195" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E195" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F195" s="5" t="n">
-        <v>0.6804</v>
-      </c>
-      <c r="G195" s="5" t="n">
-        <v>0.6687</v>
-      </c>
-      <c r="H195" s="5" t="n">
-        <v>0.0117</v>
-      </c>
-      <c r="I195" s="5" t="n">
-        <v>0.09470000000000001</v>
-      </c>
-      <c r="J195" s="5" t="n">
-        <v>0.8295</v>
-      </c>
-      <c r="K195" s="5" t="n">
-        <v>0.8268</v>
-      </c>
-      <c r="L195" s="5" t="inlineStr">
-        <is>
-          <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30/fold_0/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s1337_f0_0e113f30_xgb_optuna100-bfe9577d-28adfca1/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_native_text_only/text_only/turkish/tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd/fold_1/20260903T213549Z-tpq_prod_v1_qwen_native_text_only_s1337_f1_22dd2ccd_xgb_optuna100-bfe9577d-667cf4ba/xgb_optuna100_harmonized_v1/metrics.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="4" t="inlineStr">
-        <is>
-          <t>turkish_pooled</t>
-        </is>
-      </c>
-      <c r="B196" s="4" t="inlineStr">
-        <is>
-          <t>Turkish</t>
-        </is>
-      </c>
-      <c r="C196" s="4" t="inlineStr">
-        <is>
-          <t>Text only</t>
-        </is>
-      </c>
-      <c r="D196" s="4" t="inlineStr">
-        <is>
-          <t>qwen</t>
-        </is>
-      </c>
-      <c r="E196" s="4" t="inlineStr">
-        <is>
-          <t>XGB optuna-100</t>
-        </is>
-      </c>
-      <c r="F196" s="5" t="n">
-        <v>0.637</v>
-      </c>
-      <c r="G196" s="5" t="n">
-        <v>0.6306</v>
-      </c>
-      <c r="H196" s="5" t="n">
-        <v>0.0063</v>
-      </c>
-      <c r="I196" s="5" t="n">
-        <v>0.0293</v>
-      </c>
-      <c r="J196" s="5" t="n">
-        <v>0.7882</v>
-      </c>
-      <c r="K196" s="5" t="n">
-        <v>0.7843</v>
-      </c>
-      <c r="L196" s="5" t="inlineStr">
         <is>
           <t>/home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f0_49e543a1/fold_0/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s1337_f0_49e543a1_xgb_optuna100-bfe9577d-4de3f596/xgb_optuna100_harmonized_v1/metrics.json; /home/emre/worktrees/LLM-Depression-exp-turkish-pooled-qcond-clean-v1/output_model/turkish_pooled_qcond_clean_v1_qwen_english_text_only/text_only/turkish/tpq_prod_v1_qwen_english_text_only_s1337_f1_7a0529bf/fold_1/20260903T213549Z-tpq_prod_v1_qwen_english_text_only_s1337_f1_7a0529bf_xgb_optuna100-bfe9577d-b5c41eb8/xgb_optuna100_harmonized_v1/metrics.json</t>
         </is>

</xml_diff>

<commit_message>
Align Provenance rows with pooled headline cells
The pooled override refreshed the headline lookups but several
Provenance groups still read pre-pooled sources: EN Translation CMDC
(HARMONIZED_EN_QWEN), EN/native heads (HARMONIZED_EN_HEADS), Gemma
native and Optuna100 native/english/merged rows kept legacy fold-mean
values and '5-fold mean'/'fold-mean' aggregation labels. Refresh those
lookups and labels from the pooled audit; legacy fixed-XGB heads stay
labelled as such.
</commit_message>
<xml_diff>
--- a/depression_results_clean.xlsx
+++ b/depression_results_clean.xlsx
@@ -28771,7 +28771,7 @@
         </is>
       </c>
       <c r="E19" s="15" t="n">
-        <v>0.5465</v>
+        <v>0.546499</v>
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
@@ -28816,7 +28816,7 @@
         </is>
       </c>
       <c r="E20" s="15" t="n">
-        <v>0.5758</v>
+        <v>0.575758</v>
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
@@ -28861,7 +28861,7 @@
         </is>
       </c>
       <c r="E21" s="15" t="n">
-        <v>0.8873</v>
+        <v>0.887252</v>
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
@@ -29041,7 +29041,7 @@
         </is>
       </c>
       <c r="E25" s="15" t="n">
-        <v>0.7921</v>
+        <v>0.792115</v>
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
@@ -29086,7 +29086,7 @@
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>0.8065</v>
+        <v>0.8064519999999999</v>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="E27" s="15" t="n">
-        <v>0.9856</v>
+        <v>0.985712</v>
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
@@ -29140,7 +29140,7 @@
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H27" s="16" t="inlineStr">
@@ -29176,7 +29176,7 @@
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>0.9818</v>
+        <v>0.981132</v>
       </c>
       <c r="F28" s="16" t="inlineStr">
         <is>
@@ -29185,7 +29185,7 @@
       </c>
       <c r="G28" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H28" s="16" t="inlineStr">
@@ -29230,7 +29230,7 @@
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H29" s="16" t="inlineStr">
@@ -29275,7 +29275,7 @@
       </c>
       <c r="G30" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H30" s="16" t="inlineStr">
@@ -29311,7 +29311,7 @@
         </is>
       </c>
       <c r="E31" s="15" t="n">
-        <v>0.9713000000000001</v>
+        <v>0.971678</v>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
@@ -29320,7 +29320,7 @@
       </c>
       <c r="G31" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H31" s="16" t="inlineStr">
@@ -29356,7 +29356,7 @@
         </is>
       </c>
       <c r="E32" s="15" t="n">
-        <v>0.9636</v>
+        <v>0.962963</v>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
@@ -29365,7 +29365,7 @@
       </c>
       <c r="G32" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H32" s="16" t="inlineStr">
@@ -29401,7 +29401,7 @@
         </is>
       </c>
       <c r="E33" s="15" t="n">
-        <v>0.5464</v>
+        <v>0.555142</v>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
@@ -29410,7 +29410,7 @@
       </c>
       <c r="G33" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H33" s="16" t="inlineStr">
@@ -29455,7 +29455,7 @@
       </c>
       <c r="G34" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H34" s="16" t="inlineStr">
@@ -29500,7 +29500,7 @@
       </c>
       <c r="G35" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H35" s="16" t="inlineStr">
@@ -29545,7 +29545,7 @@
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H36" s="16" t="inlineStr">
@@ -29581,7 +29581,7 @@
         </is>
       </c>
       <c r="E37" s="15" t="n">
-        <v>0.5226</v>
+        <v>0.5321360000000001</v>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
@@ -29590,7 +29590,7 @@
       </c>
       <c r="G37" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H37" s="16" t="inlineStr">
@@ -29635,7 +29635,7 @@
       </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H38" s="16" t="inlineStr">
@@ -29671,7 +29671,7 @@
         </is>
       </c>
       <c r="E39" s="15" t="n">
-        <v>0.8802</v>
+        <v>0.886914</v>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
@@ -29680,7 +29680,7 @@
       </c>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H39" s="16" t="inlineStr">
@@ -29725,7 +29725,7 @@
       </c>
       <c r="G40" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H40" s="16" t="inlineStr">
@@ -29770,7 +29770,7 @@
       </c>
       <c r="G41" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H41" s="16" t="inlineStr">
@@ -29815,7 +29815,7 @@
       </c>
       <c r="G42" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H42" s="16" t="inlineStr">
@@ -29851,7 +29851,7 @@
         </is>
       </c>
       <c r="E43" s="15" t="n">
-        <v>0.8298</v>
+        <v>0.835608</v>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
@@ -29860,7 +29860,7 @@
       </c>
       <c r="G43" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H43" s="16" t="inlineStr">
@@ -29905,7 +29905,7 @@
       </c>
       <c r="G44" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H44" s="16" t="inlineStr">
@@ -29941,7 +29941,7 @@
         </is>
       </c>
       <c r="E45" s="15" t="n">
-        <v>0.9856</v>
+        <v>0.985712</v>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
@@ -29950,7 +29950,7 @@
       </c>
       <c r="G45" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H45" s="16" t="inlineStr">
@@ -29995,7 +29995,7 @@
       </c>
       <c r="G46" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H46" s="16" t="inlineStr">
@@ -30040,7 +30040,7 @@
       </c>
       <c r="G47" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H47" s="16" t="inlineStr">
@@ -30085,7 +30085,7 @@
       </c>
       <c r="G48" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H48" s="16" t="inlineStr">
@@ -30121,7 +30121,7 @@
         </is>
       </c>
       <c r="E49" s="15" t="n">
-        <v>0.9698</v>
+        <v>0.971154</v>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
@@ -30130,7 +30130,7 @@
       </c>
       <c r="G49" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H49" s="16" t="inlineStr">
@@ -30175,7 +30175,7 @@
       </c>
       <c r="G50" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H50" s="16" t="inlineStr">
@@ -30211,7 +30211,7 @@
         </is>
       </c>
       <c r="E51" s="15" t="n">
-        <v>0.4988</v>
+        <v>0.52219</v>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
@@ -30220,7 +30220,7 @@
       </c>
       <c r="G51" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H51" s="16" t="inlineStr">
@@ -30265,7 +30265,7 @@
       </c>
       <c r="G52" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H52" s="16" t="inlineStr">
@@ -30301,7 +30301,7 @@
         </is>
       </c>
       <c r="E53" s="15" t="n">
-        <v>0.6031</v>
+        <v>0.621047</v>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
@@ -30310,7 +30310,7 @@
       </c>
       <c r="G53" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H53" s="16" t="inlineStr">
@@ -30355,7 +30355,7 @@
       </c>
       <c r="G54" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H54" s="16" t="inlineStr">
@@ -30391,7 +30391,7 @@
         </is>
       </c>
       <c r="E55" s="15" t="n">
-        <v>0.4651</v>
+        <v>0.483871</v>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
@@ -30400,7 +30400,7 @@
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H55" s="16" t="inlineStr">
@@ -30445,7 +30445,7 @@
       </c>
       <c r="G56" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H56" s="16" t="inlineStr">
@@ -30481,7 +30481,7 @@
         </is>
       </c>
       <c r="E57" s="15" t="n">
-        <v>0.8745000000000001</v>
+        <v>0.878734</v>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
@@ -30490,7 +30490,7 @@
       </c>
       <c r="G57" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H57" s="16" t="inlineStr">
@@ -30535,7 +30535,7 @@
       </c>
       <c r="G58" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H58" s="16" t="inlineStr">
@@ -30571,7 +30571,7 @@
         </is>
       </c>
       <c r="E59" s="15" t="n">
-        <v>0.8512</v>
+        <v>0.86141</v>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
@@ -30580,7 +30580,7 @@
       </c>
       <c r="G59" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H59" s="16" t="inlineStr">
@@ -30625,7 +30625,7 @@
       </c>
       <c r="G60" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H60" s="16" t="inlineStr">
@@ -30661,7 +30661,7 @@
         </is>
       </c>
       <c r="E61" s="15" t="n">
-        <v>0.8326</v>
+        <v>0.844086</v>
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
@@ -30670,7 +30670,7 @@
       </c>
       <c r="G61" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H61" s="16" t="inlineStr">
@@ -30715,7 +30715,7 @@
       </c>
       <c r="G62" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H62" s="16" t="inlineStr">
@@ -30751,7 +30751,7 @@
         </is>
       </c>
       <c r="E63" s="15" t="n">
-        <v>0.9614</v>
+        <v>0.9578759999999999</v>
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
@@ -30760,7 +30760,7 @@
       </c>
       <c r="G63" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H63" s="16" t="inlineStr">
@@ -30805,7 +30805,7 @@
       </c>
       <c r="G64" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H64" s="16" t="inlineStr">
@@ -30841,7 +30841,7 @@
         </is>
       </c>
       <c r="E65" s="15" t="n">
-        <v>0.9841</v>
+        <v>0.985434</v>
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
@@ -30850,7 +30850,7 @@
       </c>
       <c r="G65" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H65" s="16" t="inlineStr">
@@ -30895,7 +30895,7 @@
       </c>
       <c r="G66" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H66" s="16" t="inlineStr">
@@ -30931,7 +30931,7 @@
         </is>
       </c>
       <c r="E67" s="15" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9433550000000001</v>
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
@@ -30940,7 +30940,7 @@
       </c>
       <c r="G67" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H67" s="16" t="inlineStr">
@@ -30985,7 +30985,7 @@
       </c>
       <c r="G68" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean, subject-level macro-F1 (STANDALONE_HEADS convention)</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H68" s="16" t="inlineStr">
@@ -31030,7 +31030,7 @@
       </c>
       <c r="G69" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H69" s="16" t="inlineStr">
@@ -31075,7 +31075,7 @@
       </c>
       <c r="G70" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H70" s="16" t="inlineStr">
@@ -31120,7 +31120,7 @@
       </c>
       <c r="G71" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H71" s="16" t="inlineStr">
@@ -31165,7 +31165,7 @@
       </c>
       <c r="G72" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H72" s="16" t="inlineStr">
@@ -31210,7 +31210,7 @@
       </c>
       <c r="G73" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H73" s="16" t="inlineStr">
@@ -31255,7 +31255,7 @@
       </c>
       <c r="G74" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H74" s="16" t="inlineStr">
@@ -31300,7 +31300,7 @@
       </c>
       <c r="G75" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H75" s="16" t="inlineStr">
@@ -31345,7 +31345,7 @@
       </c>
       <c r="G76" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H76" s="16" t="inlineStr">
@@ -31390,7 +31390,7 @@
       </c>
       <c r="G77" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H77" s="16" t="inlineStr">
@@ -31435,7 +31435,7 @@
       </c>
       <c r="G78" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H78" s="16" t="inlineStr">
@@ -31480,7 +31480,7 @@
       </c>
       <c r="G79" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H79" s="16" t="inlineStr">
@@ -31525,7 +31525,7 @@
       </c>
       <c r="G80" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H80" s="16" t="inlineStr">
@@ -31570,7 +31570,7 @@
       </c>
       <c r="G81" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H81" s="16" t="inlineStr">
@@ -31615,7 +31615,7 @@
       </c>
       <c r="G82" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H82" s="16" t="inlineStr">
@@ -31660,7 +31660,7 @@
       </c>
       <c r="G83" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H83" s="16" t="inlineStr">
@@ -31705,7 +31705,7 @@
       </c>
       <c r="G84" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H84" s="16" t="inlineStr">
@@ -31750,7 +31750,7 @@
       </c>
       <c r="G85" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H85" s="16" t="inlineStr">
@@ -31795,7 +31795,7 @@
       </c>
       <c r="G86" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H86" s="16" t="inlineStr">
@@ -31840,7 +31840,7 @@
       </c>
       <c r="G87" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H87" s="16" t="inlineStr">
@@ -31885,7 +31885,7 @@
       </c>
       <c r="G88" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H88" s="16" t="inlineStr">
@@ -31930,7 +31930,7 @@
       </c>
       <c r="G89" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H89" s="16" t="inlineStr">
@@ -31975,7 +31975,7 @@
       </c>
       <c r="G90" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H90" s="16" t="inlineStr">
@@ -32020,7 +32020,7 @@
       </c>
       <c r="G91" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>seed-1337 pooled subject-level, macro-F1 (INVALID counts as wrong)</t>
         </is>
       </c>
       <c r="H91" s="16" t="inlineStr">
@@ -32065,7 +32065,7 @@
       </c>
       <c r="G92" s="16" t="inlineStr">
         <is>
-          <t>pooled subject-level, 5-fold</t>
+          <t>fixed XGB head, 5-fold mean, subject-level macro-F1 (legacy)</t>
         </is>
       </c>
       <c r="H92" s="16" t="inlineStr">
@@ -37393,7 +37393,7 @@
       </c>
       <c r="G210" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H210" s="16" t="inlineStr">
@@ -37438,7 +37438,7 @@
       </c>
       <c r="G211" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H211" s="16" t="inlineStr">
@@ -37483,7 +37483,7 @@
       </c>
       <c r="G212" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
+          <t>seed-1337 pooled subject-level, 100 Optuna trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
         </is>
       </c>
       <c r="H212" s="16" t="inlineStr">
@@ -37528,7 +37528,7 @@
       </c>
       <c r="G213" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H213" s="16" t="inlineStr">
@@ -37573,7 +37573,7 @@
       </c>
       <c r="G214" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H214" s="16" t="inlineStr">
@@ -37618,7 +37618,7 @@
       </c>
       <c r="G215" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
+          <t>seed-1337 pooled subject-level, 100 Optuna trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
         </is>
       </c>
       <c r="H215" s="16" t="inlineStr">
@@ -37663,7 +37663,7 @@
       </c>
       <c r="G216" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H216" s="16" t="inlineStr">
@@ -37708,7 +37708,7 @@
       </c>
       <c r="G217" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H217" s="16" t="inlineStr">
@@ -37753,7 +37753,7 @@
       </c>
       <c r="G218" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
+          <t>seed-1337 pooled subject-level, 100 Optuna trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
         </is>
       </c>
       <c r="H218" s="16" t="inlineStr">
@@ -37798,7 +37798,7 @@
       </c>
       <c r="G219" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H219" s="16" t="inlineStr">
@@ -37843,7 +37843,7 @@
       </c>
       <c r="G220" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H220" s="16" t="inlineStr">
@@ -37888,7 +37888,7 @@
       </c>
       <c r="G221" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
+          <t>seed-1337 pooled subject-level, 100 Optuna trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
         </is>
       </c>
       <c r="H221" s="16" t="inlineStr">
@@ -37933,7 +37933,7 @@
       </c>
       <c r="G222" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H222" s="16" t="inlineStr">
@@ -37978,7 +37978,7 @@
       </c>
       <c r="G223" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H223" s="16" t="inlineStr">
@@ -38023,7 +38023,7 @@
       </c>
       <c r="G224" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
+          <t>seed-1337 pooled subject-level, 100 Optuna trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
         </is>
       </c>
       <c r="H224" s="16" t="inlineStr">
@@ -38068,7 +38068,7 @@
       </c>
       <c r="G225" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H225" s="16" t="inlineStr">
@@ -38113,7 +38113,7 @@
       </c>
       <c r="G226" s="16" t="inlineStr">
         <is>
-          <t>pooled 5-fold subject-level, LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H226" s="16" t="inlineStr">
@@ -38158,7 +38158,7 @@
       </c>
       <c r="G227" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
+          <t>seed-1337 pooled subject-level, 100 Optuna trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
         </is>
       </c>
       <c r="H227" s="16" t="inlineStr">
@@ -38203,7 +38203,7 @@
       </c>
       <c r="G228" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean (train_val protocol), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H228" s="16" t="inlineStr">
@@ -38248,7 +38248,7 @@
       </c>
       <c r="G229" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean (train_val protocol), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H229" s="16" t="inlineStr">
@@ -38293,7 +38293,7 @@
       </c>
       <c r="G230" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
+          <t>seed-1337 pooled subject-level, 100 Optuna trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
         </is>
       </c>
       <c r="H230" s="16" t="inlineStr">
@@ -38338,7 +38338,7 @@
       </c>
       <c r="G231" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean (train_val protocol), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H231" s="16" t="inlineStr">
@@ -38383,7 +38383,7 @@
       </c>
       <c r="G232" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean (train_val protocol), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H232" s="16" t="inlineStr">
@@ -38428,7 +38428,7 @@
       </c>
       <c r="G233" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
+          <t>seed-1337 pooled subject-level, 100 Optuna trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
         </is>
       </c>
       <c r="H233" s="16" t="inlineStr">
@@ -38473,7 +38473,7 @@
       </c>
       <c r="G234" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean (train_val protocol), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), teacher-forced, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H234" s="16" t="inlineStr">
@@ -38518,7 +38518,7 @@
       </c>
       <c r="G235" s="16" t="inlineStr">
         <is>
-          <t>5-fold mean (train_val protocol), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
+          <t>seed-1337 pooled subject-level (5-fold subjects in one pool, single F1; INVALID counts as wrong), LogReg raw hidden head, binary-strict, harmonized_all_windows_full_coverage</t>
         </is>
       </c>
       <c r="H235" s="16" t="inlineStr">
@@ -38563,7 +38563,7 @@
       </c>
       <c r="G236" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
+          <t>seed-1337 pooled subject-level, 100 Optuna trials seed 1337, 3 inner folds, subject-level macro-F1 objective</t>
         </is>
       </c>
       <c r="H236" s="16" t="inlineStr">
@@ -38599,7 +38599,7 @@
         </is>
       </c>
       <c r="E237" s="15" t="n">
-        <v>0.5233976549766023</v>
+        <v>0.558893</v>
       </c>
       <c r="F237" s="16" t="inlineStr">
         <is>
@@ -38608,7 +38608,7 @@
       </c>
       <c r="G237" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H237" s="16" t="inlineStr">
@@ -38644,7 +38644,7 @@
         </is>
       </c>
       <c r="E238" s="15" t="n">
-        <v>0.5832267732267733</v>
+        <v>0.595828</v>
       </c>
       <c r="F238" s="16" t="inlineStr">
         <is>
@@ -38653,7 +38653,7 @@
       </c>
       <c r="G238" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H238" s="16" t="inlineStr">
@@ -38689,7 +38689,7 @@
         </is>
       </c>
       <c r="E239" s="15" t="n">
-        <v>0.5194749694749694</v>
+        <v>0.561665</v>
       </c>
       <c r="F239" s="16" t="inlineStr">
         <is>
@@ -38698,7 +38698,7 @@
       </c>
       <c r="G239" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H239" s="16" t="inlineStr">
@@ -38734,7 +38734,7 @@
         </is>
       </c>
       <c r="E240" s="15" t="n">
-        <v>0.546075036075036</v>
+        <v>0.558893</v>
       </c>
       <c r="F240" s="16" t="inlineStr">
         <is>
@@ -38743,7 +38743,7 @@
       </c>
       <c r="G240" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H240" s="16" t="inlineStr">
@@ -38779,7 +38779,7 @@
         </is>
       </c>
       <c r="E241" s="15" t="n">
-        <v>0.634534632034632</v>
+        <v>0.644792</v>
       </c>
       <c r="F241" s="16" t="inlineStr">
         <is>
@@ -38788,7 +38788,7 @@
       </c>
       <c r="G241" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H241" s="16" t="inlineStr">
@@ -38824,7 +38824,7 @@
         </is>
       </c>
       <c r="E242" s="15" t="n">
-        <v>0.5719417862838915</v>
+        <v>0.611285</v>
       </c>
       <c r="F242" s="16" t="inlineStr">
         <is>
@@ -38833,7 +38833,7 @@
       </c>
       <c r="G242" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H242" s="16" t="inlineStr">
@@ -38869,7 +38869,7 @@
         </is>
       </c>
       <c r="E243" s="15" t="n">
-        <v>0.8543052605446494</v>
+        <v>0.861699</v>
       </c>
       <c r="F243" s="16" t="inlineStr">
         <is>
@@ -38878,7 +38878,7 @@
       </c>
       <c r="G243" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H243" s="16" t="inlineStr">
@@ -38914,7 +38914,7 @@
         </is>
       </c>
       <c r="E244" s="15" t="n">
-        <v>0.8565473598042608</v>
+        <v>0.861699</v>
       </c>
       <c r="F244" s="16" t="inlineStr">
         <is>
@@ -38923,7 +38923,7 @@
       </c>
       <c r="G244" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H244" s="16" t="inlineStr">
@@ -38959,7 +38959,7 @@
         </is>
       </c>
       <c r="E245" s="15" t="n">
-        <v>0.8109429700734049</v>
+        <v>0.825038</v>
       </c>
       <c r="F245" s="16" t="inlineStr">
         <is>
@@ -38968,7 +38968,7 @@
       </c>
       <c r="G245" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H245" s="16" t="inlineStr">
@@ -39004,7 +39004,7 @@
         </is>
       </c>
       <c r="E246" s="15" t="n">
-        <v>0.8020237849525775</v>
+        <v>0.817323</v>
       </c>
       <c r="F246" s="16" t="inlineStr">
         <is>
@@ -39013,7 +39013,7 @@
       </c>
       <c r="G246" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H246" s="16" t="inlineStr">
@@ -39049,7 +39049,7 @@
         </is>
       </c>
       <c r="E247" s="15" t="n">
-        <v>0.8465966593792681</v>
+        <v>0.861036</v>
       </c>
       <c r="F247" s="16" t="inlineStr">
         <is>
@@ -39058,7 +39058,7 @@
       </c>
       <c r="G247" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H247" s="16" t="inlineStr">
@@ -39094,7 +39094,7 @@
         </is>
       </c>
       <c r="E248" s="15" t="n">
-        <v>0.7481770520323419</v>
+        <v>0.75601</v>
       </c>
       <c r="F248" s="16" t="inlineStr">
         <is>
@@ -39103,7 +39103,7 @@
       </c>
       <c r="G248" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H248" s="16" t="inlineStr">
@@ -39139,7 +39139,7 @@
         </is>
       </c>
       <c r="E249" s="15" t="n">
-        <v>0.9250894033502728</v>
+        <v>0.927171</v>
       </c>
       <c r="F249" s="16" t="inlineStr">
         <is>
@@ -39148,7 +39148,7 @@
       </c>
       <c r="G249" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H249" s="16" t="inlineStr">
@@ -39184,7 +39184,7 @@
         </is>
       </c>
       <c r="E250" s="15" t="n">
-        <v>0.9841269841269842</v>
+        <v>0.985434</v>
       </c>
       <c r="F250" s="16" t="inlineStr">
         <is>
@@ -39193,7 +39193,7 @@
       </c>
       <c r="G250" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H250" s="16" t="inlineStr">
@@ -39229,7 +39229,7 @@
         </is>
       </c>
       <c r="E251" s="15" t="n">
-        <v>0.951555023923445</v>
+        <v>0.956303</v>
       </c>
       <c r="F251" s="16" t="inlineStr">
         <is>
@@ -39238,7 +39238,7 @@
       </c>
       <c r="G251" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H251" s="16" t="inlineStr">
@@ -39274,7 +39274,7 @@
         </is>
       </c>
       <c r="E252" s="15" t="n">
-        <v>0.9583694083694084</v>
+        <v>0.956303</v>
       </c>
       <c r="F252" s="16" t="inlineStr">
         <is>
@@ -39283,7 +39283,7 @@
       </c>
       <c r="G252" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H252" s="16" t="inlineStr">
@@ -39319,7 +39319,7 @@
         </is>
       </c>
       <c r="E253" s="15" t="n">
-        <v>0.9538999012683224</v>
+        <v>0.956303</v>
       </c>
       <c r="F253" s="16" t="inlineStr">
         <is>
@@ -39328,7 +39328,7 @@
       </c>
       <c r="G253" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H253" s="16" t="inlineStr">
@@ -39364,7 +39364,7 @@
         </is>
       </c>
       <c r="E254" s="15" t="n">
-        <v>0.9245881502174408</v>
+        <v>0.927171</v>
       </c>
       <c r="F254" s="16" t="inlineStr">
         <is>
@@ -39373,7 +39373,7 @@
       </c>
       <c r="G254" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H254" s="16" t="inlineStr">
@@ -39409,7 +39409,7 @@
         </is>
       </c>
       <c r="E255" s="15" t="n">
-        <v>0.715725806451613</v>
+        <v>0.715726</v>
       </c>
       <c r="F255" s="16" t="inlineStr">
         <is>
@@ -39418,7 +39418,7 @@
       </c>
       <c r="G255" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H255" s="16" t="inlineStr">
@@ -39454,7 +39454,7 @@
         </is>
       </c>
       <c r="E256" s="15" t="n">
-        <v>0.8156862745098039</v>
+        <v>0.815686</v>
       </c>
       <c r="F256" s="16" t="inlineStr">
         <is>
@@ -39463,7 +39463,7 @@
       </c>
       <c r="G256" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H256" s="16" t="inlineStr">
@@ -39499,7 +39499,7 @@
         </is>
       </c>
       <c r="E257" s="15" t="n">
-        <v>0.5761273209549072</v>
+        <v>0.5761269999999999</v>
       </c>
       <c r="F257" s="16" t="inlineStr">
         <is>
@@ -39508,7 +39508,7 @@
       </c>
       <c r="G257" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H257" s="16" t="inlineStr">
@@ -39544,7 +39544,7 @@
         </is>
       </c>
       <c r="E258" s="15" t="n">
-        <v>0.7257294429708223</v>
+        <v>0.725729</v>
       </c>
       <c r="F258" s="16" t="inlineStr">
         <is>
@@ -39553,7 +39553,7 @@
       </c>
       <c r="G258" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H258" s="16" t="inlineStr">
@@ -39589,7 +39589,7 @@
         </is>
       </c>
       <c r="E259" s="15" t="n">
-        <v>0.7257294429708223</v>
+        <v>0.725729</v>
       </c>
       <c r="F259" s="16" t="inlineStr">
         <is>
@@ -39598,7 +39598,7 @@
       </c>
       <c r="G259" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H259" s="16" t="inlineStr">
@@ -39634,7 +39634,7 @@
         </is>
       </c>
       <c r="E260" s="15" t="n">
-        <v>0.7696078431372548</v>
+        <v>0.769608</v>
       </c>
       <c r="F260" s="16" t="inlineStr">
         <is>
@@ -39643,7 +39643,7 @@
       </c>
       <c r="G260" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H260" s="16" t="inlineStr">
@@ -39679,7 +39679,7 @@
         </is>
       </c>
       <c r="E261" s="15" t="n">
-        <v>0.598161968750204</v>
+        <v>0.609244</v>
       </c>
       <c r="F261" s="16" t="inlineStr">
         <is>
@@ -39688,7 +39688,7 @@
       </c>
       <c r="G261" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H261" s="16" t="inlineStr">
@@ -39724,7 +39724,7 @@
         </is>
       </c>
       <c r="E262" s="15" t="n">
-        <v>0.5467279942279942</v>
+        <v>0.5802079999999999</v>
       </c>
       <c r="F262" s="16" t="inlineStr">
         <is>
@@ -39733,7 +39733,7 @@
       </c>
       <c r="G262" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H262" s="16" t="inlineStr">
@@ -39769,7 +39769,7 @@
         </is>
       </c>
       <c r="E263" s="15" t="n">
-        <v>0.5289319014319014</v>
+        <v>0.540741</v>
       </c>
       <c r="F263" s="16" t="inlineStr">
         <is>
@@ -39778,7 +39778,7 @@
       </c>
       <c r="G263" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H263" s="16" t="inlineStr">
@@ -39814,7 +39814,7 @@
         </is>
       </c>
       <c r="E264" s="15" t="n">
-        <v>0.5599448942869996</v>
+        <v>0.583669</v>
       </c>
       <c r="F264" s="16" t="inlineStr">
         <is>
@@ -39823,7 +39823,7 @@
       </c>
       <c r="G264" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H264" s="16" t="inlineStr">
@@ -39859,7 +39859,7 @@
         </is>
       </c>
       <c r="E265" s="15" t="n">
-        <v>0.8727292418997225</v>
+        <v>0.878734</v>
       </c>
       <c r="F265" s="16" t="inlineStr">
         <is>
@@ -39868,7 +39868,7 @@
       </c>
       <c r="G265" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H265" s="16" t="inlineStr">
@@ -39904,7 +39904,7 @@
         </is>
       </c>
       <c r="E266" s="15" t="n">
-        <v>0.9027865444158352</v>
+        <v>0.913381</v>
       </c>
       <c r="F266" s="16" t="inlineStr">
         <is>
@@ -39913,7 +39913,7 @@
       </c>
       <c r="G266" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H266" s="16" t="inlineStr">
@@ -39949,7 +39949,7 @@
         </is>
       </c>
       <c r="E267" s="15" t="n">
-        <v>0.8111428571428572</v>
+        <v>0.817869</v>
       </c>
       <c r="F267" s="16" t="inlineStr">
         <is>
@@ -39958,7 +39958,7 @@
       </c>
       <c r="G267" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H267" s="16" t="inlineStr">
@@ -39994,7 +39994,7 @@
         </is>
       </c>
       <c r="E268" s="15" t="n">
-        <v>0.808360039884658</v>
+        <v>0.817869</v>
       </c>
       <c r="F268" s="16" t="inlineStr">
         <is>
@@ -40003,7 +40003,7 @@
       </c>
       <c r="G268" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H268" s="16" t="inlineStr">
@@ -40039,7 +40039,7 @@
         </is>
       </c>
       <c r="E269" s="15" t="n">
-        <v>0.9133968253968254</v>
+        <v>0.9238730000000001</v>
       </c>
       <c r="F269" s="16" t="inlineStr">
         <is>
@@ -40048,7 +40048,7 @@
       </c>
       <c r="G269" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H269" s="16" t="inlineStr">
@@ -40084,7 +40084,7 @@
         </is>
       </c>
       <c r="E270" s="15" t="n">
-        <v>0.9682539682539684</v>
+        <v>0.970566</v>
       </c>
       <c r="F270" s="16" t="inlineStr">
         <is>
@@ -40093,7 +40093,7 @@
       </c>
       <c r="G270" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H270" s="16" t="inlineStr">
@@ -40129,7 +40129,7 @@
         </is>
       </c>
       <c r="E271" s="15" t="n">
-        <v>0.9697729171413382</v>
+        <v>0.971154</v>
       </c>
       <c r="F271" s="16" t="inlineStr">
         <is>
@@ -40138,7 +40138,7 @@
       </c>
       <c r="G271" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H271" s="16" t="inlineStr">
@@ -40174,7 +40174,7 @@
         </is>
       </c>
       <c r="E272" s="15" t="n">
-        <v>0.9397729171413381</v>
+        <v>0.942308</v>
       </c>
       <c r="F272" s="16" t="inlineStr">
         <is>
@@ -40183,7 +40183,7 @@
       </c>
       <c r="G272" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H272" s="16" t="inlineStr">
@@ -40219,7 +40219,7 @@
         </is>
       </c>
       <c r="E273" s="15" t="n">
-        <v>0.7411720992361243</v>
+        <v>0.711871</v>
       </c>
       <c r="F273" s="16" t="inlineStr">
         <is>
@@ -40228,7 +40228,7 @@
       </c>
       <c r="G273" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H273" s="16" t="inlineStr">
@@ -40264,7 +40264,7 @@
         </is>
       </c>
       <c r="E274" s="15" t="n">
-        <v>0.7644488625062797</v>
+        <v>0.739764</v>
       </c>
       <c r="F274" s="16" t="inlineStr">
         <is>
@@ -40273,7 +40273,7 @@
       </c>
       <c r="G274" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H274" s="16" t="inlineStr">
@@ -40309,7 +40309,7 @@
         </is>
       </c>
       <c r="E275" s="15" t="n">
-        <v>0.7431693989071039</v>
+        <v>0.711871</v>
       </c>
       <c r="F275" s="16" t="inlineStr">
         <is>
@@ -40318,7 +40318,7 @@
       </c>
       <c r="G275" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H275" s="16" t="inlineStr">
@@ -40354,7 +40354,7 @@
         </is>
       </c>
       <c r="E276" s="15" t="n">
-        <v>0.7456709956709957</v>
+        <v>0.739764</v>
       </c>
       <c r="F276" s="16" t="inlineStr">
         <is>
@@ -40363,7 +40363,7 @@
       </c>
       <c r="G276" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H276" s="16" t="inlineStr">
@@ -40399,7 +40399,7 @@
         </is>
       </c>
       <c r="E277" s="15" t="n">
-        <v>0.7473717357888511</v>
+        <v>0.679007</v>
       </c>
       <c r="F277" s="16" t="inlineStr">
         <is>
@@ -40408,7 +40408,7 @@
       </c>
       <c r="G277" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H277" s="16" t="inlineStr">
@@ -40444,7 +40444,7 @@
         </is>
       </c>
       <c r="E278" s="15" t="n">
-        <v>0.700813968808538</v>
+        <v>0.609322</v>
       </c>
       <c r="F278" s="16" t="inlineStr">
         <is>
@@ -40453,7 +40453,7 @@
       </c>
       <c r="G278" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H278" s="16" t="inlineStr">
@@ -40489,7 +40489,7 @@
         </is>
       </c>
       <c r="E279" s="15" t="n">
-        <v>0.4727564102564102</v>
+        <v>0.679007</v>
       </c>
       <c r="F279" s="16" t="inlineStr">
         <is>
@@ -40498,7 +40498,7 @@
       </c>
       <c r="G279" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H279" s="16" t="inlineStr">
@@ -40534,7 +40534,7 @@
         </is>
       </c>
       <c r="E280" s="15" t="n">
-        <v>0.5554054054054054</v>
+        <v>0.609322</v>
       </c>
       <c r="F280" s="16" t="inlineStr">
         <is>
@@ -40543,7 +40543,7 @@
       </c>
       <c r="G280" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H280" s="16" t="inlineStr">
@@ -40579,7 +40579,7 @@
         </is>
       </c>
       <c r="E281" s="15" t="n">
-        <v>0.7602906132436795</v>
+        <v>0.738472</v>
       </c>
       <c r="F281" s="16" t="inlineStr">
         <is>
@@ -40588,7 +40588,7 @@
       </c>
       <c r="G281" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H281" s="16" t="inlineStr">
@@ -40624,7 +40624,7 @@
         </is>
       </c>
       <c r="E282" s="15" t="n">
-        <v>0.7657973784875042</v>
+        <v>0.74547</v>
       </c>
       <c r="F282" s="16" t="inlineStr">
         <is>
@@ -40633,7 +40633,7 @@
       </c>
       <c r="G282" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H282" s="16" t="inlineStr">
@@ -40669,7 +40669,7 @@
         </is>
       </c>
       <c r="E283" s="15" t="n">
-        <v>0.7552083333333333</v>
+        <v>0.738472</v>
       </c>
       <c r="F283" s="16" t="inlineStr">
         <is>
@@ -40678,7 +40678,7 @@
       </c>
       <c r="G283" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H283" s="16" t="inlineStr">
@@ -40714,7 +40714,7 @@
         </is>
       </c>
       <c r="E284" s="15" t="n">
-        <v>0.7631048387096775</v>
+        <v>0.74547</v>
       </c>
       <c r="F284" s="16" t="inlineStr">
         <is>
@@ -40723,7 +40723,7 @@
       </c>
       <c r="G284" s="16" t="inlineStr">
         <is>
-          <t>Optuna-100 fold-mean, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
+          <t>seed-1337 pooled subject-level, 100 TPE trials seed 1337, 3 subject-grouped inner folds, macro-F1 objective, harmonized_all_windows_full_coverage, headline/binary-strict</t>
         </is>
       </c>
       <c r="H284" s="16" t="inlineStr">

</xml_diff>